<commit_message>
Start acutal (without evil)
</commit_message>
<xml_diff>
--- a/CIFAR_Global.xlsx
+++ b/CIFAR_Global.xlsx
@@ -1,41 +1,81 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ashleyau/Documents/PhD/Practical_Experiment/Finalised/Finalised_Algorithm_ResNet/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{491F8CC9-D909-134A-9168-6C8CFA6AF6A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19980" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-41520" yWindow="-1660" windowWidth="34560" windowHeight="19980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="181029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+  <si>
+    <t>100 Rounds</t>
+  </si>
+  <si>
+    <t>IID</t>
+  </si>
+  <si>
+    <t>Global Accuracy</t>
+  </si>
+  <si>
+    <t>Round</t>
+  </si>
+  <si>
+    <t>Clustering Accuracy</t>
+  </si>
+  <si>
+    <t>Round number</t>
+  </si>
+  <si>
+    <t>Poisoning Accuracy</t>
+  </si>
+  <si>
+    <t>Global Poisoning Accuracy</t>
+  </si>
+  <si>
+    <t>5 rounds</t>
+  </si>
+  <si>
+    <t>Actual</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="12"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -54,87 +94,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -454,2144 +435,2126 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B415"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C415"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col width="15.1640625" customWidth="1" min="1" max="1"/>
+    <col min="1" max="1" width="15.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>100 Rounds</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>IID</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Global Accuracy</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Round</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B5" t="n">
-        <v>0.1078</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B6" t="n">
-        <v>0.4665</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B7" t="n">
-        <v>0.644</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>1</v>
+      </c>
+      <c r="B5">
+        <v>0.10780000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>2</v>
+      </c>
+      <c r="B6">
+        <v>0.46650000000000003</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>3</v>
+      </c>
+      <c r="B7">
+        <v>0.64400000000000002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
         <v>4</v>
       </c>
-      <c r="B8" t="n">
-        <v>0.6624</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="B8">
+        <v>0.66239999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
         <v>5</v>
       </c>
-      <c r="B9" t="n">
-        <v>0.7010999999999999</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="B9">
+        <v>0.70109999999999995</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="n">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
         <v>7</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="n">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
         <v>8</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="n">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
         <v>9</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="n">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="n">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="1">
         <v>11</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="n">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="1">
         <v>12</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="n">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="1">
         <v>13</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="1" t="n">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="1">
         <v>14</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="n">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="1">
         <v>15</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="1" t="n">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="1">
         <v>16</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="1" t="n">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="1">
         <v>17</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="n">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="1">
         <v>18</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="n">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="1">
         <v>19</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="1" t="n">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="1">
         <v>20</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="1" t="n">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="1">
         <v>21</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="1" t="n">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="1">
         <v>22</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="1" t="n">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="1">
         <v>23</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="1" t="n">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="1">
         <v>24</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="1" t="n">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="1">
         <v>25</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="1" t="n">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="1">
         <v>26</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="1" t="n">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="1">
         <v>27</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="1" t="n">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="1">
         <v>28</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="1" t="n">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="1">
         <v>29</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="1" t="n">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" s="1">
         <v>30</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="1" t="n">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" s="1">
         <v>31</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="1" t="n">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" s="1">
         <v>32</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="1" t="n">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A37" s="1">
         <v>33</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="1" t="n">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A38" s="1">
         <v>34</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="1" t="n">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A39" s="1">
         <v>35</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="1" t="n">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A40" s="1">
         <v>36</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="1" t="n">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A41" s="1">
         <v>37</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="1" t="n">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A42" s="1">
         <v>38</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="1" t="n">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A43" s="1">
         <v>39</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="1" t="n">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A44" s="1">
         <v>40</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="1" t="n">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A45" s="1">
         <v>41</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="1" t="n">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A46" s="1">
         <v>42</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="1" t="n">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A47" s="1">
         <v>43</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="1" t="n">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A48" s="1">
         <v>44</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="1" t="n">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A49" s="1">
         <v>45</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="1" t="n">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A50" s="1">
         <v>46</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="1" t="n">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A51" s="1">
         <v>47</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="1" t="n">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A52" s="1">
         <v>48</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="1" t="n">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A53" s="1">
         <v>49</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="1" t="n">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A54" s="1">
         <v>50</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="1" t="n">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A55" s="1">
         <v>51</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="1" t="n">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A56" s="1">
         <v>52</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="1" t="n">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A57" s="1">
         <v>53</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="1" t="n">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A58" s="1">
         <v>54</v>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="1" t="n">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A59" s="1">
         <v>55</v>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="1" t="n">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A60" s="1">
         <v>56</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="1" t="n">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A61" s="1">
         <v>57</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="1" t="n">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A62" s="1">
         <v>58</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="1" t="n">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A63" s="1">
         <v>59</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="1" t="n">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A64" s="1">
         <v>60</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="1" t="n">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A65" s="1">
         <v>61</v>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="1" t="n">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A66" s="1">
         <v>62</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="1" t="n">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A67" s="1">
         <v>63</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="1" t="n">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A68" s="1">
         <v>64</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="1" t="n">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A69" s="1">
         <v>65</v>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="1" t="n">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A70" s="1">
         <v>66</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="1" t="n">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A71" s="1">
         <v>67</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="1" t="n">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A72" s="1">
         <v>68</v>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="1" t="n">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A73" s="1">
         <v>69</v>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="1" t="n">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A74" s="1">
         <v>70</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="1" t="n">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A75" s="1">
         <v>71</v>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="1" t="n">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A76" s="1">
         <v>72</v>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="1" t="n">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A77" s="1">
         <v>73</v>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="1" t="n">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A78" s="1">
         <v>74</v>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="1" t="n">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A79" s="1">
         <v>75</v>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="1" t="n">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A80" s="1">
         <v>76</v>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="1" t="n">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A81" s="1">
         <v>77</v>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="1" t="n">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A82" s="1">
         <v>78</v>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="1" t="n">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A83" s="1">
         <v>79</v>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="1" t="n">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A84" s="1">
         <v>80</v>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="1" t="n">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A85" s="1">
         <v>81</v>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="1" t="n">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A86" s="1">
         <v>82</v>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="1" t="n">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A87" s="1">
         <v>83</v>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="1" t="n">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A88" s="1">
         <v>84</v>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="1" t="n">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A89" s="1">
         <v>85</v>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="1" t="n">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A90" s="1">
         <v>86</v>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="1" t="n">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A91" s="1">
         <v>87</v>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="1" t="n">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A92" s="1">
         <v>88</v>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="1" t="n">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A93" s="1">
         <v>89</v>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="1" t="n">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A94" s="1">
         <v>90</v>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="1" t="n">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A95" s="1">
         <v>91</v>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="1" t="n">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A96" s="1">
         <v>92</v>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="1" t="n">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A97" s="1">
         <v>93</v>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="1" t="n">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A98" s="1">
         <v>94</v>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="1" t="n">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A99" s="1">
         <v>95</v>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="1" t="n">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A100" s="1">
         <v>96</v>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="1" t="n">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A101" s="1">
         <v>97</v>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="1" t="n">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A102" s="1">
         <v>98</v>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="1" t="n">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A103" s="1">
         <v>99</v>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="1" t="n">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A104" s="1">
         <v>100</v>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="1" t="inlineStr">
-        <is>
-          <t>Clustering Accuracy</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="3" t="inlineStr">
-        <is>
-          <t>Round number</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="1" t="n">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A106" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A107" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A108" s="1">
         <v>1</v>
       </c>
-      <c r="B108" t="n">
+      <c r="B108">
         <v>1</v>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" s="1" t="n">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A109" s="1">
         <v>2</v>
       </c>
-      <c r="B109" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="1" t="n">
+      <c r="B109">
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A110" s="1">
         <v>3</v>
       </c>
-      <c r="B110" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="1" t="n">
+      <c r="B110">
+        <v>0.33333333333333331</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A111" s="1">
         <v>4</v>
       </c>
-      <c r="B111" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="1" t="n">
+      <c r="B111">
+        <v>0.33333333333333331</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A112" s="1">
         <v>5</v>
       </c>
-      <c r="B112" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="1" t="n">
+      <c r="B112">
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A113" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="1" t="n">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A114" s="1">
         <v>7</v>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" s="1" t="n">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A115" s="1">
         <v>8</v>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" s="1" t="n">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A116" s="1">
         <v>9</v>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" s="1" t="n">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A117" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" s="1" t="n">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A118" s="1">
         <v>11</v>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="1" t="n">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A119" s="1">
         <v>12</v>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" s="1" t="n">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A120" s="1">
         <v>13</v>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" s="1" t="n">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A121" s="1">
         <v>14</v>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="1" t="n">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A122" s="1">
         <v>15</v>
       </c>
     </row>
-    <row r="123">
-      <c r="A123" s="1" t="n">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A123" s="1">
         <v>16</v>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" s="1" t="n">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A124" s="1">
         <v>17</v>
       </c>
     </row>
-    <row r="125">
-      <c r="A125" s="1" t="n">
+    <row r="125" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A125" s="1">
         <v>18</v>
       </c>
     </row>
-    <row r="126">
-      <c r="A126" s="1" t="n">
+    <row r="126" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A126" s="1">
         <v>19</v>
       </c>
     </row>
-    <row r="127">
-      <c r="A127" s="1" t="n">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A127" s="1">
         <v>20</v>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" s="1" t="n">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A128" s="1">
         <v>21</v>
       </c>
     </row>
-    <row r="129">
-      <c r="A129" s="1" t="n">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A129" s="1">
         <v>22</v>
       </c>
     </row>
-    <row r="130">
-      <c r="A130" s="1" t="n">
+    <row r="130" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A130" s="1">
         <v>23</v>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" s="1" t="n">
+    <row r="131" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A131" s="1">
         <v>24</v>
       </c>
     </row>
-    <row r="132">
-      <c r="A132" s="1" t="n">
+    <row r="132" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A132" s="1">
         <v>25</v>
       </c>
     </row>
-    <row r="133">
-      <c r="A133" s="1" t="n">
+    <row r="133" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A133" s="1">
         <v>26</v>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" s="1" t="n">
+    <row r="134" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A134" s="1">
         <v>27</v>
       </c>
     </row>
-    <row r="135">
-      <c r="A135" s="1" t="n">
+    <row r="135" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A135" s="1">
         <v>28</v>
       </c>
     </row>
-    <row r="136">
-      <c r="A136" s="1" t="n">
+    <row r="136" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A136" s="1">
         <v>29</v>
       </c>
     </row>
-    <row r="137">
-      <c r="A137" s="1" t="n">
+    <row r="137" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A137" s="1">
         <v>30</v>
       </c>
     </row>
-    <row r="138">
-      <c r="A138" s="1" t="n">
+    <row r="138" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A138" s="1">
         <v>31</v>
       </c>
     </row>
-    <row r="139">
-      <c r="A139" s="1" t="n">
+    <row r="139" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A139" s="1">
         <v>32</v>
       </c>
     </row>
-    <row r="140">
-      <c r="A140" s="1" t="n">
+    <row r="140" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A140" s="1">
         <v>33</v>
       </c>
     </row>
-    <row r="141">
-      <c r="A141" s="1" t="n">
+    <row r="141" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A141" s="1">
         <v>34</v>
       </c>
     </row>
-    <row r="142">
-      <c r="A142" s="1" t="n">
+    <row r="142" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A142" s="1">
         <v>35</v>
       </c>
     </row>
-    <row r="143">
-      <c r="A143" s="1" t="n">
+    <row r="143" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A143" s="1">
         <v>36</v>
       </c>
     </row>
-    <row r="144">
-      <c r="A144" s="1" t="n">
+    <row r="144" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A144" s="1">
         <v>37</v>
       </c>
     </row>
-    <row r="145">
-      <c r="A145" s="1" t="n">
+    <row r="145" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A145" s="1">
         <v>38</v>
       </c>
     </row>
-    <row r="146">
-      <c r="A146" s="1" t="n">
+    <row r="146" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A146" s="1">
         <v>39</v>
       </c>
     </row>
-    <row r="147">
-      <c r="A147" s="1" t="n">
+    <row r="147" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A147" s="1">
         <v>40</v>
       </c>
     </row>
-    <row r="148">
-      <c r="A148" s="1" t="n">
+    <row r="148" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A148" s="1">
         <v>41</v>
       </c>
     </row>
-    <row r="149">
-      <c r="A149" s="1" t="n">
+    <row r="149" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A149" s="1">
         <v>42</v>
       </c>
     </row>
-    <row r="150">
-      <c r="A150" s="1" t="n">
+    <row r="150" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A150" s="1">
         <v>43</v>
       </c>
     </row>
-    <row r="151">
-      <c r="A151" s="1" t="n">
+    <row r="151" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A151" s="1">
         <v>44</v>
       </c>
     </row>
-    <row r="152">
-      <c r="A152" s="1" t="n">
+    <row r="152" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A152" s="1">
         <v>45</v>
       </c>
     </row>
-    <row r="153">
-      <c r="A153" s="1" t="n">
+    <row r="153" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A153" s="1">
         <v>46</v>
       </c>
     </row>
-    <row r="154">
-      <c r="A154" s="1" t="n">
+    <row r="154" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A154" s="1">
         <v>47</v>
       </c>
     </row>
-    <row r="155">
-      <c r="A155" s="1" t="n">
+    <row r="155" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A155" s="1">
         <v>48</v>
       </c>
     </row>
-    <row r="156">
-      <c r="A156" s="1" t="n">
+    <row r="156" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A156" s="1">
         <v>49</v>
       </c>
     </row>
-    <row r="157">
-      <c r="A157" s="1" t="n">
+    <row r="157" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A157" s="1">
         <v>50</v>
       </c>
     </row>
-    <row r="158">
-      <c r="A158" s="1" t="n">
+    <row r="158" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A158" s="1">
         <v>51</v>
       </c>
     </row>
-    <row r="159">
-      <c r="A159" s="1" t="n">
+    <row r="159" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A159" s="1">
         <v>52</v>
       </c>
     </row>
-    <row r="160">
-      <c r="A160" s="1" t="n">
+    <row r="160" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A160" s="1">
         <v>53</v>
       </c>
     </row>
-    <row r="161">
-      <c r="A161" s="1" t="n">
+    <row r="161" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A161" s="1">
         <v>54</v>
       </c>
     </row>
-    <row r="162">
-      <c r="A162" s="1" t="n">
+    <row r="162" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A162" s="1">
         <v>55</v>
       </c>
     </row>
-    <row r="163">
-      <c r="A163" s="1" t="n">
+    <row r="163" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A163" s="1">
         <v>56</v>
       </c>
     </row>
-    <row r="164">
-      <c r="A164" s="1" t="n">
+    <row r="164" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A164" s="1">
         <v>57</v>
       </c>
     </row>
-    <row r="165">
-      <c r="A165" s="1" t="n">
+    <row r="165" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A165" s="1">
         <v>58</v>
       </c>
     </row>
-    <row r="166">
-      <c r="A166" s="1" t="n">
+    <row r="166" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A166" s="1">
         <v>59</v>
       </c>
     </row>
-    <row r="167">
-      <c r="A167" s="1" t="n">
+    <row r="167" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A167" s="1">
         <v>60</v>
       </c>
     </row>
-    <row r="168">
-      <c r="A168" s="1" t="n">
+    <row r="168" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A168" s="1">
         <v>61</v>
       </c>
     </row>
-    <row r="169">
-      <c r="A169" s="1" t="n">
+    <row r="169" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A169" s="1">
         <v>62</v>
       </c>
     </row>
-    <row r="170">
-      <c r="A170" s="1" t="n">
+    <row r="170" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A170" s="1">
         <v>63</v>
       </c>
     </row>
-    <row r="171">
-      <c r="A171" s="1" t="n">
+    <row r="171" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A171" s="1">
         <v>64</v>
       </c>
     </row>
-    <row r="172">
-      <c r="A172" s="1" t="n">
+    <row r="172" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A172" s="1">
         <v>65</v>
       </c>
     </row>
-    <row r="173">
-      <c r="A173" s="1" t="n">
+    <row r="173" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A173" s="1">
         <v>66</v>
       </c>
     </row>
-    <row r="174">
-      <c r="A174" s="1" t="n">
+    <row r="174" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A174" s="1">
         <v>67</v>
       </c>
     </row>
-    <row r="175">
-      <c r="A175" s="1" t="n">
+    <row r="175" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A175" s="1">
         <v>68</v>
       </c>
     </row>
-    <row r="176">
-      <c r="A176" s="1" t="n">
+    <row r="176" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A176" s="1">
         <v>69</v>
       </c>
     </row>
-    <row r="177">
-      <c r="A177" s="1" t="n">
+    <row r="177" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A177" s="1">
         <v>70</v>
       </c>
     </row>
-    <row r="178">
-      <c r="A178" s="1" t="n">
+    <row r="178" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A178" s="1">
         <v>71</v>
       </c>
     </row>
-    <row r="179">
-      <c r="A179" s="1" t="n">
+    <row r="179" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A179" s="1">
         <v>72</v>
       </c>
     </row>
-    <row r="180">
-      <c r="A180" s="1" t="n">
+    <row r="180" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A180" s="1">
         <v>73</v>
       </c>
     </row>
-    <row r="181">
-      <c r="A181" s="1" t="n">
+    <row r="181" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A181" s="1">
         <v>74</v>
       </c>
     </row>
-    <row r="182">
-      <c r="A182" s="1" t="n">
+    <row r="182" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A182" s="1">
         <v>75</v>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="1" t="n">
+    <row r="183" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A183" s="1">
         <v>76</v>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="1" t="n">
+    <row r="184" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A184" s="1">
         <v>77</v>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" s="1" t="n">
+    <row r="185" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A185" s="1">
         <v>78</v>
       </c>
     </row>
-    <row r="186">
-      <c r="A186" s="1" t="n">
+    <row r="186" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A186" s="1">
         <v>79</v>
       </c>
     </row>
-    <row r="187">
-      <c r="A187" s="1" t="n">
+    <row r="187" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A187" s="1">
         <v>80</v>
       </c>
     </row>
-    <row r="188">
-      <c r="A188" s="1" t="n">
+    <row r="188" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A188" s="1">
         <v>81</v>
       </c>
     </row>
-    <row r="189">
-      <c r="A189" s="1" t="n">
+    <row r="189" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A189" s="1">
         <v>82</v>
       </c>
     </row>
-    <row r="190">
-      <c r="A190" s="1" t="n">
+    <row r="190" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A190" s="1">
         <v>83</v>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" s="1" t="n">
+    <row r="191" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A191" s="1">
         <v>84</v>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" s="1" t="n">
+    <row r="192" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A192" s="1">
         <v>85</v>
       </c>
     </row>
-    <row r="193">
-      <c r="A193" s="1" t="n">
+    <row r="193" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A193" s="1">
         <v>86</v>
       </c>
     </row>
-    <row r="194">
-      <c r="A194" s="1" t="n">
+    <row r="194" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A194" s="1">
         <v>87</v>
       </c>
     </row>
-    <row r="195">
-      <c r="A195" s="1" t="n">
+    <row r="195" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A195" s="1">
         <v>88</v>
       </c>
     </row>
-    <row r="196">
-      <c r="A196" s="1" t="n">
+    <row r="196" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A196" s="1">
         <v>89</v>
       </c>
     </row>
-    <row r="197">
-      <c r="A197" s="1" t="n">
+    <row r="197" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A197" s="1">
         <v>90</v>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" s="1" t="n">
+    <row r="198" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A198" s="1">
         <v>91</v>
       </c>
     </row>
-    <row r="199">
-      <c r="A199" s="1" t="n">
+    <row r="199" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A199" s="1">
         <v>92</v>
       </c>
     </row>
-    <row r="200">
-      <c r="A200" s="1" t="n">
+    <row r="200" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A200" s="1">
         <v>93</v>
       </c>
     </row>
-    <row r="201">
-      <c r="A201" s="1" t="n">
+    <row r="201" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A201" s="1">
         <v>94</v>
       </c>
     </row>
-    <row r="202">
-      <c r="A202" s="1" t="n">
+    <row r="202" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A202" s="1">
         <v>95</v>
       </c>
     </row>
-    <row r="203">
-      <c r="A203" s="1" t="n">
+    <row r="203" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A203" s="1">
         <v>96</v>
       </c>
     </row>
-    <row r="204">
-      <c r="A204" s="1" t="n">
+    <row r="204" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A204" s="1">
         <v>97</v>
       </c>
     </row>
-    <row r="205">
-      <c r="A205" s="1" t="n">
+    <row r="205" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A205" s="1">
         <v>98</v>
       </c>
     </row>
-    <row r="206">
-      <c r="A206" s="1" t="n">
+    <row r="206" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A206" s="1">
         <v>99</v>
       </c>
     </row>
-    <row r="207">
-      <c r="A207" s="1" t="n">
+    <row r="207" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A207" s="1">
         <v>100</v>
       </c>
     </row>
-    <row r="210">
-      <c r="A210" s="1" t="inlineStr">
-        <is>
-          <t>Poisoning Accuracy</t>
-        </is>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" s="3" t="inlineStr">
-        <is>
-          <t>Round number</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" s="1" t="n">
+    <row r="210" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A210" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A211" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A212" s="1">
         <v>1</v>
       </c>
-      <c r="B212" t="n">
-        <v>0.99725</v>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" s="1" t="n">
+      <c r="B212">
+        <v>0.99724999999999997</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A213" s="1">
         <v>2</v>
       </c>
-      <c r="B213" t="n">
-        <v>0.99065</v>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" s="1" t="n">
+      <c r="B213">
+        <v>0.99065000000000003</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A214" s="1">
         <v>3</v>
       </c>
-      <c r="B214" t="n">
+      <c r="B214">
         <v>0.9869</v>
       </c>
     </row>
-    <row r="215">
-      <c r="A215" s="1" t="n">
+    <row r="215" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A215" s="1">
         <v>4</v>
       </c>
-      <c r="B215" t="n">
-        <v>0.97765</v>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" s="1" t="n">
+      <c r="B215">
+        <v>0.97765000000000002</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A216" s="1">
         <v>5</v>
       </c>
-      <c r="B216" t="n">
-        <v>0.9846</v>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" s="1" t="n">
+      <c r="B216">
+        <v>0.98460000000000003</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A217" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="218">
-      <c r="A218" s="1" t="n">
+    <row r="218" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A218" s="1">
         <v>7</v>
       </c>
     </row>
-    <row r="219">
-      <c r="A219" s="1" t="n">
+    <row r="219" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A219" s="1">
         <v>8</v>
       </c>
     </row>
-    <row r="220">
-      <c r="A220" s="1" t="n">
+    <row r="220" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A220" s="1">
         <v>9</v>
       </c>
     </row>
-    <row r="221">
-      <c r="A221" s="1" t="n">
+    <row r="221" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A221" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="222">
-      <c r="A222" s="1" t="n">
+    <row r="222" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A222" s="1">
         <v>11</v>
       </c>
     </row>
-    <row r="223">
-      <c r="A223" s="1" t="n">
+    <row r="223" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A223" s="1">
         <v>12</v>
       </c>
     </row>
-    <row r="224">
-      <c r="A224" s="1" t="n">
+    <row r="224" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A224" s="1">
         <v>13</v>
       </c>
     </row>
-    <row r="225">
-      <c r="A225" s="1" t="n">
+    <row r="225" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A225" s="1">
         <v>14</v>
       </c>
     </row>
-    <row r="226">
-      <c r="A226" s="1" t="n">
+    <row r="226" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A226" s="1">
         <v>15</v>
       </c>
     </row>
-    <row r="227">
-      <c r="A227" s="1" t="n">
+    <row r="227" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A227" s="1">
         <v>16</v>
       </c>
     </row>
-    <row r="228">
-      <c r="A228" s="1" t="n">
+    <row r="228" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A228" s="1">
         <v>17</v>
       </c>
     </row>
-    <row r="229">
-      <c r="A229" s="1" t="n">
+    <row r="229" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A229" s="1">
         <v>18</v>
       </c>
     </row>
-    <row r="230">
-      <c r="A230" s="1" t="n">
+    <row r="230" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A230" s="1">
         <v>19</v>
       </c>
     </row>
-    <row r="231">
-      <c r="A231" s="1" t="n">
+    <row r="231" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A231" s="1">
         <v>20</v>
       </c>
     </row>
-    <row r="232">
-      <c r="A232" s="1" t="n">
+    <row r="232" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A232" s="1">
         <v>21</v>
       </c>
     </row>
-    <row r="233">
-      <c r="A233" s="1" t="n">
+    <row r="233" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A233" s="1">
         <v>22</v>
       </c>
     </row>
-    <row r="234">
-      <c r="A234" s="1" t="n">
+    <row r="234" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A234" s="1">
         <v>23</v>
       </c>
     </row>
-    <row r="235">
-      <c r="A235" s="1" t="n">
+    <row r="235" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A235" s="1">
         <v>24</v>
       </c>
     </row>
-    <row r="236">
-      <c r="A236" s="1" t="n">
+    <row r="236" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A236" s="1">
         <v>25</v>
       </c>
     </row>
-    <row r="237">
-      <c r="A237" s="1" t="n">
+    <row r="237" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A237" s="1">
         <v>26</v>
       </c>
     </row>
-    <row r="238">
-      <c r="A238" s="1" t="n">
+    <row r="238" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A238" s="1">
         <v>27</v>
       </c>
     </row>
-    <row r="239">
-      <c r="A239" s="1" t="n">
+    <row r="239" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A239" s="1">
         <v>28</v>
       </c>
     </row>
-    <row r="240">
-      <c r="A240" s="1" t="n">
+    <row r="240" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A240" s="1">
         <v>29</v>
       </c>
     </row>
-    <row r="241">
-      <c r="A241" s="1" t="n">
+    <row r="241" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A241" s="1">
         <v>30</v>
       </c>
     </row>
-    <row r="242">
-      <c r="A242" s="1" t="n">
+    <row r="242" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A242" s="1">
         <v>31</v>
       </c>
     </row>
-    <row r="243">
-      <c r="A243" s="1" t="n">
+    <row r="243" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A243" s="1">
         <v>32</v>
       </c>
     </row>
-    <row r="244">
-      <c r="A244" s="1" t="n">
+    <row r="244" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A244" s="1">
         <v>33</v>
       </c>
     </row>
-    <row r="245">
-      <c r="A245" s="1" t="n">
+    <row r="245" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A245" s="1">
         <v>34</v>
       </c>
     </row>
-    <row r="246">
-      <c r="A246" s="1" t="n">
+    <row r="246" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A246" s="1">
         <v>35</v>
       </c>
     </row>
-    <row r="247">
-      <c r="A247" s="1" t="n">
+    <row r="247" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A247" s="1">
         <v>36</v>
       </c>
     </row>
-    <row r="248">
-      <c r="A248" s="1" t="n">
+    <row r="248" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A248" s="1">
         <v>37</v>
       </c>
     </row>
-    <row r="249">
-      <c r="A249" s="1" t="n">
+    <row r="249" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A249" s="1">
         <v>38</v>
       </c>
     </row>
-    <row r="250">
-      <c r="A250" s="1" t="n">
+    <row r="250" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A250" s="1">
         <v>39</v>
       </c>
     </row>
-    <row r="251">
-      <c r="A251" s="1" t="n">
+    <row r="251" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A251" s="1">
         <v>40</v>
       </c>
     </row>
-    <row r="252">
-      <c r="A252" s="1" t="n">
+    <row r="252" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A252" s="1">
         <v>41</v>
       </c>
     </row>
-    <row r="253">
-      <c r="A253" s="1" t="n">
+    <row r="253" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A253" s="1">
         <v>42</v>
       </c>
     </row>
-    <row r="254">
-      <c r="A254" s="1" t="n">
+    <row r="254" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A254" s="1">
         <v>43</v>
       </c>
     </row>
-    <row r="255">
-      <c r="A255" s="1" t="n">
+    <row r="255" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A255" s="1">
         <v>44</v>
       </c>
     </row>
-    <row r="256">
-      <c r="A256" s="1" t="n">
+    <row r="256" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A256" s="1">
         <v>45</v>
       </c>
     </row>
-    <row r="257">
-      <c r="A257" s="1" t="n">
+    <row r="257" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A257" s="1">
         <v>46</v>
       </c>
     </row>
-    <row r="258">
-      <c r="A258" s="1" t="n">
+    <row r="258" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A258" s="1">
         <v>47</v>
       </c>
     </row>
-    <row r="259">
-      <c r="A259" s="1" t="n">
+    <row r="259" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A259" s="1">
         <v>48</v>
       </c>
     </row>
-    <row r="260">
-      <c r="A260" s="1" t="n">
+    <row r="260" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A260" s="1">
         <v>49</v>
       </c>
     </row>
-    <row r="261">
-      <c r="A261" s="1" t="n">
+    <row r="261" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A261" s="1">
         <v>50</v>
       </c>
     </row>
-    <row r="262">
-      <c r="A262" s="1" t="n">
+    <row r="262" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A262" s="1">
         <v>51</v>
       </c>
     </row>
-    <row r="263">
-      <c r="A263" s="1" t="n">
+    <row r="263" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A263" s="1">
         <v>52</v>
       </c>
     </row>
-    <row r="264">
-      <c r="A264" s="1" t="n">
+    <row r="264" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A264" s="1">
         <v>53</v>
       </c>
     </row>
-    <row r="265">
-      <c r="A265" s="1" t="n">
+    <row r="265" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A265" s="1">
         <v>54</v>
       </c>
     </row>
-    <row r="266">
-      <c r="A266" s="1" t="n">
+    <row r="266" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A266" s="1">
         <v>55</v>
       </c>
     </row>
-    <row r="267">
-      <c r="A267" s="1" t="n">
+    <row r="267" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A267" s="1">
         <v>56</v>
       </c>
     </row>
-    <row r="268">
-      <c r="A268" s="1" t="n">
+    <row r="268" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A268" s="1">
         <v>57</v>
       </c>
     </row>
-    <row r="269">
-      <c r="A269" s="1" t="n">
+    <row r="269" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A269" s="1">
         <v>58</v>
       </c>
     </row>
-    <row r="270">
-      <c r="A270" s="1" t="n">
+    <row r="270" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A270" s="1">
         <v>59</v>
       </c>
     </row>
-    <row r="271">
-      <c r="A271" s="1" t="n">
+    <row r="271" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A271" s="1">
         <v>60</v>
       </c>
     </row>
-    <row r="272">
-      <c r="A272" s="1" t="n">
+    <row r="272" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A272" s="1">
         <v>61</v>
       </c>
     </row>
-    <row r="273">
-      <c r="A273" s="1" t="n">
+    <row r="273" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A273" s="1">
         <v>62</v>
       </c>
     </row>
-    <row r="274">
-      <c r="A274" s="1" t="n">
+    <row r="274" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A274" s="1">
         <v>63</v>
       </c>
     </row>
-    <row r="275">
-      <c r="A275" s="1" t="n">
+    <row r="275" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A275" s="1">
         <v>64</v>
       </c>
     </row>
-    <row r="276">
-      <c r="A276" s="1" t="n">
+    <row r="276" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A276" s="1">
         <v>65</v>
       </c>
     </row>
-    <row r="277">
-      <c r="A277" s="1" t="n">
+    <row r="277" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A277" s="1">
         <v>66</v>
       </c>
     </row>
-    <row r="278">
-      <c r="A278" s="1" t="n">
+    <row r="278" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A278" s="1">
         <v>67</v>
       </c>
     </row>
-    <row r="279">
-      <c r="A279" s="1" t="n">
+    <row r="279" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A279" s="1">
         <v>68</v>
       </c>
     </row>
-    <row r="280">
-      <c r="A280" s="1" t="n">
+    <row r="280" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A280" s="1">
         <v>69</v>
       </c>
     </row>
-    <row r="281">
-      <c r="A281" s="1" t="n">
+    <row r="281" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A281" s="1">
         <v>70</v>
       </c>
     </row>
-    <row r="282">
-      <c r="A282" s="1" t="n">
+    <row r="282" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A282" s="1">
         <v>71</v>
       </c>
     </row>
-    <row r="283">
-      <c r="A283" s="1" t="n">
+    <row r="283" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A283" s="1">
         <v>72</v>
       </c>
     </row>
-    <row r="284">
-      <c r="A284" s="1" t="n">
+    <row r="284" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A284" s="1">
         <v>73</v>
       </c>
     </row>
-    <row r="285">
-      <c r="A285" s="1" t="n">
+    <row r="285" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A285" s="1">
         <v>74</v>
       </c>
     </row>
-    <row r="286">
-      <c r="A286" s="1" t="n">
+    <row r="286" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A286" s="1">
         <v>75</v>
       </c>
     </row>
-    <row r="287">
-      <c r="A287" s="1" t="n">
+    <row r="287" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A287" s="1">
         <v>76</v>
       </c>
     </row>
-    <row r="288">
-      <c r="A288" s="1" t="n">
+    <row r="288" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A288" s="1">
         <v>77</v>
       </c>
     </row>
-    <row r="289">
-      <c r="A289" s="1" t="n">
+    <row r="289" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A289" s="1">
         <v>78</v>
       </c>
     </row>
-    <row r="290">
-      <c r="A290" s="1" t="n">
+    <row r="290" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A290" s="1">
         <v>79</v>
       </c>
     </row>
-    <row r="291">
-      <c r="A291" s="1" t="n">
+    <row r="291" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A291" s="1">
         <v>80</v>
       </c>
     </row>
-    <row r="292">
-      <c r="A292" s="1" t="n">
+    <row r="292" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A292" s="1">
         <v>81</v>
       </c>
     </row>
-    <row r="293">
-      <c r="A293" s="1" t="n">
+    <row r="293" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A293" s="1">
         <v>82</v>
       </c>
     </row>
-    <row r="294">
-      <c r="A294" s="1" t="n">
+    <row r="294" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A294" s="1">
         <v>83</v>
       </c>
     </row>
-    <row r="295">
-      <c r="A295" s="1" t="n">
+    <row r="295" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A295" s="1">
         <v>84</v>
       </c>
     </row>
-    <row r="296">
-      <c r="A296" s="1" t="n">
+    <row r="296" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A296" s="1">
         <v>85</v>
       </c>
     </row>
-    <row r="297">
-      <c r="A297" s="1" t="n">
+    <row r="297" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A297" s="1">
         <v>86</v>
       </c>
     </row>
-    <row r="298">
-      <c r="A298" s="1" t="n">
+    <row r="298" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A298" s="1">
         <v>87</v>
       </c>
     </row>
-    <row r="299">
-      <c r="A299" s="1" t="n">
+    <row r="299" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A299" s="1">
         <v>88</v>
       </c>
     </row>
-    <row r="300">
-      <c r="A300" s="1" t="n">
+    <row r="300" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A300" s="1">
         <v>89</v>
       </c>
     </row>
-    <row r="301">
-      <c r="A301" s="1" t="n">
+    <row r="301" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A301" s="1">
         <v>90</v>
       </c>
     </row>
-    <row r="302">
-      <c r="A302" s="1" t="n">
+    <row r="302" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A302" s="1">
         <v>91</v>
       </c>
     </row>
-    <row r="303">
-      <c r="A303" s="1" t="n">
+    <row r="303" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A303" s="1">
         <v>92</v>
       </c>
     </row>
-    <row r="304">
-      <c r="A304" s="1" t="n">
+    <row r="304" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A304" s="1">
         <v>93</v>
       </c>
     </row>
-    <row r="305">
-      <c r="A305" s="1" t="n">
+    <row r="305" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A305" s="1">
         <v>94</v>
       </c>
     </row>
-    <row r="306">
-      <c r="A306" s="1" t="n">
+    <row r="306" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A306" s="1">
         <v>95</v>
       </c>
     </row>
-    <row r="307">
-      <c r="A307" s="1" t="n">
+    <row r="307" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A307" s="1">
         <v>96</v>
       </c>
     </row>
-    <row r="308">
-      <c r="A308" s="1" t="n">
+    <row r="308" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A308" s="1">
         <v>97</v>
       </c>
     </row>
-    <row r="309">
-      <c r="A309" s="1" t="n">
+    <row r="309" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A309" s="1">
         <v>98</v>
       </c>
     </row>
-    <row r="310">
-      <c r="A310" s="1" t="n">
+    <row r="310" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A310" s="1">
         <v>99</v>
       </c>
     </row>
-    <row r="311">
-      <c r="A311" s="1" t="n">
+    <row r="311" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A311" s="1">
         <v>100</v>
       </c>
     </row>
-    <row r="314">
-      <c r="A314" s="1" t="inlineStr">
-        <is>
-          <t>Global Poisoning Accuracy</t>
-        </is>
-      </c>
-    </row>
-    <row r="315">
-      <c r="A315" s="3" t="inlineStr">
-        <is>
-          <t>Round number</t>
-        </is>
-      </c>
-    </row>
-    <row r="316">
-      <c r="A316" s="1" t="n">
+    <row r="314" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A314" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="315" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A315" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="316" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A316" s="1">
         <v>1</v>
       </c>
-      <c r="B316" t="n">
+      <c r="B316">
         <v>0</v>
       </c>
     </row>
-    <row r="317">
-      <c r="A317" s="1" t="n">
+    <row r="317" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A317" s="1">
         <v>2</v>
       </c>
-      <c r="B317" t="n">
-        <v>0.0939</v>
-      </c>
-    </row>
-    <row r="318">
-      <c r="A318" s="1" t="n">
+      <c r="B317">
+        <v>9.3899999999999997E-2</v>
+      </c>
+    </row>
+    <row r="318" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A318" s="1">
         <v>3</v>
       </c>
-      <c r="B318" t="n">
+      <c r="B318">
         <v>0.1361</v>
       </c>
     </row>
-    <row r="319">
-      <c r="A319" s="1" t="n">
+    <row r="319" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A319" s="1">
         <v>4</v>
       </c>
-      <c r="B319" t="n">
-        <v>0.0891</v>
-      </c>
-    </row>
-    <row r="320">
-      <c r="A320" s="1" t="n">
+      <c r="B319">
+        <v>8.9099999999999999E-2</v>
+      </c>
+    </row>
+    <row r="320" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A320" s="1">
         <v>5</v>
       </c>
-      <c r="B320" t="n">
+      <c r="B320">
         <v>0.1075</v>
       </c>
     </row>
-    <row r="321">
-      <c r="A321" s="1" t="n">
+    <row r="321" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A321" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="322">
-      <c r="A322" s="1" t="n">
+    <row r="322" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A322" s="1">
         <v>7</v>
       </c>
     </row>
-    <row r="323">
-      <c r="A323" s="1" t="n">
+    <row r="323" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A323" s="1">
         <v>8</v>
       </c>
     </row>
-    <row r="324">
-      <c r="A324" s="1" t="n">
+    <row r="324" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A324" s="1">
         <v>9</v>
       </c>
     </row>
-    <row r="325">
-      <c r="A325" s="1" t="n">
+    <row r="325" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A325" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="326">
-      <c r="A326" s="1" t="n">
+    <row r="326" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A326" s="1">
         <v>11</v>
       </c>
     </row>
-    <row r="327">
-      <c r="A327" s="1" t="n">
+    <row r="327" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A327" s="1">
         <v>12</v>
       </c>
     </row>
-    <row r="328">
-      <c r="A328" s="1" t="n">
+    <row r="328" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A328" s="1">
         <v>13</v>
       </c>
     </row>
-    <row r="329">
-      <c r="A329" s="1" t="n">
+    <row r="329" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A329" s="1">
         <v>14</v>
       </c>
     </row>
-    <row r="330">
-      <c r="A330" s="1" t="n">
+    <row r="330" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A330" s="1">
         <v>15</v>
       </c>
     </row>
-    <row r="331">
-      <c r="A331" s="1" t="n">
+    <row r="331" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A331" s="1">
         <v>16</v>
       </c>
     </row>
-    <row r="332">
-      <c r="A332" s="1" t="n">
+    <row r="332" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A332" s="1">
         <v>17</v>
       </c>
     </row>
-    <row r="333">
-      <c r="A333" s="1" t="n">
+    <row r="333" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A333" s="1">
         <v>18</v>
       </c>
     </row>
-    <row r="334">
-      <c r="A334" s="1" t="n">
+    <row r="334" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A334" s="1">
         <v>19</v>
       </c>
     </row>
-    <row r="335">
-      <c r="A335" s="1" t="n">
+    <row r="335" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A335" s="1">
         <v>20</v>
       </c>
     </row>
-    <row r="336">
-      <c r="A336" s="1" t="n">
+    <row r="336" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A336" s="1">
         <v>21</v>
       </c>
     </row>
-    <row r="337">
-      <c r="A337" s="1" t="n">
+    <row r="337" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A337" s="1">
         <v>22</v>
       </c>
     </row>
-    <row r="338">
-      <c r="A338" s="1" t="n">
+    <row r="338" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A338" s="1">
         <v>23</v>
       </c>
     </row>
-    <row r="339">
-      <c r="A339" s="1" t="n">
+    <row r="339" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A339" s="1">
         <v>24</v>
       </c>
     </row>
-    <row r="340">
-      <c r="A340" s="1" t="n">
+    <row r="340" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A340" s="1">
         <v>25</v>
       </c>
     </row>
-    <row r="341">
-      <c r="A341" s="1" t="n">
+    <row r="341" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A341" s="1">
         <v>26</v>
       </c>
     </row>
-    <row r="342">
-      <c r="A342" s="1" t="n">
+    <row r="342" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A342" s="1">
         <v>27</v>
       </c>
     </row>
-    <row r="343">
-      <c r="A343" s="1" t="n">
+    <row r="343" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A343" s="1">
         <v>28</v>
       </c>
     </row>
-    <row r="344">
-      <c r="A344" s="1" t="n">
+    <row r="344" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A344" s="1">
         <v>29</v>
       </c>
     </row>
-    <row r="345">
-      <c r="A345" s="1" t="n">
+    <row r="345" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A345" s="1">
         <v>30</v>
       </c>
     </row>
-    <row r="346">
-      <c r="A346" s="1" t="n">
+    <row r="346" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A346" s="1">
         <v>31</v>
       </c>
     </row>
-    <row r="347">
-      <c r="A347" s="1" t="n">
+    <row r="347" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A347" s="1">
         <v>32</v>
       </c>
     </row>
-    <row r="348">
-      <c r="A348" s="1" t="n">
+    <row r="348" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A348" s="1">
         <v>33</v>
       </c>
     </row>
-    <row r="349">
-      <c r="A349" s="1" t="n">
+    <row r="349" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A349" s="1">
         <v>34</v>
       </c>
     </row>
-    <row r="350">
-      <c r="A350" s="1" t="n">
+    <row r="350" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A350" s="1">
         <v>35</v>
       </c>
     </row>
-    <row r="351">
-      <c r="A351" s="1" t="n">
+    <row r="351" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A351" s="1">
         <v>36</v>
       </c>
     </row>
-    <row r="352">
-      <c r="A352" s="1" t="n">
+    <row r="352" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A352" s="1">
         <v>37</v>
       </c>
     </row>
-    <row r="353">
-      <c r="A353" s="1" t="n">
+    <row r="353" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A353" s="1">
         <v>38</v>
       </c>
     </row>
-    <row r="354">
-      <c r="A354" s="1" t="n">
+    <row r="354" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A354" s="1">
         <v>39</v>
       </c>
     </row>
-    <row r="355">
-      <c r="A355" s="1" t="n">
+    <row r="355" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A355" s="1">
         <v>40</v>
       </c>
     </row>
-    <row r="356">
-      <c r="A356" s="1" t="n">
+    <row r="356" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A356" s="1">
         <v>41</v>
       </c>
     </row>
-    <row r="357">
-      <c r="A357" s="1" t="n">
+    <row r="357" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A357" s="1">
         <v>42</v>
       </c>
     </row>
-    <row r="358">
-      <c r="A358" s="1" t="n">
+    <row r="358" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A358" s="1">
         <v>43</v>
       </c>
     </row>
-    <row r="359">
-      <c r="A359" s="1" t="n">
+    <row r="359" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A359" s="1">
         <v>44</v>
       </c>
     </row>
-    <row r="360">
-      <c r="A360" s="1" t="n">
+    <row r="360" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A360" s="1">
         <v>45</v>
       </c>
     </row>
-    <row r="361">
-      <c r="A361" s="1" t="n">
+    <row r="361" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A361" s="1">
         <v>46</v>
       </c>
     </row>
-    <row r="362">
-      <c r="A362" s="1" t="n">
+    <row r="362" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A362" s="1">
         <v>47</v>
       </c>
     </row>
-    <row r="363">
-      <c r="A363" s="1" t="n">
+    <row r="363" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A363" s="1">
         <v>48</v>
       </c>
     </row>
-    <row r="364">
-      <c r="A364" s="1" t="n">
+    <row r="364" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A364" s="1">
         <v>49</v>
       </c>
     </row>
-    <row r="365">
-      <c r="A365" s="1" t="n">
+    <row r="365" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A365" s="1">
         <v>50</v>
       </c>
     </row>
-    <row r="366">
-      <c r="A366" s="1" t="n">
+    <row r="366" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A366" s="1">
         <v>51</v>
       </c>
     </row>
-    <row r="367">
-      <c r="A367" s="1" t="n">
+    <row r="367" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A367" s="1">
         <v>52</v>
       </c>
     </row>
-    <row r="368">
-      <c r="A368" s="1" t="n">
+    <row r="368" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A368" s="1">
         <v>53</v>
       </c>
     </row>
-    <row r="369">
-      <c r="A369" s="1" t="n">
+    <row r="369" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A369" s="1">
         <v>54</v>
       </c>
     </row>
-    <row r="370">
-      <c r="A370" s="1" t="n">
+    <row r="370" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A370" s="1">
         <v>55</v>
       </c>
     </row>
-    <row r="371">
-      <c r="A371" s="1" t="n">
+    <row r="371" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A371" s="1">
         <v>56</v>
       </c>
     </row>
-    <row r="372">
-      <c r="A372" s="1" t="n">
+    <row r="372" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A372" s="1">
         <v>57</v>
       </c>
     </row>
-    <row r="373">
-      <c r="A373" s="1" t="n">
+    <row r="373" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A373" s="1">
         <v>58</v>
       </c>
     </row>
-    <row r="374">
-      <c r="A374" s="1" t="n">
+    <row r="374" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A374" s="1">
         <v>59</v>
       </c>
     </row>
-    <row r="375">
-      <c r="A375" s="1" t="n">
+    <row r="375" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A375" s="1">
         <v>60</v>
       </c>
     </row>
-    <row r="376">
-      <c r="A376" s="1" t="n">
+    <row r="376" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A376" s="1">
         <v>61</v>
       </c>
     </row>
-    <row r="377">
-      <c r="A377" s="1" t="n">
+    <row r="377" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A377" s="1">
         <v>62</v>
       </c>
     </row>
-    <row r="378">
-      <c r="A378" s="1" t="n">
+    <row r="378" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A378" s="1">
         <v>63</v>
       </c>
     </row>
-    <row r="379">
-      <c r="A379" s="1" t="n">
+    <row r="379" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A379" s="1">
         <v>64</v>
       </c>
     </row>
-    <row r="380">
-      <c r="A380" s="1" t="n">
+    <row r="380" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A380" s="1">
         <v>65</v>
       </c>
     </row>
-    <row r="381">
-      <c r="A381" s="1" t="n">
+    <row r="381" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A381" s="1">
         <v>66</v>
       </c>
     </row>
-    <row r="382">
-      <c r="A382" s="1" t="n">
+    <row r="382" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A382" s="1">
         <v>67</v>
       </c>
     </row>
-    <row r="383">
-      <c r="A383" s="1" t="n">
+    <row r="383" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A383" s="1">
         <v>68</v>
       </c>
     </row>
-    <row r="384">
-      <c r="A384" s="1" t="n">
+    <row r="384" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A384" s="1">
         <v>69</v>
       </c>
     </row>
-    <row r="385">
-      <c r="A385" s="1" t="n">
+    <row r="385" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A385" s="1">
         <v>70</v>
       </c>
     </row>
-    <row r="386">
-      <c r="A386" s="1" t="n">
+    <row r="386" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A386" s="1">
         <v>71</v>
       </c>
     </row>
-    <row r="387">
-      <c r="A387" s="1" t="n">
+    <row r="387" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A387" s="1">
         <v>72</v>
       </c>
     </row>
-    <row r="388">
-      <c r="A388" s="1" t="n">
+    <row r="388" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A388" s="1">
         <v>73</v>
       </c>
     </row>
-    <row r="389">
-      <c r="A389" s="1" t="n">
+    <row r="389" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A389" s="1">
         <v>74</v>
       </c>
     </row>
-    <row r="390">
-      <c r="A390" s="1" t="n">
+    <row r="390" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A390" s="1">
         <v>75</v>
       </c>
     </row>
-    <row r="391">
-      <c r="A391" s="1" t="n">
+    <row r="391" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A391" s="1">
         <v>76</v>
       </c>
     </row>
-    <row r="392">
-      <c r="A392" s="1" t="n">
+    <row r="392" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A392" s="1">
         <v>77</v>
       </c>
     </row>
-    <row r="393">
-      <c r="A393" s="1" t="n">
+    <row r="393" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A393" s="1">
         <v>78</v>
       </c>
     </row>
-    <row r="394">
-      <c r="A394" s="1" t="n">
+    <row r="394" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A394" s="1">
         <v>79</v>
       </c>
     </row>
-    <row r="395">
-      <c r="A395" s="1" t="n">
+    <row r="395" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A395" s="1">
         <v>80</v>
       </c>
     </row>
-    <row r="396">
-      <c r="A396" s="1" t="n">
+    <row r="396" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A396" s="1">
         <v>81</v>
       </c>
     </row>
-    <row r="397">
-      <c r="A397" s="1" t="n">
+    <row r="397" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A397" s="1">
         <v>82</v>
       </c>
     </row>
-    <row r="398">
-      <c r="A398" s="1" t="n">
+    <row r="398" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A398" s="1">
         <v>83</v>
       </c>
     </row>
-    <row r="399">
-      <c r="A399" s="1" t="n">
+    <row r="399" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A399" s="1">
         <v>84</v>
       </c>
     </row>
-    <row r="400">
-      <c r="A400" s="1" t="n">
+    <row r="400" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A400" s="1">
         <v>85</v>
       </c>
     </row>
-    <row r="401">
-      <c r="A401" s="1" t="n">
+    <row r="401" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A401" s="1">
         <v>86</v>
       </c>
     </row>
-    <row r="402">
-      <c r="A402" s="1" t="n">
+    <row r="402" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A402" s="1">
         <v>87</v>
       </c>
     </row>
-    <row r="403">
-      <c r="A403" s="1" t="n">
+    <row r="403" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A403" s="1">
         <v>88</v>
       </c>
     </row>
-    <row r="404">
-      <c r="A404" s="1" t="n">
+    <row r="404" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A404" s="1">
         <v>89</v>
       </c>
     </row>
-    <row r="405">
-      <c r="A405" s="1" t="n">
+    <row r="405" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A405" s="1">
         <v>90</v>
       </c>
     </row>
-    <row r="406">
-      <c r="A406" s="1" t="n">
+    <row r="406" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A406" s="1">
         <v>91</v>
       </c>
     </row>
-    <row r="407">
-      <c r="A407" s="1" t="n">
+    <row r="407" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A407" s="1">
         <v>92</v>
       </c>
     </row>
-    <row r="408">
-      <c r="A408" s="1" t="n">
+    <row r="408" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A408" s="1">
         <v>93</v>
       </c>
     </row>
-    <row r="409">
-      <c r="A409" s="1" t="n">
+    <row r="409" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A409" s="1">
         <v>94</v>
       </c>
     </row>
-    <row r="410">
-      <c r="A410" s="1" t="n">
+    <row r="410" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A410" s="1">
         <v>95</v>
       </c>
     </row>
-    <row r="411">
-      <c r="A411" s="1" t="n">
+    <row r="411" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A411" s="1">
         <v>96</v>
       </c>
     </row>
-    <row r="412">
-      <c r="A412" s="1" t="n">
+    <row r="412" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A412" s="1">
         <v>97</v>
       </c>
     </row>
-    <row r="413">
-      <c r="A413" s="1" t="n">
+    <row r="413" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A413" s="1">
         <v>98</v>
       </c>
     </row>
-    <row r="414">
-      <c r="A414" s="1" t="n">
+    <row r="414" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A414" s="1">
         <v>99</v>
       </c>
     </row>
-    <row r="415">
-      <c r="A415" s="1" t="n">
+    <row r="415" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A415" s="1">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Run 20 choose 20 for related work comparison
</commit_message>
<xml_diff>
--- a/CIFAR_Global.xlsx
+++ b/CIFAR_Global.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ashleyau/Documents/PhD/Practical_Experiment/Finalised/Finalised_Algorithm_ResNet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30B1412-69DE-4744-9E6A-84CBBE4EC5BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB6B3852-47CC-874E-8D1E-0A211ADEADE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -82,10 +82,10 @@
     <t>Global Poisoning Accuracy</t>
   </si>
   <si>
-    <t>20 choose 10</t>
+    <t>From now on, I will use my algorithm's clustering and exclude conv</t>
   </si>
   <si>
-    <t>From now on, I will use my algorithm's clustering and exclude conv</t>
+    <t>20 choose 20</t>
   </si>
 </sst>
 </file>
@@ -192,10 +192,10 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -4385,10 +4385,10 @@
       <c r="H2" s="8"/>
       <c r="I2" s="8"/>
       <c r="J2" s="8"/>
-      <c r="Q2" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="R2" s="12"/>
+      <c r="Q2" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="R2" s="11"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -4421,14 +4421,14 @@
       <c r="J3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K3" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="11"/>
-      <c r="P3" s="11"/>
+      <c r="K3" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="12"/>
+      <c r="P3" s="12"/>
       <c r="Q3" s="4" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Ran my alg Dirichlet 100% clustering
</commit_message>
<xml_diff>
--- a/CIFAR_Global.xlsx
+++ b/CIFAR_Global.xlsx
@@ -8314,7 +8314,7 @@
         <v>0.0999</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0.1015875007843383</v>
+        <v>0.1451</v>
       </c>
     </row>
     <row r="6">
@@ -8385,7 +8385,7 @@
         <v>0.0999</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0.102340465583234</v>
+        <v>0.1776</v>
       </c>
     </row>
     <row r="7">
@@ -8456,7 +8456,7 @@
         <v>0.1529</v>
       </c>
       <c r="AJ7" t="n">
-        <v>0.1670326912216854</v>
+        <v>0.2412</v>
       </c>
     </row>
     <row r="8">
@@ -8527,7 +8527,7 @@
         <v>0.1115</v>
       </c>
       <c r="AJ8" t="n">
-        <v>0.2157871619501788</v>
+        <v>0.2753</v>
       </c>
     </row>
     <row r="9">
@@ -8598,7 +8598,7 @@
         <v>0.1121</v>
       </c>
       <c r="AJ9" t="n">
-        <v>0.1</v>
+        <v>0.3397</v>
       </c>
     </row>
     <row r="10">
@@ -8666,7 +8666,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0.1078</v>
+        <v>0.3398</v>
       </c>
     </row>
     <row r="11">
@@ -8734,7 +8734,7 @@
         <v>0.1122</v>
       </c>
       <c r="AJ11" t="n">
-        <v>0.1078</v>
+        <v>0.371</v>
       </c>
     </row>
     <row r="12">
@@ -8802,7 +8802,7 @@
         <v>0.1314</v>
       </c>
       <c r="AJ12" t="n">
-        <v>0.1078</v>
+        <v>0.3819</v>
       </c>
     </row>
     <row r="13">
@@ -8869,6 +8869,9 @@
       <c r="AI13" t="n">
         <v>0.1433</v>
       </c>
+      <c r="AJ13" t="n">
+        <v>0.3639</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -8934,6 +8937,9 @@
       <c r="AI14" t="n">
         <v>0.1074</v>
       </c>
+      <c r="AJ14" t="n">
+        <v>0.3883</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -8993,6 +8999,9 @@
       <c r="AI15" t="n">
         <v>0.107</v>
       </c>
+      <c r="AJ15" t="n">
+        <v>0.3739</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -9052,6 +9061,9 @@
       <c r="AI16" t="n">
         <v>0.1092</v>
       </c>
+      <c r="AJ16" t="n">
+        <v>0.4131</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -9111,6 +9123,9 @@
       <c r="AI17" t="n">
         <v>0.094</v>
       </c>
+      <c r="AJ17" t="n">
+        <v>0.4237</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -9170,6 +9185,9 @@
       <c r="AI18" t="n">
         <v>0.0944</v>
       </c>
+      <c r="AJ18" t="n">
+        <v>0.4181</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -9229,6 +9247,9 @@
       <c r="AI19" t="n">
         <v>0.0955</v>
       </c>
+      <c r="AJ19" t="n">
+        <v>0.4194</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -9288,6 +9309,9 @@
       <c r="AI20" t="n">
         <v>0.1</v>
       </c>
+      <c r="AJ20" t="n">
+        <v>0.4259</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -9347,6 +9371,9 @@
       <c r="AI21" t="n">
         <v>0.1228</v>
       </c>
+      <c r="AJ21" t="n">
+        <v>0.4252</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -9406,6 +9433,9 @@
       <c r="AI22" t="n">
         <v>0.1179</v>
       </c>
+      <c r="AJ22" t="n">
+        <v>0.4283</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -9465,6 +9495,9 @@
       <c r="AI23" t="n">
         <v>0.1213</v>
       </c>
+      <c r="AJ23" t="n">
+        <v>0.4113</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -9524,6 +9557,9 @@
       <c r="AI24" t="n">
         <v>0.09760000000000001</v>
       </c>
+      <c r="AJ24" t="n">
+        <v>0.4335</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -9583,6 +9619,9 @@
       <c r="AI25" t="n">
         <v>0.1238</v>
       </c>
+      <c r="AJ25" t="n">
+        <v>0.4277</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -9642,6 +9681,9 @@
       <c r="AI26" t="n">
         <v>0.1253</v>
       </c>
+      <c r="AJ26" t="n">
+        <v>0.4239</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -9701,6 +9743,9 @@
       <c r="AI27" t="n">
         <v>0.1174</v>
       </c>
+      <c r="AJ27" t="n">
+        <v>0.4287</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -9760,6 +9805,9 @@
       <c r="AI28" t="n">
         <v>0.1014</v>
       </c>
+      <c r="AJ28" t="n">
+        <v>0.4235</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -9819,6 +9867,9 @@
       <c r="AI29" t="n">
         <v>0.103</v>
       </c>
+      <c r="AJ29" t="n">
+        <v>0.4191</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -9878,6 +9929,9 @@
       <c r="AI30" t="n">
         <v>0.1132</v>
       </c>
+      <c r="AJ30" t="n">
+        <v>0.4324</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -9937,6 +9991,9 @@
       <c r="AI31" t="n">
         <v>0.1195</v>
       </c>
+      <c r="AJ31" t="n">
+        <v>0.4328</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -9996,6 +10053,9 @@
       <c r="AI32" t="n">
         <v>0.1026</v>
       </c>
+      <c r="AJ32" t="n">
+        <v>0.4318</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -10055,6 +10115,9 @@
       <c r="AI33" t="n">
         <v>0.1197</v>
       </c>
+      <c r="AJ33" t="n">
+        <v>0.4186</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -10114,6 +10177,9 @@
       <c r="AI34" t="n">
         <v>0.097</v>
       </c>
+      <c r="AJ34" t="n">
+        <v>0.4335</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -10173,6 +10239,9 @@
       <c r="AI35" t="n">
         <v>0.1</v>
       </c>
+      <c r="AJ35" t="n">
+        <v>0.437</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -10232,6 +10301,9 @@
       <c r="AI36" t="n">
         <v>0.1132</v>
       </c>
+      <c r="AJ36" t="n">
+        <v>0.4241</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -10291,6 +10363,9 @@
       <c r="AI37" t="n">
         <v>0.1135</v>
       </c>
+      <c r="AJ37" t="n">
+        <v>0.4346</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -10350,6 +10425,9 @@
       <c r="AI38" t="n">
         <v>0.1462</v>
       </c>
+      <c r="AJ38" t="n">
+        <v>0.4284</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -10409,6 +10487,9 @@
       <c r="AI39" t="n">
         <v>0.1282</v>
       </c>
+      <c r="AJ39" t="n">
+        <v>0.4229</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -10468,6 +10549,9 @@
       <c r="AI40" t="n">
         <v>0.1</v>
       </c>
+      <c r="AJ40" t="n">
+        <v>0.4185</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -10527,6 +10611,9 @@
       <c r="AI41" t="n">
         <v>0.121</v>
       </c>
+      <c r="AJ41" t="n">
+        <v>0.4242</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -10586,6 +10673,9 @@
       <c r="AI42" t="n">
         <v>0.1</v>
       </c>
+      <c r="AJ42" t="n">
+        <v>0.4321</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
@@ -10645,6 +10735,9 @@
       <c r="AI43" t="n">
         <v>0.1129</v>
       </c>
+      <c r="AJ43" t="n">
+        <v>0.4232</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -10704,6 +10797,9 @@
       <c r="AI44" t="n">
         <v>0.1</v>
       </c>
+      <c r="AJ44" t="n">
+        <v>0.4193</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
@@ -10763,6 +10859,9 @@
       <c r="AI45" t="n">
         <v>0.1446</v>
       </c>
+      <c r="AJ45" t="n">
+        <v>0.4272</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
@@ -10822,6 +10921,9 @@
       <c r="AI46" t="n">
         <v>0.1577</v>
       </c>
+      <c r="AJ46" t="n">
+        <v>0.4304</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
@@ -10881,6 +10983,9 @@
       <c r="AI47" t="n">
         <v>0.1</v>
       </c>
+      <c r="AJ47" t="n">
+        <v>0.431</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
@@ -10940,6 +11045,9 @@
       <c r="AI48" t="n">
         <v>0.1606</v>
       </c>
+      <c r="AJ48" t="n">
+        <v>0.4311</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -10999,6 +11107,9 @@
       <c r="AI49" t="n">
         <v>0.1216</v>
       </c>
+      <c r="AJ49" t="n">
+        <v>0.4364</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
@@ -11058,6 +11169,9 @@
       <c r="AI50" t="n">
         <v>0.1731</v>
       </c>
+      <c r="AJ50" t="n">
+        <v>0.4297</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
@@ -11117,6 +11231,9 @@
       <c r="AI51" t="n">
         <v>0.1475</v>
       </c>
+      <c r="AJ51" t="n">
+        <v>0.4325</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
@@ -11176,6 +11293,9 @@
       <c r="AI52" t="n">
         <v>0.2121</v>
       </c>
+      <c r="AJ52" t="n">
+        <v>0.439</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
@@ -11235,6 +11355,9 @@
       <c r="AI53" t="n">
         <v>0.1404</v>
       </c>
+      <c r="AJ53" t="n">
+        <v>0.4266</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
@@ -11294,6 +11417,9 @@
       <c r="AI54" t="n">
         <v>0.1</v>
       </c>
+      <c r="AJ54" t="n">
+        <v>0.4419</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
@@ -11353,6 +11479,9 @@
       <c r="AI55" t="n">
         <v>0.1</v>
       </c>
+      <c r="AJ55" t="n">
+        <v>0.4387</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -11412,6 +11541,9 @@
       <c r="AI56" t="n">
         <v>0.1787</v>
       </c>
+      <c r="AJ56" t="n">
+        <v>0.4397</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -11471,6 +11603,9 @@
       <c r="AI57" t="n">
         <v>0.1458</v>
       </c>
+      <c r="AJ57" t="n">
+        <v>0.4382</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
@@ -11530,6 +11665,9 @@
       <c r="AI58" t="n">
         <v>0.1687</v>
       </c>
+      <c r="AJ58" t="n">
+        <v>0.4371</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
@@ -11589,6 +11727,9 @@
       <c r="AI59" t="n">
         <v>0.1</v>
       </c>
+      <c r="AJ59" t="n">
+        <v>0.4341</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
@@ -11648,6 +11789,9 @@
       <c r="AI60" t="n">
         <v>0.1279</v>
       </c>
+      <c r="AJ60" t="n">
+        <v>0.4353</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -11707,6 +11851,9 @@
       <c r="AI61" t="n">
         <v>0.1275</v>
       </c>
+      <c r="AJ61" t="n">
+        <v>0.4351</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -11766,6 +11913,9 @@
       <c r="AI62" t="n">
         <v>0.1001</v>
       </c>
+      <c r="AJ62" t="n">
+        <v>0.4377</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
@@ -11825,6 +11975,9 @@
       <c r="AI63" t="n">
         <v>0.1215</v>
       </c>
+      <c r="AJ63" t="n">
+        <v>0.432</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
@@ -11884,6 +12037,9 @@
       <c r="AI64" t="n">
         <v>0.1</v>
       </c>
+      <c r="AJ64" t="n">
+        <v>0.4269</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
@@ -11943,6 +12099,9 @@
       <c r="AI65" t="n">
         <v>0.1</v>
       </c>
+      <c r="AJ65" t="n">
+        <v>0.4252</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
@@ -12002,6 +12161,9 @@
       <c r="AI66" t="n">
         <v>0.1438</v>
       </c>
+      <c r="AJ66" t="n">
+        <v>0.433</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
@@ -12061,6 +12223,9 @@
       <c r="AI67" t="n">
         <v>0.1539</v>
       </c>
+      <c r="AJ67" t="n">
+        <v>0.4323</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
@@ -12120,6 +12285,9 @@
       <c r="AI68" t="n">
         <v>0.1323</v>
       </c>
+      <c r="AJ68" t="n">
+        <v>0.4351</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
@@ -12179,6 +12347,9 @@
       <c r="AI69" t="n">
         <v>0.1294</v>
       </c>
+      <c r="AJ69" t="n">
+        <v>0.4403</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
@@ -12238,6 +12409,9 @@
       <c r="AI70" t="n">
         <v>0.155</v>
       </c>
+      <c r="AJ70" t="n">
+        <v>0.4417</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
@@ -12297,6 +12471,9 @@
       <c r="AI71" t="n">
         <v>0.1347</v>
       </c>
+      <c r="AJ71" t="n">
+        <v>0.4382</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
@@ -12356,6 +12533,9 @@
       <c r="AI72" t="n">
         <v>0.1642</v>
       </c>
+      <c r="AJ72" t="n">
+        <v>0.4358</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
@@ -12415,6 +12595,9 @@
       <c r="AI73" t="n">
         <v>0.1646</v>
       </c>
+      <c r="AJ73" t="n">
+        <v>0.437</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
@@ -12474,6 +12657,9 @@
       <c r="AI74" t="n">
         <v>0.1509</v>
       </c>
+      <c r="AJ74" t="n">
+        <v>0.44</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
@@ -12533,6 +12719,9 @@
       <c r="AI75" t="n">
         <v>0.1643</v>
       </c>
+      <c r="AJ75" t="n">
+        <v>0.4343</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
@@ -12592,6 +12781,9 @@
       <c r="AI76" t="n">
         <v>0.1</v>
       </c>
+      <c r="AJ76" t="n">
+        <v>0.419</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
@@ -12651,6 +12843,9 @@
       <c r="AI77" t="n">
         <v>0.1346</v>
       </c>
+      <c r="AJ77" t="n">
+        <v>0.4327</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
@@ -12710,6 +12905,9 @@
       <c r="AI78" t="n">
         <v>0.1402</v>
       </c>
+      <c r="AJ78" t="n">
+        <v>0.4404</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
@@ -12769,6 +12967,9 @@
       <c r="AI79" t="n">
         <v>0.1613</v>
       </c>
+      <c r="AJ79" t="n">
+        <v>0.443</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
@@ -12828,6 +13029,9 @@
       <c r="AI80" t="n">
         <v>0.138</v>
       </c>
+      <c r="AJ80" t="n">
+        <v>0.4426</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
@@ -12887,6 +13091,9 @@
       <c r="AI81" t="n">
         <v>0.1527</v>
       </c>
+      <c r="AJ81" t="n">
+        <v>0.443</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
@@ -12946,6 +13153,9 @@
       <c r="AI82" t="n">
         <v>0.1347</v>
       </c>
+      <c r="AJ82" t="n">
+        <v>0.4362</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
@@ -13005,6 +13215,9 @@
       <c r="AI83" t="n">
         <v>0.117</v>
       </c>
+      <c r="AJ83" t="n">
+        <v>0.44</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
@@ -13064,6 +13277,9 @@
       <c r="AI84" t="n">
         <v>0.1112</v>
       </c>
+      <c r="AJ84" t="n">
+        <v>0.4432</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
@@ -13123,6 +13339,9 @@
       <c r="AI85" t="n">
         <v>0.1</v>
       </c>
+      <c r="AJ85" t="n">
+        <v>0.4457</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
@@ -13182,6 +13401,9 @@
       <c r="AI86" t="n">
         <v>0.1444</v>
       </c>
+      <c r="AJ86" t="n">
+        <v>0.4423</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
@@ -13241,6 +13463,9 @@
       <c r="AI87" t="n">
         <v>0.1127</v>
       </c>
+      <c r="AJ87" t="n">
+        <v>0.4405</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
@@ -13300,6 +13525,9 @@
       <c r="AI88" t="n">
         <v>0.131</v>
       </c>
+      <c r="AJ88" t="n">
+        <v>0.4459</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
@@ -13359,6 +13587,9 @@
       <c r="AI89" t="n">
         <v>0.1833</v>
       </c>
+      <c r="AJ89" t="n">
+        <v>0.4325</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
@@ -13418,6 +13649,9 @@
       <c r="AI90" t="n">
         <v>0.2327</v>
       </c>
+      <c r="AJ90" t="n">
+        <v>0.4422</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
@@ -13477,6 +13711,9 @@
       <c r="AI91" t="n">
         <v>0.2327</v>
       </c>
+      <c r="AJ91" t="n">
+        <v>0.4332</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
@@ -13536,6 +13773,9 @@
       <c r="AI92" t="n">
         <v>0.1</v>
       </c>
+      <c r="AJ92" t="n">
+        <v>0.442</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
@@ -13595,6 +13835,9 @@
       <c r="AI93" t="n">
         <v>0.1949</v>
       </c>
+      <c r="AJ93" t="n">
+        <v>0.4348</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
@@ -13654,6 +13897,9 @@
       <c r="AI94" t="n">
         <v>0.1447</v>
       </c>
+      <c r="AJ94" t="n">
+        <v>0.4344</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
@@ -13712,6 +13958,9 @@
       </c>
       <c r="AI95" t="n">
         <v>0.1</v>
+      </c>
+      <c r="AJ95" t="n">
+        <v>0.435</v>
       </c>
     </row>
     <row r="96">
@@ -14348,7 +14597,7 @@
         <v>0.9333333333333333</v>
       </c>
       <c r="AJ108" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="109">
@@ -14412,7 +14661,7 @@
         <v>1</v>
       </c>
       <c r="AJ109" t="n">
-        <v>0.5333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="110">
@@ -14476,7 +14725,7 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="AJ110" t="n">
-        <v>0.6</v>
+        <v>0.7692307692307693</v>
       </c>
     </row>
     <row r="111">
@@ -14540,7 +14789,7 @@
         <v>0.8181818181818182</v>
       </c>
       <c r="AJ111" t="n">
-        <v>0.7692307692307693</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="112">
@@ -14604,7 +14853,7 @@
         <v>0.8181818181818182</v>
       </c>
       <c r="AJ112" t="n">
-        <v>1</v>
+        <v>0.7857142857142857</v>
       </c>
     </row>
     <row r="113">
@@ -14665,7 +14914,7 @@
         <v>0.7272727272727273</v>
       </c>
       <c r="AJ113" t="n">
-        <v>0.6363636363636364</v>
+        <v>0.8181818181818182</v>
       </c>
     </row>
     <row r="114">
@@ -14726,7 +14975,7 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="AJ114" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.6923076923076923</v>
       </c>
     </row>
     <row r="115">
@@ -14786,6 +15035,9 @@
       <c r="AI115" t="n">
         <v>0.7</v>
       </c>
+      <c r="AJ115" t="n">
+        <v>0.8333333333333334</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
@@ -14844,6 +15096,9 @@
       <c r="AI116" t="n">
         <v>0.7</v>
       </c>
+      <c r="AJ116" t="n">
+        <v>0.8461538461538461</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
@@ -14902,6 +15157,9 @@
       <c r="AI117" t="n">
         <v>0.7272727272727273</v>
       </c>
+      <c r="AJ117" t="n">
+        <v>0.3333333333333333</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
@@ -14954,6 +15212,9 @@
       <c r="AI118" t="n">
         <v>0.7777777777777778</v>
       </c>
+      <c r="AJ118" t="n">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
@@ -15006,6 +15267,9 @@
       <c r="AI119" t="n">
         <v>0.8333333333333334</v>
       </c>
+      <c r="AJ119" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
@@ -15058,6 +15322,9 @@
       <c r="AI120" t="n">
         <v>0.7272727272727273</v>
       </c>
+      <c r="AJ120" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
@@ -15110,6 +15377,9 @@
       <c r="AI121" t="n">
         <v>0.9</v>
       </c>
+      <c r="AJ121" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
@@ -15162,6 +15432,9 @@
       <c r="AI122" t="n">
         <v>0.9166666666666666</v>
       </c>
+      <c r="AJ122" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
@@ -15214,6 +15487,9 @@
       <c r="AI123" t="n">
         <v>0.9090909090909091</v>
       </c>
+      <c r="AJ123" t="n">
+        <v>0.7777777777777778</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
@@ -15266,6 +15542,9 @@
       <c r="AI124" t="n">
         <v>0.6666666666666666</v>
       </c>
+      <c r="AJ124" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
@@ -15318,6 +15597,9 @@
       <c r="AI125" t="n">
         <v>0.8181818181818182</v>
       </c>
+      <c r="AJ125" t="n">
+        <v>0.8181818181818182</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
@@ -15370,6 +15652,9 @@
       <c r="AI126" t="n">
         <v>1</v>
       </c>
+      <c r="AJ126" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
@@ -15422,6 +15707,9 @@
       <c r="AI127" t="n">
         <v>0.6428571428571429</v>
       </c>
+      <c r="AJ127" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
@@ -15474,6 +15762,9 @@
       <c r="AI128" t="n">
         <v>0.9</v>
       </c>
+      <c r="AJ128" t="n">
+        <v>0.7777777777777778</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
@@ -15526,6 +15817,9 @@
       <c r="AI129" t="n">
         <v>0.8</v>
       </c>
+      <c r="AJ129" t="n">
+        <v>0.7142857142857143</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
@@ -15578,6 +15872,9 @@
       <c r="AI130" t="n">
         <v>0.8</v>
       </c>
+      <c r="AJ130" t="n">
+        <v>0.5454545454545454</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
@@ -15630,6 +15927,9 @@
       <c r="AI131" t="n">
         <v>0.875</v>
       </c>
+      <c r="AJ131" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
@@ -15682,6 +15982,9 @@
       <c r="AI132" t="n">
         <v>0.9090909090909091</v>
       </c>
+      <c r="AJ132" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
@@ -15734,6 +16037,9 @@
       <c r="AI133" t="n">
         <v>0.8333333333333334</v>
       </c>
+      <c r="AJ133" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
@@ -15786,6 +16092,9 @@
       <c r="AI134" t="n">
         <v>0.8888888888888888</v>
       </c>
+      <c r="AJ134" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
@@ -15838,6 +16147,9 @@
       <c r="AI135" t="n">
         <v>0.8181818181818182</v>
       </c>
+      <c r="AJ135" t="n">
+        <v>0.7777777777777778</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
@@ -15890,6 +16202,9 @@
       <c r="AI136" t="n">
         <v>0.9</v>
       </c>
+      <c r="AJ136" t="n">
+        <v>0.4285714285714285</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
@@ -15942,6 +16257,9 @@
       <c r="AI137" t="n">
         <v>0.875</v>
       </c>
+      <c r="AJ137" t="n">
+        <v>0.8181818181818182</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
@@ -15994,6 +16312,9 @@
       <c r="AI138" t="n">
         <v>1</v>
       </c>
+      <c r="AJ138" t="n">
+        <v>0.7142857142857143</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
@@ -16046,6 +16367,9 @@
       <c r="AI139" t="n">
         <v>0.8571428571428571</v>
       </c>
+      <c r="AJ139" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
@@ -16098,6 +16422,9 @@
       <c r="AI140" t="n">
         <v>1</v>
       </c>
+      <c r="AJ140" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
@@ -16150,6 +16477,9 @@
       <c r="AI141" t="n">
         <v>1</v>
       </c>
+      <c r="AJ141" t="n">
+        <v>0.08333333333333333</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
@@ -16202,6 +16532,9 @@
       <c r="AI142" t="n">
         <v>0.8888888888888888</v>
       </c>
+      <c r="AJ142" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
@@ -16254,6 +16587,9 @@
       <c r="AI143" t="n">
         <v>1</v>
       </c>
+      <c r="AJ143" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
@@ -16306,6 +16642,9 @@
       <c r="AI144" t="n">
         <v>1</v>
       </c>
+      <c r="AJ144" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
@@ -16358,6 +16697,9 @@
       <c r="AI145" t="n">
         <v>0.5</v>
       </c>
+      <c r="AJ145" t="n">
+        <v>0.4285714285714285</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
@@ -16410,6 +16752,9 @@
       <c r="AI146" t="n">
         <v>0.5</v>
       </c>
+      <c r="AJ146" t="n">
+        <v>0.3333333333333333</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
@@ -16462,6 +16807,9 @@
       <c r="AI147" t="n">
         <v>1</v>
       </c>
+      <c r="AJ147" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
@@ -16514,6 +16862,9 @@
       <c r="AI148" t="n">
         <v>0.8</v>
       </c>
+      <c r="AJ148" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
@@ -16566,6 +16917,9 @@
       <c r="AI149" t="n">
         <v>1</v>
       </c>
+      <c r="AJ149" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
@@ -16618,6 +16972,9 @@
       <c r="AI150" t="n">
         <v>1</v>
       </c>
+      <c r="AJ150" t="n">
+        <v>0.6666666666666666</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
@@ -16670,6 +17027,9 @@
       <c r="AI151" t="n">
         <v>0.6666666666666666</v>
       </c>
+      <c r="AJ151" t="n">
+        <v>0.3636363636363636</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
@@ -16722,6 +17082,9 @@
       <c r="AI152" t="n">
         <v>0.8333333333333334</v>
       </c>
+      <c r="AJ152" t="n">
+        <v>0.6363636363636364</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
@@ -16774,6 +17137,9 @@
       <c r="AI153" t="n">
         <v>1</v>
       </c>
+      <c r="AJ153" t="n">
+        <v>0.625</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
@@ -16826,6 +17192,9 @@
       <c r="AI154" t="n">
         <v>1</v>
       </c>
+      <c r="AJ154" t="n">
+        <v>0.7777777777777778</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
@@ -16878,6 +17247,9 @@
       <c r="AI155" t="n">
         <v>0.8571428571428571</v>
       </c>
+      <c r="AJ155" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
@@ -16930,6 +17302,9 @@
       <c r="AI156" t="n">
         <v>1</v>
       </c>
+      <c r="AJ156" t="n">
+        <v>0.5714285714285714</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="n">
@@ -16982,6 +17357,9 @@
       <c r="AI157" t="n">
         <v>0.8571428571428571</v>
       </c>
+      <c r="AJ157" t="n">
+        <v>0.6666666666666666</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="n">
@@ -17034,6 +17412,9 @@
       <c r="AI158" t="n">
         <v>0.8</v>
       </c>
+      <c r="AJ158" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="n">
@@ -17086,6 +17467,9 @@
       <c r="AI159" t="n">
         <v>1</v>
       </c>
+      <c r="AJ159" t="n">
+        <v>0.3333333333333333</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="n">
@@ -17138,6 +17522,9 @@
       <c r="AI160" t="n">
         <v>0.625</v>
       </c>
+      <c r="AJ160" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="n">
@@ -17190,6 +17577,9 @@
       <c r="AI161" t="n">
         <v>0.5555555555555556</v>
       </c>
+      <c r="AJ161" t="n">
+        <v>0.5555555555555556</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
@@ -17242,6 +17632,9 @@
       <c r="AI162" t="n">
         <v>0.75</v>
       </c>
+      <c r="AJ162" t="n">
+        <v>0.6363636363636364</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="n">
@@ -17294,6 +17687,9 @@
       <c r="AI163" t="n">
         <v>0.8</v>
       </c>
+      <c r="AJ163" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="n">
@@ -17346,6 +17742,9 @@
       <c r="AI164" t="n">
         <v>0.8571428571428571</v>
       </c>
+      <c r="AJ164" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="n">
@@ -17398,6 +17797,9 @@
       <c r="AI165" t="n">
         <v>1</v>
       </c>
+      <c r="AJ165" t="n">
+        <v>0.3636363636363636</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="n">
@@ -17450,6 +17852,9 @@
       <c r="AI166" t="n">
         <v>0.75</v>
       </c>
+      <c r="AJ166" t="n">
+        <v>0.625</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="n">
@@ -17502,6 +17907,9 @@
       <c r="AI167" t="n">
         <v>1</v>
       </c>
+      <c r="AJ167" t="n">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="n">
@@ -17554,6 +17962,9 @@
       <c r="AI168" t="n">
         <v>1</v>
       </c>
+      <c r="AJ168" t="n">
+        <v>0.5555555555555556</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="n">
@@ -17606,6 +18017,9 @@
       <c r="AI169" t="n">
         <v>1</v>
       </c>
+      <c r="AJ169" t="n">
+        <v>0.2222222222222222</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="n">
@@ -17658,6 +18072,9 @@
       <c r="AI170" t="n">
         <v>0.75</v>
       </c>
+      <c r="AJ170" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="1" t="n">
@@ -17710,6 +18127,9 @@
       <c r="AI171" t="n">
         <v>1</v>
       </c>
+      <c r="AJ171" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="n">
@@ -17762,6 +18182,9 @@
       <c r="AI172" t="n">
         <v>1</v>
       </c>
+      <c r="AJ172" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="n">
@@ -17814,6 +18237,9 @@
       <c r="AI173" t="n">
         <v>0.8</v>
       </c>
+      <c r="AJ173" t="n">
+        <v>0.5555555555555556</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="n">
@@ -17866,6 +18292,9 @@
       <c r="AI174" t="n">
         <v>1</v>
       </c>
+      <c r="AJ174" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="n">
@@ -17918,6 +18347,9 @@
       <c r="AI175" t="n">
         <v>1</v>
       </c>
+      <c r="AJ175" t="n">
+        <v>0.2727272727272727</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="1" t="n">
@@ -17970,6 +18402,9 @@
       <c r="AI176" t="n">
         <v>1</v>
       </c>
+      <c r="AJ176" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="1" t="n">
@@ -18022,6 +18457,9 @@
       <c r="AI177" t="n">
         <v>1</v>
       </c>
+      <c r="AJ177" t="n">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="n">
@@ -18074,6 +18512,9 @@
       <c r="AI178" t="n">
         <v>0.8</v>
       </c>
+      <c r="AJ178" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="n">
@@ -18126,6 +18567,9 @@
       <c r="AI179" t="n">
         <v>1</v>
       </c>
+      <c r="AJ179" t="n">
+        <v>0.7142857142857143</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="n">
@@ -18178,6 +18622,9 @@
       <c r="AI180" t="n">
         <v>0.5</v>
       </c>
+      <c r="AJ180" t="n">
+        <v>0.2857142857142857</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="n">
@@ -18230,6 +18677,9 @@
       <c r="AI181" t="n">
         <v>1</v>
       </c>
+      <c r="AJ181" t="n">
+        <v>0.5714285714285714</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="n">
@@ -18282,6 +18732,9 @@
       <c r="AI182" t="n">
         <v>1</v>
       </c>
+      <c r="AJ182" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="n">
@@ -18334,6 +18787,9 @@
       <c r="AI183" t="n">
         <v>1</v>
       </c>
+      <c r="AJ183" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="n">
@@ -18386,6 +18842,9 @@
       <c r="AI184" t="n">
         <v>1</v>
       </c>
+      <c r="AJ184" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="n">
@@ -18438,6 +18897,9 @@
       <c r="AI185" t="n">
         <v>1</v>
       </c>
+      <c r="AJ185" t="n">
+        <v>0.5714285714285714</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="n">
@@ -18490,6 +18952,9 @@
       <c r="AI186" t="n">
         <v>1</v>
       </c>
+      <c r="AJ186" t="n">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="n">
@@ -18542,6 +19007,9 @@
       <c r="AI187" t="n">
         <v>1</v>
       </c>
+      <c r="AJ187" t="n">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="n">
@@ -18594,6 +19062,9 @@
       <c r="AI188" t="n">
         <v>1</v>
       </c>
+      <c r="AJ188" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="n">
@@ -18646,6 +19117,9 @@
       <c r="AI189" t="n">
         <v>1</v>
       </c>
+      <c r="AJ189" t="n">
+        <v>0.4285714285714285</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="n">
@@ -18698,6 +19172,9 @@
       <c r="AI190" t="n">
         <v>1</v>
       </c>
+      <c r="AJ190" t="n">
+        <v>0.375</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="n">
@@ -18750,6 +19227,9 @@
       <c r="AI191" t="n">
         <v>0.4</v>
       </c>
+      <c r="AJ191" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="n">
@@ -18802,6 +19282,9 @@
       <c r="AI192" t="n">
         <v>0.75</v>
       </c>
+      <c r="AJ192" t="n">
+        <v>0.6666666666666666</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="n">
@@ -18854,6 +19337,9 @@
       <c r="AI193" t="n">
         <v>1</v>
       </c>
+      <c r="AJ193" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="n">
@@ -18903,6 +19389,9 @@
       <c r="AH194" t="n">
         <v>0.6</v>
       </c>
+      <c r="AJ194" t="n">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="n">
@@ -18955,6 +19444,9 @@
       <c r="AI195" t="n">
         <v>1</v>
       </c>
+      <c r="AJ195" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="n">
@@ -19007,6 +19499,9 @@
       <c r="AI196" t="n">
         <v>1</v>
       </c>
+      <c r="AJ196" t="n">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="n">
@@ -19059,6 +19554,9 @@
       <c r="AI197" t="n">
         <v>1</v>
       </c>
+      <c r="AJ197" t="n">
+        <v>0.625</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="n">
@@ -19110,6 +19608,9 @@
       </c>
       <c r="AI198" t="n">
         <v>0.8333333333333334</v>
+      </c>
+      <c r="AJ198" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="199">
@@ -19684,7 +20185,7 @@
         <v>0.9658857142857143</v>
       </c>
       <c r="AJ212" t="n">
-        <v>0.9276857142857143</v>
+        <v>0.936111111111111</v>
       </c>
     </row>
     <row r="213">
@@ -19748,7 +20249,7 @@
         <v>0.8468571428571429</v>
       </c>
       <c r="AJ213" t="n">
-        <v>0.9668428571428571</v>
+        <v>0.9478500000000001</v>
       </c>
     </row>
     <row r="214">
@@ -19812,7 +20313,7 @@
         <v>0.8858333333333334</v>
       </c>
       <c r="AJ214" t="n">
-        <v>0.9774428571428572</v>
+        <v>0.9270400000000001</v>
       </c>
     </row>
     <row r="215">
@@ -19876,7 +20377,7 @@
         <v>0.9863166666666666</v>
       </c>
       <c r="AJ215" t="n">
-        <v>0.8854875</v>
+        <v>0.9197142857142857</v>
       </c>
     </row>
     <row r="216">
@@ -19939,10 +20440,8 @@
       <c r="AI216" t="n">
         <v>0.8197333333333333</v>
       </c>
-      <c r="AJ216" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="AJ216" t="n">
+        <v>0.9202250000000001</v>
       </c>
     </row>
     <row r="217">
@@ -20003,7 +20502,7 @@
         <v>0.9927142857142855</v>
       </c>
       <c r="AJ217" t="n">
-        <v>0.3832714285714286</v>
+        <v>0.9224333333333333</v>
       </c>
     </row>
     <row r="218">
@@ -20064,7 +20563,7 @@
         <v>0.9982200000000001</v>
       </c>
       <c r="AJ218" t="n">
-        <v>0.274</v>
+        <v>0.8960333333333333</v>
       </c>
     </row>
     <row r="219">
@@ -20126,6 +20625,9 @@
       <c r="AI219" t="n">
         <v>0.8679625</v>
       </c>
+      <c r="AJ219" t="n">
+        <v>0.9205</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="n">
@@ -20186,6 +20688,9 @@
       <c r="AI220" t="n">
         <v>0.8760250000000001</v>
       </c>
+      <c r="AJ220" t="n">
+        <v>0.8922</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="n">
@@ -20244,6 +20749,9 @@
       <c r="AI221" t="n">
         <v>0.9856285714285714</v>
       </c>
+      <c r="AJ221" t="n">
+        <v>0.8915166666666666</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="n">
@@ -20296,6 +20804,9 @@
       <c r="AI222" t="n">
         <v>0.9943375</v>
       </c>
+      <c r="AJ222" t="n">
+        <v>0.9132444444444445</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="n">
@@ -20348,6 +20859,9 @@
       <c r="AI223" t="n">
         <v>0.8468199999999999</v>
       </c>
+      <c r="AJ223" t="n">
+        <v>0.8975799999999999</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="1" t="n">
@@ -20400,6 +20914,9 @@
       <c r="AI224" t="n">
         <v>0.9959571428571429</v>
       </c>
+      <c r="AJ224" t="n">
+        <v>0.86815</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="n">
@@ -20452,6 +20969,9 @@
       <c r="AI225" t="n">
         <v>0.989</v>
       </c>
+      <c r="AJ225" t="n">
+        <v>0.8668142857142858</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="n">
@@ -20504,6 +21024,9 @@
       <c r="AI226" t="n">
         <v>0.97255</v>
       </c>
+      <c r="AJ226" t="n">
+        <v>0.8794999999999999</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="n">
@@ -20556,6 +21079,9 @@
       <c r="AI227" t="n">
         <v>0.81014</v>
       </c>
+      <c r="AJ227" t="n">
+        <v>0.8617833333333335</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="1" t="n">
@@ -20608,6 +21134,9 @@
       <c r="AI228" t="n">
         <v>0.8912333333333334</v>
       </c>
+      <c r="AJ228" t="n">
+        <v>0.8654000000000001</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="1" t="n">
@@ -20660,6 +21189,9 @@
       <c r="AI229" t="n">
         <v>0.9319833333333333</v>
       </c>
+      <c r="AJ229" t="n">
+        <v>0.893925</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="1" t="n">
@@ -20712,6 +21244,9 @@
       <c r="AI230" t="n">
         <v>0.9897333333333332</v>
       </c>
+      <c r="AJ230" t="n">
+        <v>0.8520142857142857</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="1" t="n">
@@ -20764,6 +21299,9 @@
       <c r="AI231" t="n">
         <v>0.9861333333333334</v>
       </c>
+      <c r="AJ231" t="n">
+        <v>0.8441599999999999</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="1" t="n">
@@ -20816,6 +21354,9 @@
       <c r="AI232" t="n">
         <v>0.9921833333333333</v>
       </c>
+      <c r="AJ232" t="n">
+        <v>0.8473000000000001</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="1" t="n">
@@ -20868,6 +21409,9 @@
       <c r="AI233" t="n">
         <v>0.9827285714285715</v>
       </c>
+      <c r="AJ233" t="n">
+        <v>0.8876000000000001</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="1" t="n">
@@ -20920,6 +21464,9 @@
       <c r="AI234" t="n">
         <v>0.8867714285714285</v>
       </c>
+      <c r="AJ234" t="n">
+        <v>0.8675250000000001</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="1" t="n">
@@ -20972,6 +21519,9 @@
       <c r="AI235" t="n">
         <v>0.9881375</v>
       </c>
+      <c r="AJ235" t="n">
+        <v>0.877</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="1" t="n">
@@ -21024,6 +21574,9 @@
       <c r="AI236" t="n">
         <v>0.9941000000000001</v>
       </c>
+      <c r="AJ236" t="n">
+        <v>0.8574857142857143</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="1" t="n">
@@ -21076,6 +21629,9 @@
       <c r="AI237" t="n">
         <v>0.9599800000000001</v>
       </c>
+      <c r="AJ237" t="n">
+        <v>0.85584</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="1" t="n">
@@ -21128,6 +21684,9 @@
       <c r="AI238" t="n">
         <v>0.9938285714285714</v>
       </c>
+      <c r="AJ238" t="n">
+        <v>0.8513300000000001</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="1" t="n">
@@ -21180,6 +21739,9 @@
       <c r="AI239" t="n">
         <v>0.9918833333333333</v>
       </c>
+      <c r="AJ239" t="n">
+        <v>0.8556833333333334</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="n">
@@ -21232,6 +21794,9 @@
       <c r="AI240" t="n">
         <v>0.9929</v>
       </c>
+      <c r="AJ240" t="n">
+        <v>0.863625</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="n">
@@ -21284,6 +21849,9 @@
       <c r="AI241" t="n">
         <v>0.9923124999999999</v>
       </c>
+      <c r="AJ241" t="n">
+        <v>0.8387500000000001</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="1" t="n">
@@ -21336,6 +21904,9 @@
       <c r="AI242" t="n">
         <v>0.8736555555555554</v>
       </c>
+      <c r="AJ242" t="n">
+        <v>0.8280750000000001</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="n">
@@ -21388,6 +21959,9 @@
       <c r="AI243" t="n">
         <v>0.8641999999999999</v>
       </c>
+      <c r="AJ243" t="n">
+        <v>0.87582</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="1" t="n">
@@ -21440,6 +22014,9 @@
       <c r="AI244" t="n">
         <v>0.6879</v>
       </c>
+      <c r="AJ244" t="n">
+        <v>0.8493857142857143</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="n">
@@ -21492,6 +22069,9 @@
       <c r="AI245" t="n">
         <v>0.99176</v>
       </c>
+      <c r="AJ245" t="n">
+        <v>0.8000666666666666</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="1" t="n">
@@ -21544,6 +22124,9 @@
       <c r="AI246" t="n">
         <v>0.9963142857142858</v>
       </c>
+      <c r="AJ246" t="n">
+        <v>0.8438428571428572</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="1" t="n">
@@ -21596,6 +22179,9 @@
       <c r="AI247" t="n">
         <v>0.9844714285714286</v>
       </c>
+      <c r="AJ247" t="n">
+        <v>0.8600000000000001</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="1" t="n">
@@ -21648,6 +22234,9 @@
       <c r="AI248" t="n">
         <v>0.8516285714285715</v>
       </c>
+      <c r="AJ248" t="n">
+        <v>0.84902</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="1" t="n">
@@ -21700,6 +22289,9 @@
       <c r="AI249" t="n">
         <v>0.9866333333333334</v>
       </c>
+      <c r="AJ249" t="n">
+        <v>0.8609499999999999</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="1" t="n">
@@ -21752,6 +22344,9 @@
       <c r="AI250" t="n">
         <v>0.8845333333333333</v>
       </c>
+      <c r="AJ250" t="n">
+        <v>0.86485</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="1" t="n">
@@ -21804,6 +22399,9 @@
       <c r="AI251" t="n">
         <v>0.69035</v>
       </c>
+      <c r="AJ251" t="n">
+        <v>0.85972</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="1" t="n">
@@ -21856,6 +22454,9 @@
       <c r="AI252" t="n">
         <v>0.7249727272727272</v>
       </c>
+      <c r="AJ252" t="n">
+        <v>0.8108714285714286</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="1" t="n">
@@ -21908,6 +22509,9 @@
       <c r="AI253" t="n">
         <v>0.8805222222222223</v>
       </c>
+      <c r="AJ253" t="n">
+        <v>0.8481099999999999</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="1" t="n">
@@ -21960,6 +22564,9 @@
       <c r="AI254" t="n">
         <v>0.79576</v>
       </c>
+      <c r="AJ254" t="n">
+        <v>0.8564666666666666</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="1" t="n">
@@ -22012,6 +22619,9 @@
       <c r="AI255" t="n">
         <v>0.6875538461538462</v>
       </c>
+      <c r="AJ255" t="n">
+        <v>0.8437749999999999</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="1" t="n">
@@ -22064,6 +22674,9 @@
       <c r="AI256" t="n">
         <v>0.79863</v>
       </c>
+      <c r="AJ256" t="n">
+        <v>0.810275</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="1" t="n">
@@ -22116,6 +22729,9 @@
       <c r="AI257" t="n">
         <v>0.6415727272727273</v>
       </c>
+      <c r="AJ257" t="n">
+        <v>0.8225857142857144</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="1" t="n">
@@ -22168,6 +22784,9 @@
       <c r="AI258" t="n">
         <v>0.69429</v>
       </c>
+      <c r="AJ258" t="n">
+        <v>0.8418499999999999</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="1" t="n">
@@ -22220,6 +22839,9 @@
       <c r="AI259" t="n">
         <v>0.6539555555555556</v>
       </c>
+      <c r="AJ259" t="n">
+        <v>0.8089888888888888</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="1" t="n">
@@ -22272,6 +22894,9 @@
       <c r="AI260" t="n">
         <v>0.65415</v>
       </c>
+      <c r="AJ260" t="n">
+        <v>0.8360624999999999</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="1" t="n">
@@ -22324,6 +22949,9 @@
       <c r="AI261" t="n">
         <v>0.8725222222222222</v>
       </c>
+      <c r="AJ261" t="n">
+        <v>0.8252166666666666</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="1" t="n">
@@ -22376,6 +23004,9 @@
       <c r="AI262" t="n">
         <v>0.7095181818181818</v>
       </c>
+      <c r="AJ262" t="n">
+        <v>0.8382499999999999</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="1" t="n">
@@ -22428,6 +23059,9 @@
       <c r="AI263" t="n">
         <v>0.8658857142857144</v>
       </c>
+      <c r="AJ263" t="n">
+        <v>0.8127666666666666</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="1" t="n">
@@ -22480,6 +23114,9 @@
       <c r="AI264" t="n">
         <v>0.5676285714285714</v>
       </c>
+      <c r="AJ264" t="n">
+        <v>0.8460599999999999</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="1" t="n">
@@ -22532,6 +23169,9 @@
       <c r="AI265" t="n">
         <v>0.4132000000000001</v>
       </c>
+      <c r="AJ265" t="n">
+        <v>0.8023166666666667</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="1" t="n">
@@ -22584,6 +23224,9 @@
       <c r="AI266" t="n">
         <v>0.7401</v>
       </c>
+      <c r="AJ266" t="n">
+        <v>0.8532000000000001</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="1" t="n">
@@ -22636,6 +23279,9 @@
       <c r="AI267" t="n">
         <v>0.6399181818181819</v>
       </c>
+      <c r="AJ267" t="n">
+        <v>0.86492</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="1" t="n">
@@ -22688,6 +23334,9 @@
       <c r="AI268" t="n">
         <v>0.4583555555555556</v>
       </c>
+      <c r="AJ268" t="n">
+        <v>0.8317600000000001</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="1" t="n">
@@ -22740,6 +23389,9 @@
       <c r="AI269" t="n">
         <v>0.9101500000000001</v>
       </c>
+      <c r="AJ269" t="n">
+        <v>0.8783500000000001</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="1" t="n">
@@ -22792,6 +23444,9 @@
       <c r="AI270" t="n">
         <v>0.6957083333333333</v>
       </c>
+      <c r="AJ270" t="n">
+        <v>0.8458571428571429</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
@@ -22844,6 +23499,9 @@
       <c r="AI271" t="n">
         <v>0.7372083333333332</v>
       </c>
+      <c r="AJ271" t="n">
+        <v>0.8659</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
@@ -22896,6 +23554,9 @@
       <c r="AI272" t="n">
         <v>0.7539166666666667</v>
       </c>
+      <c r="AJ272" t="n">
+        <v>0.8267166666666667</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
@@ -22948,6 +23609,9 @@
       <c r="AI273" t="n">
         <v>0.4423727272727273</v>
       </c>
+      <c r="AJ273" t="n">
+        <v>0.8344499999999999</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
@@ -23000,6 +23664,9 @@
       <c r="AI274" t="n">
         <v>0.6609333333333333</v>
       </c>
+      <c r="AJ274" t="n">
+        <v>0.8324142857142857</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
@@ -23052,6 +23719,9 @@
       <c r="AI275" t="n">
         <v>0.654875</v>
       </c>
+      <c r="AJ275" t="n">
+        <v>0.8711666666666668</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
@@ -23104,6 +23774,9 @@
       <c r="AI276" t="n">
         <v>0.723509090909091</v>
       </c>
+      <c r="AJ276" t="n">
+        <v>0.8751599999999999</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
@@ -23156,6 +23829,9 @@
       <c r="AI277" t="n">
         <v>0.6337545454545453</v>
       </c>
+      <c r="AJ277" t="n">
+        <v>0.8717</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
@@ -23208,6 +23884,9 @@
       <c r="AI278" t="n">
         <v>0.6305181818181818</v>
       </c>
+      <c r="AJ278" t="n">
+        <v>0.8425428571428571</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
@@ -23260,6 +23939,9 @@
       <c r="AI279" t="n">
         <v>0.5742399999999999</v>
       </c>
+      <c r="AJ279" t="n">
+        <v>0.8514250000000001</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
@@ -23312,6 +23994,9 @@
       <c r="AI280" t="n">
         <v>0.6294818181818183</v>
       </c>
+      <c r="AJ280" t="n">
+        <v>0.8547399999999999</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
@@ -23364,6 +24049,9 @@
       <c r="AI281" t="n">
         <v>0.5350384615384616</v>
       </c>
+      <c r="AJ281" t="n">
+        <v>0.8309799999999999</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="n">
@@ -23416,6 +24104,9 @@
       <c r="AI282" t="n">
         <v>0.5364</v>
       </c>
+      <c r="AJ282" t="n">
+        <v>0.8591499999999999</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
@@ -23468,6 +24159,9 @@
       <c r="AI283" t="n">
         <v>0.6825307692307692</v>
       </c>
+      <c r="AJ283" t="n">
+        <v>0.8156625000000001</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
@@ -23520,6 +24214,9 @@
       <c r="AI284" t="n">
         <v>0.6116714285714286</v>
       </c>
+      <c r="AJ284" t="n">
+        <v>0.815625</v>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
@@ -23572,6 +24269,9 @@
       <c r="AI285" t="n">
         <v>0.4963928571428571</v>
       </c>
+      <c r="AJ285" t="n">
+        <v>0.8539875</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
@@ -23624,6 +24324,9 @@
       <c r="AI286" t="n">
         <v>0.49677</v>
       </c>
+      <c r="AJ286" t="n">
+        <v>0.8410000000000001</v>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
@@ -23676,6 +24379,9 @@
       <c r="AI287" t="n">
         <v>0.4635083333333332</v>
       </c>
+      <c r="AJ287" t="n">
+        <v>0.83048</v>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
@@ -23728,6 +24434,9 @@
       <c r="AI288" t="n">
         <v>0.7629461538461538</v>
       </c>
+      <c r="AJ288" t="n">
+        <v>0.7994285714285715</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
@@ -23780,6 +24489,9 @@
       <c r="AI289" t="n">
         <v>0.5772499999999999</v>
       </c>
+      <c r="AJ289" t="n">
+        <v>0.8455625000000001</v>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
@@ -23832,6 +24544,9 @@
       <c r="AI290" t="n">
         <v>0.6123000000000001</v>
       </c>
+      <c r="AJ290" t="n">
+        <v>0.82806</v>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
@@ -23884,6 +24599,9 @@
       <c r="AI291" t="n">
         <v>0.584790909090909</v>
       </c>
+      <c r="AJ291" t="n">
+        <v>0.82032</v>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
@@ -23936,6 +24654,9 @@
       <c r="AI292" t="n">
         <v>0.4132416666666667</v>
       </c>
+      <c r="AJ292" t="n">
+        <v>0.8719571428571429</v>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="n">
@@ -23988,6 +24709,9 @@
       <c r="AI293" t="n">
         <v>0.579175</v>
       </c>
+      <c r="AJ293" t="n">
+        <v>0.8448749999999999</v>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="n">
@@ -24040,6 +24764,9 @@
       <c r="AI294" t="n">
         <v>0.6215363636363637</v>
       </c>
+      <c r="AJ294" t="n">
+        <v>0.8622</v>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="n">
@@ -24092,6 +24819,9 @@
       <c r="AI295" t="n">
         <v>0.4937300000000001</v>
       </c>
+      <c r="AJ295" t="n">
+        <v>0.8437</v>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="n">
@@ -24144,6 +24874,9 @@
       <c r="AI296" t="n">
         <v>0.5772666666666667</v>
       </c>
+      <c r="AJ296" t="n">
+        <v>0.8250166666666666</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="n">
@@ -24196,6 +24929,9 @@
       <c r="AI297" t="n">
         <v>0.6120181818181818</v>
       </c>
+      <c r="AJ297" t="n">
+        <v>0.8578571428571429</v>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="n">
@@ -24245,6 +24981,9 @@
       <c r="AH298" t="n">
         <v>0.9347111111111109</v>
       </c>
+      <c r="AJ298" t="n">
+        <v>0.82958</v>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="n">
@@ -24297,6 +25036,9 @@
       <c r="AI299" t="n">
         <v>0.5577285714285715</v>
       </c>
+      <c r="AJ299" t="n">
+        <v>0.84924</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="n">
@@ -24349,6 +25091,9 @@
       <c r="AI300" t="n">
         <v>0.4594153846153847</v>
       </c>
+      <c r="AJ300" t="n">
+        <v>0.8211999999999999</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="n">
@@ -24401,6 +25146,9 @@
       <c r="AI301" t="n">
         <v>0.6131272727272727</v>
       </c>
+      <c r="AJ301" t="n">
+        <v>0.8440428571428571</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="n">
@@ -24452,6 +25200,9 @@
       </c>
       <c r="AI302" t="n">
         <v>0.49454</v>
+      </c>
+      <c r="AJ302" t="n">
+        <v>0.8570399999999999</v>
       </c>
     </row>
     <row r="303">
@@ -25028,7 +25779,7 @@
         <v>0.9558</v>
       </c>
       <c r="AJ316" t="n">
-        <v>0</v>
+        <v>0.0035</v>
       </c>
     </row>
     <row r="317">
@@ -25092,7 +25843,7 @@
         <v>0</v>
       </c>
       <c r="AJ317" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
     </row>
     <row r="318">
@@ -25156,7 +25907,7 @@
         <v>0</v>
       </c>
       <c r="AJ318" t="n">
-        <v>0</v>
+        <v>0.0008</v>
       </c>
     </row>
     <row r="319">
@@ -25220,7 +25971,7 @@
         <v>0.0044</v>
       </c>
       <c r="AJ319" t="n">
-        <v>0.2326</v>
+        <v>0.0188</v>
       </c>
     </row>
     <row r="320">
@@ -25284,7 +26035,7 @@
         <v>0.1013</v>
       </c>
       <c r="AJ320" t="n">
-        <v>0</v>
+        <v>0.1279</v>
       </c>
     </row>
     <row r="321">
@@ -25345,7 +26096,7 @@
         <v>1</v>
       </c>
       <c r="AJ321" t="n">
-        <v>0.743</v>
+        <v>0.1657</v>
       </c>
     </row>
     <row r="322">
@@ -25406,7 +26157,7 @@
         <v>0.9284</v>
       </c>
       <c r="AJ322" t="n">
-        <v>0.743</v>
+        <v>0.0402</v>
       </c>
     </row>
     <row r="323">
@@ -25467,7 +26218,7 @@
         <v>0.9044</v>
       </c>
       <c r="AJ323" t="n">
-        <v>0.743</v>
+        <v>0.1131</v>
       </c>
     </row>
     <row r="324">
@@ -25527,6 +26278,9 @@
       <c r="AI324" t="n">
         <v>0.7281</v>
       </c>
+      <c r="AJ324" t="n">
+        <v>0.0191</v>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="n">
@@ -25585,6 +26339,9 @@
       <c r="AI325" t="n">
         <v>0.9208</v>
       </c>
+      <c r="AJ325" t="n">
+        <v>0.105</v>
+      </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="n">
@@ -25637,6 +26394,9 @@
       <c r="AI326" t="n">
         <v>0.9681999999999999</v>
       </c>
+      <c r="AJ326" t="n">
+        <v>0.0219</v>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="n">
@@ -25689,6 +26449,9 @@
       <c r="AI327" t="n">
         <v>0.7435</v>
       </c>
+      <c r="AJ327" t="n">
+        <v>0.1532</v>
+      </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="n">
@@ -25741,6 +26504,9 @@
       <c r="AI328" t="n">
         <v>0.5639999999999999</v>
       </c>
+      <c r="AJ328" t="n">
+        <v>0.1418</v>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="n">
@@ -25793,6 +26559,9 @@
       <c r="AI329" t="n">
         <v>0.2936</v>
       </c>
+      <c r="AJ329" t="n">
+        <v>0.1263</v>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="n">
@@ -25845,6 +26614,9 @@
       <c r="AI330" t="n">
         <v>0.846</v>
       </c>
+      <c r="AJ330" t="n">
+        <v>0.0457</v>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="n">
@@ -25897,6 +26669,9 @@
       <c r="AI331" t="n">
         <v>1</v>
       </c>
+      <c r="AJ331" t="n">
+        <v>0.0926</v>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="n">
@@ -25949,6 +26724,9 @@
       <c r="AI332" t="n">
         <v>0.9996</v>
       </c>
+      <c r="AJ332" t="n">
+        <v>0.1191</v>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="n">
@@ -26001,6 +26779,9 @@
       <c r="AI333" t="n">
         <v>0.9869</v>
       </c>
+      <c r="AJ333" t="n">
+        <v>0.0677</v>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="n">
@@ -26053,6 +26834,9 @@
       <c r="AI334" t="n">
         <v>0.9952</v>
       </c>
+      <c r="AJ334" t="n">
+        <v>0.0469</v>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="n">
@@ -26105,6 +26889,9 @@
       <c r="AI335" t="n">
         <v>0.9198</v>
       </c>
+      <c r="AJ335" t="n">
+        <v>0.1161</v>
+      </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="n">
@@ -26157,6 +26944,9 @@
       <c r="AI336" t="n">
         <v>0.9959</v>
       </c>
+      <c r="AJ336" t="n">
+        <v>0.1399</v>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="n">
@@ -26209,6 +26999,9 @@
       <c r="AI337" t="n">
         <v>0.8288</v>
       </c>
+      <c r="AJ337" t="n">
+        <v>0.0672</v>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="1" t="n">
@@ -26261,6 +27054,9 @@
       <c r="AI338" t="n">
         <v>0.9957</v>
       </c>
+      <c r="AJ338" t="n">
+        <v>0.1072</v>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="1" t="n">
@@ -26313,6 +27109,9 @@
       <c r="AI339" t="n">
         <v>1</v>
       </c>
+      <c r="AJ339" t="n">
+        <v>0.0721</v>
+      </c>
     </row>
     <row r="340">
       <c r="A340" s="1" t="n">
@@ -26365,6 +27164,9 @@
       <c r="AI340" t="n">
         <v>0.9986</v>
       </c>
+      <c r="AJ340" t="n">
+        <v>0.0459</v>
+      </c>
     </row>
     <row r="341">
       <c r="A341" s="1" t="n">
@@ -26417,6 +27219,9 @@
       <c r="AI341" t="n">
         <v>0.9978</v>
       </c>
+      <c r="AJ341" t="n">
+        <v>0.1061</v>
+      </c>
     </row>
     <row r="342">
       <c r="A342" s="1" t="n">
@@ -26469,6 +27274,9 @@
       <c r="AI342" t="n">
         <v>0.9865</v>
       </c>
+      <c r="AJ342" t="n">
+        <v>0.1175</v>
+      </c>
     </row>
     <row r="343">
       <c r="A343" s="1" t="n">
@@ -26521,6 +27329,9 @@
       <c r="AI343" t="n">
         <v>0.9486</v>
       </c>
+      <c r="AJ343" t="n">
+        <v>0.1197</v>
+      </c>
     </row>
     <row r="344">
       <c r="A344" s="1" t="n">
@@ -26573,6 +27384,9 @@
       <c r="AI344" t="n">
         <v>0.9975000000000001</v>
       </c>
+      <c r="AJ344" t="n">
+        <v>0.0978</v>
+      </c>
     </row>
     <row r="345">
       <c r="A345" s="1" t="n">
@@ -26625,6 +27439,9 @@
       <c r="AI345" t="n">
         <v>0.9137999999999999</v>
       </c>
+      <c r="AJ345" t="n">
+        <v>0.09470000000000001</v>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="1" t="n">
@@ -26677,6 +27494,9 @@
       <c r="AI346" t="n">
         <v>0</v>
       </c>
+      <c r="AJ346" t="n">
+        <v>0.1342</v>
+      </c>
     </row>
     <row r="347">
       <c r="A347" s="1" t="n">
@@ -26729,6 +27549,9 @@
       <c r="AI347" t="n">
         <v>0.9943</v>
       </c>
+      <c r="AJ347" t="n">
+        <v>0.1124</v>
+      </c>
     </row>
     <row r="348">
       <c r="A348" s="1" t="n">
@@ -26781,6 +27604,9 @@
       <c r="AI348" t="n">
         <v>0</v>
       </c>
+      <c r="AJ348" t="n">
+        <v>0.1427</v>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="1" t="n">
@@ -26833,6 +27659,9 @@
       <c r="AI349" t="n">
         <v>0.0578</v>
       </c>
+      <c r="AJ349" t="n">
+        <v>0.1128</v>
+      </c>
     </row>
     <row r="350">
       <c r="A350" s="1" t="n">
@@ -26885,6 +27714,9 @@
       <c r="AI350" t="n">
         <v>0.9639</v>
       </c>
+      <c r="AJ350" t="n">
+        <v>0.1134</v>
+      </c>
     </row>
     <row r="351">
       <c r="A351" s="1" t="n">
@@ -26937,6 +27769,9 @@
       <c r="AI351" t="n">
         <v>1</v>
       </c>
+      <c r="AJ351" t="n">
+        <v>0.1091</v>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="1" t="n">
@@ -26989,6 +27824,9 @@
       <c r="AI352" t="n">
         <v>0.9802999999999999</v>
       </c>
+      <c r="AJ352" t="n">
+        <v>0.0788</v>
+      </c>
     </row>
     <row r="353">
       <c r="A353" s="1" t="n">
@@ -27041,6 +27879,9 @@
       <c r="AI353" t="n">
         <v>1</v>
       </c>
+      <c r="AJ353" t="n">
+        <v>0.09859999999999999</v>
+      </c>
     </row>
     <row r="354">
       <c r="A354" s="1" t="n">
@@ -27093,6 +27934,9 @@
       <c r="AI354" t="n">
         <v>0.9728</v>
       </c>
+      <c r="AJ354" t="n">
+        <v>0.1055</v>
+      </c>
     </row>
     <row r="355">
       <c r="A355" s="1" t="n">
@@ -27145,6 +27989,9 @@
       <c r="AI355" t="n">
         <v>0</v>
       </c>
+      <c r="AJ355" t="n">
+        <v>0.1042</v>
+      </c>
     </row>
     <row r="356">
       <c r="A356" s="1" t="n">
@@ -27197,6 +28044,9 @@
       <c r="AI356" t="n">
         <v>0.1606</v>
       </c>
+      <c r="AJ356" t="n">
+        <v>0.0961</v>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="1" t="n">
@@ -27249,6 +28099,9 @@
       <c r="AI357" t="n">
         <v>0</v>
       </c>
+      <c r="AJ357" t="n">
+        <v>0.1008</v>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="1" t="n">
@@ -27301,6 +28154,9 @@
       <c r="AI358" t="n">
         <v>0</v>
       </c>
+      <c r="AJ358" t="n">
+        <v>0.1019</v>
+      </c>
     </row>
     <row r="359">
       <c r="A359" s="1" t="n">
@@ -27353,6 +28209,9 @@
       <c r="AI359" t="n">
         <v>0.8582</v>
       </c>
+      <c r="AJ359" t="n">
+        <v>0.1123</v>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="1" t="n">
@@ -27405,6 +28264,9 @@
       <c r="AI360" t="n">
         <v>0.9298</v>
       </c>
+      <c r="AJ360" t="n">
+        <v>0.1037</v>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="1" t="n">
@@ -27457,6 +28319,9 @@
       <c r="AI361" t="n">
         <v>0</v>
       </c>
+      <c r="AJ361" t="n">
+        <v>0.07779999999999999</v>
+      </c>
     </row>
     <row r="362">
       <c r="A362" s="1" t="n">
@@ -27509,6 +28374,9 @@
       <c r="AI362" t="n">
         <v>0</v>
       </c>
+      <c r="AJ362" t="n">
+        <v>0.1028</v>
+      </c>
     </row>
     <row r="363">
       <c r="A363" s="1" t="n">
@@ -27561,6 +28429,9 @@
       <c r="AI363" t="n">
         <v>0</v>
       </c>
+      <c r="AJ363" t="n">
+        <v>0.0945</v>
+      </c>
     </row>
     <row r="364">
       <c r="A364" s="1" t="n">
@@ -27613,6 +28484,9 @@
       <c r="AI364" t="n">
         <v>0</v>
       </c>
+      <c r="AJ364" t="n">
+        <v>0.1214</v>
+      </c>
     </row>
     <row r="365">
       <c r="A365" s="1" t="n">
@@ -27665,6 +28539,9 @@
       <c r="AI365" t="n">
         <v>0</v>
       </c>
+      <c r="AJ365" t="n">
+        <v>0.097</v>
+      </c>
     </row>
     <row r="366">
       <c r="A366" s="1" t="n">
@@ -27717,6 +28594,9 @@
       <c r="AI366" t="n">
         <v>1</v>
       </c>
+      <c r="AJ366" t="n">
+        <v>0.0832</v>
+      </c>
     </row>
     <row r="367">
       <c r="A367" s="1" t="n">
@@ -27769,6 +28649,9 @@
       <c r="AI367" t="n">
         <v>0</v>
       </c>
+      <c r="AJ367" t="n">
+        <v>0.1052</v>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="1" t="n">
@@ -27821,6 +28704,9 @@
       <c r="AI368" t="n">
         <v>0</v>
       </c>
+      <c r="AJ368" t="n">
+        <v>0.1062</v>
+      </c>
     </row>
     <row r="369">
       <c r="A369" s="1" t="n">
@@ -27873,6 +28759,9 @@
       <c r="AI369" t="n">
         <v>0.4487</v>
       </c>
+      <c r="AJ369" t="n">
+        <v>0.1004</v>
+      </c>
     </row>
     <row r="370">
       <c r="A370" s="1" t="n">
@@ -27925,6 +28814,9 @@
       <c r="AI370" t="n">
         <v>1</v>
       </c>
+      <c r="AJ370" t="n">
+        <v>0.0853</v>
+      </c>
     </row>
     <row r="371">
       <c r="A371" s="1" t="n">
@@ -27977,6 +28869,9 @@
       <c r="AI371" t="n">
         <v>0.9911</v>
       </c>
+      <c r="AJ371" t="n">
+        <v>0.09279999999999999</v>
+      </c>
     </row>
     <row r="372">
       <c r="A372" s="1" t="n">
@@ -28029,6 +28924,9 @@
       <c r="AI372" t="n">
         <v>0.9928</v>
       </c>
+      <c r="AJ372" t="n">
+        <v>0.1066</v>
+      </c>
     </row>
     <row r="373">
       <c r="A373" s="1" t="n">
@@ -28081,6 +28979,9 @@
       <c r="AI373" t="n">
         <v>1</v>
       </c>
+      <c r="AJ373" t="n">
+        <v>0.09959999999999999</v>
+      </c>
     </row>
     <row r="374">
       <c r="A374" s="1" t="n">
@@ -28133,6 +29034,9 @@
       <c r="AI374" t="n">
         <v>0.9956</v>
       </c>
+      <c r="AJ374" t="n">
+        <v>0.0888</v>
+      </c>
     </row>
     <row r="375">
       <c r="A375" s="1" t="n">
@@ -28185,6 +29089,9 @@
       <c r="AI375" t="n">
         <v>1</v>
       </c>
+      <c r="AJ375" t="n">
+        <v>0.0461</v>
+      </c>
     </row>
     <row r="376">
       <c r="A376" s="1" t="n">
@@ -28237,6 +29144,9 @@
       <c r="AI376" t="n">
         <v>0</v>
       </c>
+      <c r="AJ376" t="n">
+        <v>0.0492</v>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="1" t="n">
@@ -28289,6 +29199,9 @@
       <c r="AI377" t="n">
         <v>0</v>
       </c>
+      <c r="AJ377" t="n">
+        <v>0.0615</v>
+      </c>
     </row>
     <row r="378">
       <c r="A378" s="1" t="n">
@@ -28341,6 +29254,9 @@
       <c r="AI378" t="n">
         <v>0</v>
       </c>
+      <c r="AJ378" t="n">
+        <v>0.1055</v>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="1" t="n">
@@ -28393,6 +29309,9 @@
       <c r="AI379" t="n">
         <v>0</v>
       </c>
+      <c r="AJ379" t="n">
+        <v>0.0897</v>
+      </c>
     </row>
     <row r="380">
       <c r="A380" s="1" t="n">
@@ -28445,6 +29364,9 @@
       <c r="AI380" t="n">
         <v>0.4348</v>
       </c>
+      <c r="AJ380" t="n">
+        <v>0.0881</v>
+      </c>
     </row>
     <row r="381">
       <c r="A381" s="1" t="n">
@@ -28497,6 +29419,9 @@
       <c r="AI381" t="n">
         <v>0.9605</v>
       </c>
+      <c r="AJ381" t="n">
+        <v>0.1029</v>
+      </c>
     </row>
     <row r="382">
       <c r="A382" s="1" t="n">
@@ -28549,6 +29474,9 @@
       <c r="AI382" t="n">
         <v>0</v>
       </c>
+      <c r="AJ382" t="n">
+        <v>0.1014</v>
+      </c>
     </row>
     <row r="383">
       <c r="A383" s="1" t="n">
@@ -28601,6 +29529,9 @@
       <c r="AI383" t="n">
         <v>0</v>
       </c>
+      <c r="AJ383" t="n">
+        <v>0.1244</v>
+      </c>
     </row>
     <row r="384">
       <c r="A384" s="1" t="n">
@@ -28653,6 +29584,9 @@
       <c r="AI384" t="n">
         <v>0</v>
       </c>
+      <c r="AJ384" t="n">
+        <v>0.1071</v>
+      </c>
     </row>
     <row r="385">
       <c r="A385" s="1" t="n">
@@ -28705,6 +29639,9 @@
       <c r="AI385" t="n">
         <v>0</v>
       </c>
+      <c r="AJ385" t="n">
+        <v>0.1123</v>
+      </c>
     </row>
     <row r="386">
       <c r="A386" s="1" t="n">
@@ -28757,6 +29694,9 @@
       <c r="AI386" t="n">
         <v>0</v>
       </c>
+      <c r="AJ386" t="n">
+        <v>0.09039999999999999</v>
+      </c>
     </row>
     <row r="387">
       <c r="A387" s="1" t="n">
@@ -28809,6 +29749,9 @@
       <c r="AI387" t="n">
         <v>0</v>
       </c>
+      <c r="AJ387" t="n">
+        <v>0.07920000000000001</v>
+      </c>
     </row>
     <row r="388">
       <c r="A388" s="1" t="n">
@@ -28861,6 +29804,9 @@
       <c r="AI388" t="n">
         <v>0.9457</v>
       </c>
+      <c r="AJ388" t="n">
+        <v>0.0955</v>
+      </c>
     </row>
     <row r="389">
       <c r="A389" s="1" t="n">
@@ -28913,6 +29859,9 @@
       <c r="AI389" t="n">
         <v>0</v>
       </c>
+      <c r="AJ389" t="n">
+        <v>0.1156</v>
+      </c>
     </row>
     <row r="390">
       <c r="A390" s="1" t="n">
@@ -28965,6 +29914,9 @@
       <c r="AI390" t="n">
         <v>0</v>
       </c>
+      <c r="AJ390" t="n">
+        <v>0.1201</v>
+      </c>
     </row>
     <row r="391">
       <c r="A391" s="1" t="n">
@@ -29017,6 +29969,9 @@
       <c r="AI391" t="n">
         <v>0</v>
       </c>
+      <c r="AJ391" t="n">
+        <v>0.0934</v>
+      </c>
     </row>
     <row r="392">
       <c r="A392" s="1" t="n">
@@ -29069,6 +30024,9 @@
       <c r="AI392" t="n">
         <v>0</v>
       </c>
+      <c r="AJ392" t="n">
+        <v>0.0827</v>
+      </c>
     </row>
     <row r="393">
       <c r="A393" s="1" t="n">
@@ -29121,6 +30079,9 @@
       <c r="AI393" t="n">
         <v>0.8885999999999999</v>
       </c>
+      <c r="AJ393" t="n">
+        <v>0.0983</v>
+      </c>
     </row>
     <row r="394">
       <c r="A394" s="1" t="n">
@@ -29173,6 +30134,9 @@
       <c r="AI394" t="n">
         <v>0</v>
       </c>
+      <c r="AJ394" t="n">
+        <v>0.0919</v>
+      </c>
     </row>
     <row r="395">
       <c r="A395" s="1" t="n">
@@ -29225,6 +30189,9 @@
       <c r="AI395" t="n">
         <v>0.004</v>
       </c>
+      <c r="AJ395" t="n">
+        <v>0.1099</v>
+      </c>
     </row>
     <row r="396">
       <c r="A396" s="1" t="n">
@@ -29277,6 +30244,9 @@
       <c r="AI396" t="n">
         <v>0</v>
       </c>
+      <c r="AJ396" t="n">
+        <v>0.0964</v>
+      </c>
     </row>
     <row r="397">
       <c r="A397" s="1" t="n">
@@ -29329,6 +30299,9 @@
       <c r="AI397" t="n">
         <v>0</v>
       </c>
+      <c r="AJ397" t="n">
+        <v>0.0917</v>
+      </c>
     </row>
     <row r="398">
       <c r="A398" s="1" t="n">
@@ -29381,6 +30354,9 @@
       <c r="AI398" t="n">
         <v>0</v>
       </c>
+      <c r="AJ398" t="n">
+        <v>0.0901</v>
+      </c>
     </row>
     <row r="399">
       <c r="A399" s="1" t="n">
@@ -29433,6 +30409,9 @@
       <c r="AI399" t="n">
         <v>0</v>
       </c>
+      <c r="AJ399" t="n">
+        <v>0.0955</v>
+      </c>
     </row>
     <row r="400">
       <c r="A400" s="1" t="n">
@@ -29485,6 +30464,9 @@
       <c r="AI400" t="n">
         <v>0.6539</v>
       </c>
+      <c r="AJ400" t="n">
+        <v>0.097</v>
+      </c>
     </row>
     <row r="401">
       <c r="A401" s="1" t="n">
@@ -29537,6 +30519,9 @@
       <c r="AI401" t="n">
         <v>0</v>
       </c>
+      <c r="AJ401" t="n">
+        <v>0.1237</v>
+      </c>
     </row>
     <row r="402">
       <c r="A402" s="1" t="n">
@@ -29589,6 +30574,9 @@
       <c r="AI402" t="n">
         <v>0</v>
       </c>
+      <c r="AJ402" t="n">
+        <v>0.1138</v>
+      </c>
     </row>
     <row r="403">
       <c r="A403" s="1" t="n">
@@ -29641,6 +30629,9 @@
       <c r="AI403" t="n">
         <v>0</v>
       </c>
+      <c r="AJ403" t="n">
+        <v>0.1078</v>
+      </c>
     </row>
     <row r="404">
       <c r="A404" s="1" t="n">
@@ -29693,6 +30684,9 @@
       <c r="AI404" t="n">
         <v>0</v>
       </c>
+      <c r="AJ404" t="n">
+        <v>0.0984</v>
+      </c>
     </row>
     <row r="405">
       <c r="A405" s="1" t="n">
@@ -29745,6 +30739,9 @@
       <c r="AI405" t="n">
         <v>0.0023</v>
       </c>
+      <c r="AJ405" t="n">
+        <v>0.1093</v>
+      </c>
     </row>
     <row r="406">
       <c r="A406" s="1" t="n">
@@ -29796,6 +30793,9 @@
       </c>
       <c r="AI406" t="n">
         <v>1</v>
+      </c>
+      <c r="AJ406" t="n">
+        <v>0.1216</v>
       </c>
     </row>
     <row r="407">

</xml_diff>

<commit_message>
Ran my algorithm Dirichlet 100%clustering
</commit_message>
<xml_diff>
--- a/CIFAR_Global.xlsx
+++ b/CIFAR_Global.xlsx
@@ -8314,7 +8314,7 @@
         <v>0.0999</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0.1451</v>
+        <v>0.1178</v>
       </c>
     </row>
     <row r="6">
@@ -8385,7 +8385,7 @@
         <v>0.0999</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0.1776</v>
+        <v>0.1359</v>
       </c>
     </row>
     <row r="7">
@@ -8456,7 +8456,7 @@
         <v>0.1529</v>
       </c>
       <c r="AJ7" t="n">
-        <v>0.2412</v>
+        <v>0.2568</v>
       </c>
     </row>
     <row r="8">
@@ -8527,7 +8527,7 @@
         <v>0.1115</v>
       </c>
       <c r="AJ8" t="n">
-        <v>0.2753</v>
+        <v>0.2805</v>
       </c>
     </row>
     <row r="9">
@@ -8598,7 +8598,7 @@
         <v>0.1121</v>
       </c>
       <c r="AJ9" t="n">
-        <v>0.3397</v>
+        <v>0.2879</v>
       </c>
     </row>
     <row r="10">
@@ -8666,7 +8666,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0.3398</v>
+        <v>0.3319</v>
       </c>
     </row>
     <row r="11">
@@ -8734,7 +8734,7 @@
         <v>0.1122</v>
       </c>
       <c r="AJ11" t="n">
-        <v>0.371</v>
+        <v>0.3523</v>
       </c>
     </row>
     <row r="12">
@@ -8802,7 +8802,7 @@
         <v>0.1314</v>
       </c>
       <c r="AJ12" t="n">
-        <v>0.3819</v>
+        <v>0.3623</v>
       </c>
     </row>
     <row r="13">
@@ -8870,7 +8870,7 @@
         <v>0.1433</v>
       </c>
       <c r="AJ13" t="n">
-        <v>0.3639</v>
+        <v>0.3563</v>
       </c>
     </row>
     <row r="14">
@@ -8938,7 +8938,7 @@
         <v>0.1074</v>
       </c>
       <c r="AJ14" t="n">
-        <v>0.3883</v>
+        <v>0.3897</v>
       </c>
     </row>
     <row r="15">
@@ -9000,7 +9000,7 @@
         <v>0.107</v>
       </c>
       <c r="AJ15" t="n">
-        <v>0.3739</v>
+        <v>0.4156</v>
       </c>
     </row>
     <row r="16">
@@ -9062,7 +9062,7 @@
         <v>0.1092</v>
       </c>
       <c r="AJ16" t="n">
-        <v>0.4131</v>
+        <v>0.4116</v>
       </c>
     </row>
     <row r="17">
@@ -9124,7 +9124,7 @@
         <v>0.094</v>
       </c>
       <c r="AJ17" t="n">
-        <v>0.4237</v>
+        <v>0.4178</v>
       </c>
     </row>
     <row r="18">
@@ -9186,7 +9186,7 @@
         <v>0.0944</v>
       </c>
       <c r="AJ18" t="n">
-        <v>0.4181</v>
+        <v>0.3976</v>
       </c>
     </row>
     <row r="19">
@@ -9248,7 +9248,7 @@
         <v>0.0955</v>
       </c>
       <c r="AJ19" t="n">
-        <v>0.4194</v>
+        <v>0.4065</v>
       </c>
     </row>
     <row r="20">
@@ -9310,7 +9310,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ20" t="n">
-        <v>0.4259</v>
+        <v>0.4254</v>
       </c>
     </row>
     <row r="21">
@@ -9372,7 +9372,7 @@
         <v>0.1228</v>
       </c>
       <c r="AJ21" t="n">
-        <v>0.4252</v>
+        <v>0.4087</v>
       </c>
     </row>
     <row r="22">
@@ -9434,7 +9434,7 @@
         <v>0.1179</v>
       </c>
       <c r="AJ22" t="n">
-        <v>0.4283</v>
+        <v>0.4222</v>
       </c>
     </row>
     <row r="23">
@@ -9496,7 +9496,7 @@
         <v>0.1213</v>
       </c>
       <c r="AJ23" t="n">
-        <v>0.4113</v>
+        <v>0.4327</v>
       </c>
     </row>
     <row r="24">
@@ -9558,7 +9558,7 @@
         <v>0.09760000000000001</v>
       </c>
       <c r="AJ24" t="n">
-        <v>0.4335</v>
+        <v>0.4324</v>
       </c>
     </row>
     <row r="25">
@@ -9620,7 +9620,7 @@
         <v>0.1238</v>
       </c>
       <c r="AJ25" t="n">
-        <v>0.4277</v>
+        <v>0.4212</v>
       </c>
     </row>
     <row r="26">
@@ -9682,7 +9682,7 @@
         <v>0.1253</v>
       </c>
       <c r="AJ26" t="n">
-        <v>0.4239</v>
+        <v>0.4345</v>
       </c>
     </row>
     <row r="27">
@@ -9744,7 +9744,7 @@
         <v>0.1174</v>
       </c>
       <c r="AJ27" t="n">
-        <v>0.4287</v>
+        <v>0.43</v>
       </c>
     </row>
     <row r="28">
@@ -9806,7 +9806,7 @@
         <v>0.1014</v>
       </c>
       <c r="AJ28" t="n">
-        <v>0.4235</v>
+        <v>0.4338</v>
       </c>
     </row>
     <row r="29">
@@ -9868,7 +9868,7 @@
         <v>0.103</v>
       </c>
       <c r="AJ29" t="n">
-        <v>0.4191</v>
+        <v>0.4344</v>
       </c>
     </row>
     <row r="30">
@@ -9930,7 +9930,7 @@
         <v>0.1132</v>
       </c>
       <c r="AJ30" t="n">
-        <v>0.4324</v>
+        <v>0.4319</v>
       </c>
     </row>
     <row r="31">
@@ -9992,7 +9992,7 @@
         <v>0.1195</v>
       </c>
       <c r="AJ31" t="n">
-        <v>0.4328</v>
+        <v>0.4309</v>
       </c>
     </row>
     <row r="32">
@@ -10054,7 +10054,7 @@
         <v>0.1026</v>
       </c>
       <c r="AJ32" t="n">
-        <v>0.4318</v>
+        <v>0.4393</v>
       </c>
     </row>
     <row r="33">
@@ -10116,7 +10116,7 @@
         <v>0.1197</v>
       </c>
       <c r="AJ33" t="n">
-        <v>0.4186</v>
+        <v>0.4252</v>
       </c>
     </row>
     <row r="34">
@@ -10178,7 +10178,7 @@
         <v>0.097</v>
       </c>
       <c r="AJ34" t="n">
-        <v>0.4335</v>
+        <v>0.4359</v>
       </c>
     </row>
     <row r="35">
@@ -10240,7 +10240,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ35" t="n">
-        <v>0.437</v>
+        <v>0.4432</v>
       </c>
     </row>
     <row r="36">
@@ -10302,7 +10302,7 @@
         <v>0.1132</v>
       </c>
       <c r="AJ36" t="n">
-        <v>0.4241</v>
+        <v>0.4367</v>
       </c>
     </row>
     <row r="37">
@@ -10364,7 +10364,7 @@
         <v>0.1135</v>
       </c>
       <c r="AJ37" t="n">
-        <v>0.4346</v>
+        <v>0.4375</v>
       </c>
     </row>
     <row r="38">
@@ -10426,7 +10426,7 @@
         <v>0.1462</v>
       </c>
       <c r="AJ38" t="n">
-        <v>0.4284</v>
+        <v>0.4375</v>
       </c>
     </row>
     <row r="39">
@@ -10488,7 +10488,7 @@
         <v>0.1282</v>
       </c>
       <c r="AJ39" t="n">
-        <v>0.4229</v>
+        <v>0.4254</v>
       </c>
     </row>
     <row r="40">
@@ -10550,7 +10550,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ40" t="n">
-        <v>0.4185</v>
+        <v>0.4379</v>
       </c>
     </row>
     <row r="41">
@@ -10612,7 +10612,7 @@
         <v>0.121</v>
       </c>
       <c r="AJ41" t="n">
-        <v>0.4242</v>
+        <v>0.4403</v>
       </c>
     </row>
     <row r="42">
@@ -10674,7 +10674,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ42" t="n">
-        <v>0.4321</v>
+        <v>0.4301</v>
       </c>
     </row>
     <row r="43">
@@ -10736,7 +10736,7 @@
         <v>0.1129</v>
       </c>
       <c r="AJ43" t="n">
-        <v>0.4232</v>
+        <v>0.4226</v>
       </c>
     </row>
     <row r="44">
@@ -10798,7 +10798,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ44" t="n">
-        <v>0.4193</v>
+        <v>0.4324</v>
       </c>
     </row>
     <row r="45">
@@ -10860,7 +10860,7 @@
         <v>0.1446</v>
       </c>
       <c r="AJ45" t="n">
-        <v>0.4272</v>
+        <v>0.4436</v>
       </c>
     </row>
     <row r="46">
@@ -10922,7 +10922,7 @@
         <v>0.1577</v>
       </c>
       <c r="AJ46" t="n">
-        <v>0.4304</v>
+        <v>0.4406</v>
       </c>
     </row>
     <row r="47">
@@ -10984,7 +10984,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ47" t="n">
-        <v>0.431</v>
+        <v>0.4378</v>
       </c>
     </row>
     <row r="48">
@@ -11046,7 +11046,7 @@
         <v>0.1606</v>
       </c>
       <c r="AJ48" t="n">
-        <v>0.4311</v>
+        <v>0.4387</v>
       </c>
     </row>
     <row r="49">
@@ -11108,7 +11108,7 @@
         <v>0.1216</v>
       </c>
       <c r="AJ49" t="n">
-        <v>0.4364</v>
+        <v>0.4355</v>
       </c>
     </row>
     <row r="50">
@@ -11170,7 +11170,7 @@
         <v>0.1731</v>
       </c>
       <c r="AJ50" t="n">
-        <v>0.4297</v>
+        <v>0.4341</v>
       </c>
     </row>
     <row r="51">
@@ -11232,7 +11232,7 @@
         <v>0.1475</v>
       </c>
       <c r="AJ51" t="n">
-        <v>0.4325</v>
+        <v>0.4388</v>
       </c>
     </row>
     <row r="52">
@@ -11294,7 +11294,7 @@
         <v>0.2121</v>
       </c>
       <c r="AJ52" t="n">
-        <v>0.439</v>
+        <v>0.4387</v>
       </c>
     </row>
     <row r="53">
@@ -11356,7 +11356,7 @@
         <v>0.1404</v>
       </c>
       <c r="AJ53" t="n">
-        <v>0.4266</v>
+        <v>0.4432</v>
       </c>
     </row>
     <row r="54">
@@ -11418,7 +11418,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ54" t="n">
-        <v>0.4419</v>
+        <v>0.4442</v>
       </c>
     </row>
     <row r="55">
@@ -11480,7 +11480,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ55" t="n">
-        <v>0.4387</v>
+        <v>0.4409</v>
       </c>
     </row>
     <row r="56">
@@ -11542,7 +11542,7 @@
         <v>0.1787</v>
       </c>
       <c r="AJ56" t="n">
-        <v>0.4397</v>
+        <v>0.4364</v>
       </c>
     </row>
     <row r="57">
@@ -11604,7 +11604,7 @@
         <v>0.1458</v>
       </c>
       <c r="AJ57" t="n">
-        <v>0.4382</v>
+        <v>0.4346</v>
       </c>
     </row>
     <row r="58">
@@ -11666,7 +11666,7 @@
         <v>0.1687</v>
       </c>
       <c r="AJ58" t="n">
-        <v>0.4371</v>
+        <v>0.4414</v>
       </c>
     </row>
     <row r="59">
@@ -11728,7 +11728,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ59" t="n">
-        <v>0.4341</v>
+        <v>0.4398</v>
       </c>
     </row>
     <row r="60">
@@ -11790,7 +11790,7 @@
         <v>0.1279</v>
       </c>
       <c r="AJ60" t="n">
-        <v>0.4353</v>
+        <v>0.4417</v>
       </c>
     </row>
     <row r="61">
@@ -11852,7 +11852,7 @@
         <v>0.1275</v>
       </c>
       <c r="AJ61" t="n">
-        <v>0.4351</v>
+        <v>0.4441</v>
       </c>
     </row>
     <row r="62">
@@ -11914,7 +11914,7 @@
         <v>0.1001</v>
       </c>
       <c r="AJ62" t="n">
-        <v>0.4377</v>
+        <v>0.4471</v>
       </c>
     </row>
     <row r="63">
@@ -11976,7 +11976,7 @@
         <v>0.1215</v>
       </c>
       <c r="AJ63" t="n">
-        <v>0.432</v>
+        <v>0.4402</v>
       </c>
     </row>
     <row r="64">
@@ -12038,7 +12038,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ64" t="n">
-        <v>0.4269</v>
+        <v>0.4411</v>
       </c>
     </row>
     <row r="65">
@@ -12100,7 +12100,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ65" t="n">
-        <v>0.4252</v>
+        <v>0.4438</v>
       </c>
     </row>
     <row r="66">
@@ -12162,7 +12162,7 @@
         <v>0.1438</v>
       </c>
       <c r="AJ66" t="n">
-        <v>0.433</v>
+        <v>0.4507</v>
       </c>
     </row>
     <row r="67">
@@ -12224,7 +12224,7 @@
         <v>0.1539</v>
       </c>
       <c r="AJ67" t="n">
-        <v>0.4323</v>
+        <v>0.4478</v>
       </c>
     </row>
     <row r="68">
@@ -12286,7 +12286,7 @@
         <v>0.1323</v>
       </c>
       <c r="AJ68" t="n">
-        <v>0.4351</v>
+        <v>0.4435</v>
       </c>
     </row>
     <row r="69">
@@ -12348,7 +12348,7 @@
         <v>0.1294</v>
       </c>
       <c r="AJ69" t="n">
-        <v>0.4403</v>
+        <v>0.4447</v>
       </c>
     </row>
     <row r="70">
@@ -12410,7 +12410,7 @@
         <v>0.155</v>
       </c>
       <c r="AJ70" t="n">
-        <v>0.4417</v>
+        <v>0.4431</v>
       </c>
     </row>
     <row r="71">
@@ -12472,7 +12472,7 @@
         <v>0.1347</v>
       </c>
       <c r="AJ71" t="n">
-        <v>0.4382</v>
+        <v>0.4365</v>
       </c>
     </row>
     <row r="72">
@@ -12534,7 +12534,7 @@
         <v>0.1642</v>
       </c>
       <c r="AJ72" t="n">
-        <v>0.4358</v>
+        <v>0.4402</v>
       </c>
     </row>
     <row r="73">
@@ -12596,7 +12596,7 @@
         <v>0.1646</v>
       </c>
       <c r="AJ73" t="n">
-        <v>0.437</v>
+        <v>0.4417</v>
       </c>
     </row>
     <row r="74">
@@ -12658,7 +12658,7 @@
         <v>0.1509</v>
       </c>
       <c r="AJ74" t="n">
-        <v>0.44</v>
+        <v>0.4323</v>
       </c>
     </row>
     <row r="75">
@@ -12720,7 +12720,7 @@
         <v>0.1643</v>
       </c>
       <c r="AJ75" t="n">
-        <v>0.4343</v>
+        <v>0.4397</v>
       </c>
     </row>
     <row r="76">
@@ -12782,7 +12782,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ76" t="n">
-        <v>0.419</v>
+        <v>0.4451</v>
       </c>
     </row>
     <row r="77">
@@ -12844,7 +12844,7 @@
         <v>0.1346</v>
       </c>
       <c r="AJ77" t="n">
-        <v>0.4327</v>
+        <v>0.4387</v>
       </c>
     </row>
     <row r="78">
@@ -12906,7 +12906,7 @@
         <v>0.1402</v>
       </c>
       <c r="AJ78" t="n">
-        <v>0.4404</v>
+        <v>0.4463</v>
       </c>
     </row>
     <row r="79">
@@ -12968,7 +12968,7 @@
         <v>0.1613</v>
       </c>
       <c r="AJ79" t="n">
-        <v>0.443</v>
+        <v>0.444</v>
       </c>
     </row>
     <row r="80">
@@ -13030,7 +13030,7 @@
         <v>0.138</v>
       </c>
       <c r="AJ80" t="n">
-        <v>0.4426</v>
+        <v>0.4459</v>
       </c>
     </row>
     <row r="81">
@@ -13092,7 +13092,7 @@
         <v>0.1527</v>
       </c>
       <c r="AJ81" t="n">
-        <v>0.443</v>
+        <v>0.4501</v>
       </c>
     </row>
     <row r="82">
@@ -13154,7 +13154,7 @@
         <v>0.1347</v>
       </c>
       <c r="AJ82" t="n">
-        <v>0.4362</v>
+        <v>0.443</v>
       </c>
     </row>
     <row r="83">
@@ -13216,7 +13216,7 @@
         <v>0.117</v>
       </c>
       <c r="AJ83" t="n">
-        <v>0.44</v>
+        <v>0.4391</v>
       </c>
     </row>
     <row r="84">
@@ -13278,7 +13278,7 @@
         <v>0.1112</v>
       </c>
       <c r="AJ84" t="n">
-        <v>0.4432</v>
+        <v>0.4372</v>
       </c>
     </row>
     <row r="85">
@@ -13340,7 +13340,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ85" t="n">
-        <v>0.4457</v>
+        <v>0.4398</v>
       </c>
     </row>
     <row r="86">
@@ -13402,7 +13402,7 @@
         <v>0.1444</v>
       </c>
       <c r="AJ86" t="n">
-        <v>0.4423</v>
+        <v>0.4451</v>
       </c>
     </row>
     <row r="87">
@@ -13464,7 +13464,7 @@
         <v>0.1127</v>
       </c>
       <c r="AJ87" t="n">
-        <v>0.4405</v>
+        <v>0.448</v>
       </c>
     </row>
     <row r="88">
@@ -13526,7 +13526,7 @@
         <v>0.131</v>
       </c>
       <c r="AJ88" t="n">
-        <v>0.4459</v>
+        <v>0.4299</v>
       </c>
     </row>
     <row r="89">
@@ -13588,7 +13588,7 @@
         <v>0.1833</v>
       </c>
       <c r="AJ89" t="n">
-        <v>0.4325</v>
+        <v>0.4279</v>
       </c>
     </row>
     <row r="90">
@@ -13650,7 +13650,7 @@
         <v>0.2327</v>
       </c>
       <c r="AJ90" t="n">
-        <v>0.4422</v>
+        <v>0.4384</v>
       </c>
     </row>
     <row r="91">
@@ -13712,7 +13712,7 @@
         <v>0.2327</v>
       </c>
       <c r="AJ91" t="n">
-        <v>0.4332</v>
+        <v>0.4458</v>
       </c>
     </row>
     <row r="92">
@@ -13774,7 +13774,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ92" t="n">
-        <v>0.442</v>
+        <v>0.4474</v>
       </c>
     </row>
     <row r="93">
@@ -13836,7 +13836,7 @@
         <v>0.1949</v>
       </c>
       <c r="AJ93" t="n">
-        <v>0.4348</v>
+        <v>0.449</v>
       </c>
     </row>
     <row r="94">
@@ -13898,7 +13898,7 @@
         <v>0.1447</v>
       </c>
       <c r="AJ94" t="n">
-        <v>0.4344</v>
+        <v>0.4493</v>
       </c>
     </row>
     <row r="95">
@@ -13960,7 +13960,7 @@
         <v>0.1</v>
       </c>
       <c r="AJ95" t="n">
-        <v>0.435</v>
+        <v>0.4427</v>
       </c>
     </row>
     <row r="96">
@@ -14021,6 +14021,9 @@
       <c r="AI96" t="n">
         <v>0.1</v>
       </c>
+      <c r="AJ96" t="n">
+        <v>0.4413</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
@@ -14080,6 +14083,9 @@
       <c r="AI97" t="n">
         <v>0.1</v>
       </c>
+      <c r="AJ97" t="n">
+        <v>0.4379</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
@@ -14139,6 +14145,9 @@
       <c r="AI98" t="n">
         <v>0.2139</v>
       </c>
+      <c r="AJ98" t="n">
+        <v>0.4374</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
@@ -14198,6 +14207,9 @@
       <c r="AI99" t="n">
         <v>0.2222</v>
       </c>
+      <c r="AJ99" t="n">
+        <v>0.4365</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
@@ -14257,6 +14269,9 @@
       <c r="AI100" t="n">
         <v>0.1079</v>
       </c>
+      <c r="AJ100" t="n">
+        <v>0.4451</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
@@ -14316,6 +14331,9 @@
       <c r="AI101" t="n">
         <v>0.1193</v>
       </c>
+      <c r="AJ101" t="n">
+        <v>0.4381</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
@@ -14375,6 +14393,9 @@
       <c r="AI102" t="n">
         <v>0.1</v>
       </c>
+      <c r="AJ102" t="n">
+        <v>0.4397</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
@@ -14434,6 +14455,9 @@
       <c r="AI103" t="n">
         <v>0.1046</v>
       </c>
+      <c r="AJ103" t="n">
+        <v>0.4445</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
@@ -14492,6 +14516,9 @@
       </c>
       <c r="AI104" t="n">
         <v>0.1046</v>
+      </c>
+      <c r="AJ104" t="n">
+        <v>0.446</v>
       </c>
     </row>
     <row r="105">
@@ -14597,7 +14624,7 @@
         <v>0.9333333333333333</v>
       </c>
       <c r="AJ108" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5333333333333333</v>
       </c>
     </row>
     <row r="109">
@@ -14661,7 +14688,7 @@
         <v>1</v>
       </c>
       <c r="AJ109" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="110">
@@ -14725,7 +14752,7 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="AJ110" t="n">
-        <v>0.7692307692307693</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="111">
@@ -14789,7 +14816,7 @@
         <v>0.8181818181818182</v>
       </c>
       <c r="AJ111" t="n">
-        <v>0.75</v>
+        <v>0.7142857142857143</v>
       </c>
     </row>
     <row r="112">
@@ -14853,7 +14880,7 @@
         <v>0.8181818181818182</v>
       </c>
       <c r="AJ112" t="n">
-        <v>0.7857142857142857</v>
+        <v>0.3076923076923077</v>
       </c>
     </row>
     <row r="113">
@@ -14914,7 +14941,7 @@
         <v>0.7272727272727273</v>
       </c>
       <c r="AJ113" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.6923076923076923</v>
       </c>
     </row>
     <row r="114">
@@ -14975,7 +15002,7 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="AJ114" t="n">
-        <v>0.6923076923076923</v>
+        <v>0.8333333333333334</v>
       </c>
     </row>
     <row r="115">
@@ -15036,7 +15063,7 @@
         <v>0.7</v>
       </c>
       <c r="AJ115" t="n">
-        <v>0.8333333333333334</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116">
@@ -15097,7 +15124,7 @@
         <v>0.7</v>
       </c>
       <c r="AJ116" t="n">
-        <v>0.8461538461538461</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="117">
@@ -15158,7 +15185,7 @@
         <v>0.7272727272727273</v>
       </c>
       <c r="AJ117" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.8571428571428571</v>
       </c>
     </row>
     <row r="118">
@@ -15213,7 +15240,7 @@
         <v>0.7777777777777778</v>
       </c>
       <c r="AJ118" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="119">
@@ -15268,7 +15295,7 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="AJ119" t="n">
-        <v>0.8</v>
+        <v>0.6363636363636364</v>
       </c>
     </row>
     <row r="120">
@@ -15378,7 +15405,7 @@
         <v>0.9</v>
       </c>
       <c r="AJ121" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122">
@@ -15433,7 +15460,7 @@
         <v>0.9166666666666666</v>
       </c>
       <c r="AJ122" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="123">
@@ -15488,7 +15515,7 @@
         <v>0.9090909090909091</v>
       </c>
       <c r="AJ123" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.8181818181818182</v>
       </c>
     </row>
     <row r="124">
@@ -15543,7 +15570,7 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="AJ124" t="n">
-        <v>0.75</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="125">
@@ -15653,7 +15680,7 @@
         <v>1</v>
       </c>
       <c r="AJ126" t="n">
-        <v>0.75</v>
+        <v>0.9166666666666666</v>
       </c>
     </row>
     <row r="127">
@@ -15708,7 +15735,7 @@
         <v>0.6428571428571429</v>
       </c>
       <c r="AJ127" t="n">
-        <v>0.6</v>
+        <v>0.8181818181818182</v>
       </c>
     </row>
     <row r="128">
@@ -15763,7 +15790,7 @@
         <v>0.9</v>
       </c>
       <c r="AJ128" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.8888888888888888</v>
       </c>
     </row>
     <row r="129">
@@ -15818,7 +15845,7 @@
         <v>0.8</v>
       </c>
       <c r="AJ129" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="130">
@@ -15873,7 +15900,7 @@
         <v>0.8</v>
       </c>
       <c r="AJ130" t="n">
-        <v>0.5454545454545454</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="131">
@@ -15928,7 +15955,7 @@
         <v>0.875</v>
       </c>
       <c r="AJ131" t="n">
-        <v>0.75</v>
+        <v>0.8888888888888888</v>
       </c>
     </row>
     <row r="132">
@@ -15983,7 +16010,7 @@
         <v>0.9090909090909091</v>
       </c>
       <c r="AJ132" t="n">
-        <v>0.75</v>
+        <v>0.3571428571428572</v>
       </c>
     </row>
     <row r="133">
@@ -16038,7 +16065,7 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="AJ133" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="134">
@@ -16093,7 +16120,7 @@
         <v>0.8888888888888888</v>
       </c>
       <c r="AJ134" t="n">
-        <v>0.6</v>
+        <v>0.6363636363636364</v>
       </c>
     </row>
     <row r="135">
@@ -16148,7 +16175,7 @@
         <v>0.8181818181818182</v>
       </c>
       <c r="AJ135" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.5454545454545454</v>
       </c>
     </row>
     <row r="136">
@@ -16203,7 +16230,7 @@
         <v>0.9</v>
       </c>
       <c r="AJ136" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="137">
@@ -16258,7 +16285,7 @@
         <v>0.875</v>
       </c>
       <c r="AJ137" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="138">
@@ -16313,7 +16340,7 @@
         <v>1</v>
       </c>
       <c r="AJ138" t="n">
-        <v>0.7142857142857143</v>
+        <v>1</v>
       </c>
     </row>
     <row r="139">
@@ -16368,7 +16395,7 @@
         <v>0.8571428571428571</v>
       </c>
       <c r="AJ139" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="140">
@@ -16423,7 +16450,7 @@
         <v>1</v>
       </c>
       <c r="AJ140" t="n">
-        <v>0.75</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="141">
@@ -16478,7 +16505,7 @@
         <v>1</v>
       </c>
       <c r="AJ141" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="142">
@@ -16533,7 +16560,7 @@
         <v>0.8888888888888888</v>
       </c>
       <c r="AJ142" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="143">
@@ -16588,7 +16615,7 @@
         <v>1</v>
       </c>
       <c r="AJ143" t="n">
-        <v>1</v>
+        <v>0.5555555555555556</v>
       </c>
     </row>
     <row r="144">
@@ -16643,7 +16670,7 @@
         <v>1</v>
       </c>
       <c r="AJ144" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="145">
@@ -16698,7 +16725,7 @@
         <v>0.5</v>
       </c>
       <c r="AJ145" t="n">
-        <v>0.4285714285714285</v>
+        <v>1</v>
       </c>
     </row>
     <row r="146">
@@ -16753,7 +16780,7 @@
         <v>0.5</v>
       </c>
       <c r="AJ146" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="147">
@@ -16808,7 +16835,7 @@
         <v>1</v>
       </c>
       <c r="AJ147" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="148">
@@ -16863,7 +16890,7 @@
         <v>0.8</v>
       </c>
       <c r="AJ148" t="n">
-        <v>0.5</v>
+        <v>0.7777777777777778</v>
       </c>
     </row>
     <row r="149">
@@ -16918,7 +16945,7 @@
         <v>1</v>
       </c>
       <c r="AJ149" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="150">
@@ -16973,7 +17000,7 @@
         <v>1</v>
       </c>
       <c r="AJ150" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.3846153846153846</v>
       </c>
     </row>
     <row r="151">
@@ -17028,7 +17055,7 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="AJ151" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.5454545454545454</v>
       </c>
     </row>
     <row r="152">
@@ -17083,7 +17110,7 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="AJ152" t="n">
-        <v>0.6363636363636364</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="153">
@@ -17138,7 +17165,7 @@
         <v>1</v>
       </c>
       <c r="AJ153" t="n">
-        <v>0.625</v>
+        <v>0.3636363636363636</v>
       </c>
     </row>
     <row r="154">
@@ -17193,7 +17220,7 @@
         <v>1</v>
       </c>
       <c r="AJ154" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="155">
@@ -17248,7 +17275,7 @@
         <v>0.8571428571428571</v>
       </c>
       <c r="AJ155" t="n">
-        <v>1</v>
+        <v>0.2727272727272727</v>
       </c>
     </row>
     <row r="156">
@@ -17303,7 +17330,7 @@
         <v>1</v>
       </c>
       <c r="AJ156" t="n">
-        <v>0.5714285714285714</v>
+        <v>1</v>
       </c>
     </row>
     <row r="157">
@@ -17358,7 +17385,7 @@
         <v>0.8571428571428571</v>
       </c>
       <c r="AJ157" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="158">
@@ -17413,7 +17440,7 @@
         <v>0.8</v>
       </c>
       <c r="AJ158" t="n">
-        <v>1</v>
+        <v>0.1818181818181818</v>
       </c>
     </row>
     <row r="159">
@@ -17468,7 +17495,7 @@
         <v>1</v>
       </c>
       <c r="AJ159" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.3636363636363636</v>
       </c>
     </row>
     <row r="160">
@@ -17523,7 +17550,7 @@
         <v>0.625</v>
       </c>
       <c r="AJ160" t="n">
-        <v>0.8</v>
+        <v>0.2307692307692308</v>
       </c>
     </row>
     <row r="161">
@@ -17578,7 +17605,7 @@
         <v>0.5555555555555556</v>
       </c>
       <c r="AJ161" t="n">
-        <v>0.5555555555555556</v>
+        <v>0</v>
       </c>
     </row>
     <row r="162">
@@ -17633,7 +17660,7 @@
         <v>0.75</v>
       </c>
       <c r="AJ162" t="n">
-        <v>0.6363636363636364</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="163">
@@ -17688,7 +17715,7 @@
         <v>0.8</v>
       </c>
       <c r="AJ163" t="n">
-        <v>0.7</v>
+        <v>0.2222222222222222</v>
       </c>
     </row>
     <row r="164">
@@ -17743,7 +17770,7 @@
         <v>0.8571428571428571</v>
       </c>
       <c r="AJ164" t="n">
-        <v>0.3</v>
+        <v>0.2222222222222222</v>
       </c>
     </row>
     <row r="165">
@@ -17798,7 +17825,7 @@
         <v>1</v>
       </c>
       <c r="AJ165" t="n">
-        <v>0.3636363636363636</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="166">
@@ -17853,7 +17880,7 @@
         <v>0.75</v>
       </c>
       <c r="AJ166" t="n">
-        <v>0.625</v>
+        <v>0.4285714285714285</v>
       </c>
     </row>
     <row r="167">
@@ -17908,7 +17935,7 @@
         <v>1</v>
       </c>
       <c r="AJ167" t="n">
-        <v>0.25</v>
+        <v>0.4285714285714285</v>
       </c>
     </row>
     <row r="168">
@@ -17963,7 +17990,7 @@
         <v>1</v>
       </c>
       <c r="AJ168" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="169">
@@ -18018,7 +18045,7 @@
         <v>1</v>
       </c>
       <c r="AJ169" t="n">
-        <v>0.2222222222222222</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="170">
@@ -18073,7 +18100,7 @@
         <v>0.75</v>
       </c>
       <c r="AJ170" t="n">
-        <v>0.5</v>
+        <v>0.4444444444444444</v>
       </c>
     </row>
     <row r="171">
@@ -18128,7 +18155,7 @@
         <v>1</v>
       </c>
       <c r="AJ171" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="172">
@@ -18183,7 +18210,7 @@
         <v>1</v>
       </c>
       <c r="AJ172" t="n">
-        <v>0.5</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="173">
@@ -18238,7 +18265,7 @@
         <v>0.8</v>
       </c>
       <c r="AJ173" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="174">
@@ -18293,7 +18320,7 @@
         <v>1</v>
       </c>
       <c r="AJ174" t="n">
-        <v>1</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="175">
@@ -18348,7 +18375,7 @@
         <v>1</v>
       </c>
       <c r="AJ175" t="n">
-        <v>0.2727272727272727</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="176">
@@ -18403,7 +18430,7 @@
         <v>1</v>
       </c>
       <c r="AJ176" t="n">
-        <v>0.8</v>
+        <v>0.4444444444444444</v>
       </c>
     </row>
     <row r="177">
@@ -18458,7 +18485,7 @@
         <v>1</v>
       </c>
       <c r="AJ177" t="n">
-        <v>0.4</v>
+        <v>0.2857142857142857</v>
       </c>
     </row>
     <row r="178">
@@ -18513,7 +18540,7 @@
         <v>0.8</v>
       </c>
       <c r="AJ178" t="n">
-        <v>1</v>
+        <v>0.4444444444444444</v>
       </c>
     </row>
     <row r="179">
@@ -18568,7 +18595,7 @@
         <v>1</v>
       </c>
       <c r="AJ179" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.2222222222222222</v>
       </c>
     </row>
     <row r="180">
@@ -18623,7 +18650,7 @@
         <v>0.5</v>
       </c>
       <c r="AJ180" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="181">
@@ -18678,7 +18705,7 @@
         <v>1</v>
       </c>
       <c r="AJ181" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="182">
@@ -18733,7 +18760,7 @@
         <v>1</v>
       </c>
       <c r="AJ182" t="n">
-        <v>0.75</v>
+        <v>0.4166666666666667</v>
       </c>
     </row>
     <row r="183">
@@ -18843,7 +18870,7 @@
         <v>1</v>
       </c>
       <c r="AJ184" t="n">
-        <v>0.5</v>
+        <v>0.1111111111111111</v>
       </c>
     </row>
     <row r="185">
@@ -18898,7 +18925,7 @@
         <v>1</v>
       </c>
       <c r="AJ185" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="186">
@@ -18953,7 +18980,7 @@
         <v>1</v>
       </c>
       <c r="AJ186" t="n">
-        <v>0.4</v>
+        <v>0.3636363636363636</v>
       </c>
     </row>
     <row r="187">
@@ -19063,7 +19090,7 @@
         <v>1</v>
       </c>
       <c r="AJ188" t="n">
-        <v>0.75</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="189">
@@ -19118,7 +19145,7 @@
         <v>1</v>
       </c>
       <c r="AJ189" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="190">
@@ -19173,7 +19200,7 @@
         <v>1</v>
       </c>
       <c r="AJ190" t="n">
-        <v>0.375</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="191">
@@ -19228,7 +19255,7 @@
         <v>0.4</v>
       </c>
       <c r="AJ191" t="n">
-        <v>0.75</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="192">
@@ -19283,7 +19310,7 @@
         <v>0.75</v>
       </c>
       <c r="AJ192" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4545454545454545</v>
       </c>
     </row>
     <row r="193">
@@ -19338,7 +19365,7 @@
         <v>1</v>
       </c>
       <c r="AJ193" t="n">
-        <v>0.75</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="194">
@@ -19390,7 +19417,7 @@
         <v>0.6</v>
       </c>
       <c r="AJ194" t="n">
-        <v>0.4</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="195">
@@ -19445,7 +19472,7 @@
         <v>1</v>
       </c>
       <c r="AJ195" t="n">
-        <v>0.5</v>
+        <v>0.1666666666666667</v>
       </c>
     </row>
     <row r="196">
@@ -19555,7 +19582,7 @@
         <v>1</v>
       </c>
       <c r="AJ197" t="n">
-        <v>0.625</v>
+        <v>0.08333333333333333</v>
       </c>
     </row>
     <row r="198">
@@ -19610,7 +19637,7 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="AJ198" t="n">
-        <v>0.7</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="199">
@@ -19664,6 +19691,9 @@
       <c r="AI199" t="n">
         <v>1</v>
       </c>
+      <c r="AJ199" t="n">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="n">
@@ -19716,6 +19746,9 @@
       <c r="AI200" t="n">
         <v>1</v>
       </c>
+      <c r="AJ200" t="n">
+        <v>0.4285714285714285</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="n">
@@ -19768,6 +19801,9 @@
       <c r="AI201" t="n">
         <v>1</v>
       </c>
+      <c r="AJ201" t="n">
+        <v>0.2222222222222222</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="n">
@@ -19820,6 +19856,9 @@
       <c r="AI202" t="n">
         <v>1</v>
       </c>
+      <c r="AJ202" t="n">
+        <v>0.1111111111111111</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="n">
@@ -19872,6 +19911,9 @@
       <c r="AI203" t="n">
         <v>0.75</v>
       </c>
+      <c r="AJ203" t="n">
+        <v>0.2222222222222222</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="n">
@@ -19924,6 +19966,9 @@
       <c r="AI204" t="n">
         <v>1</v>
       </c>
+      <c r="AJ204" t="n">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="n">
@@ -19976,6 +20021,9 @@
       <c r="AI205" t="n">
         <v>0.8</v>
       </c>
+      <c r="AJ205" t="n">
+        <v>0.4444444444444444</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="n">
@@ -20028,6 +20076,9 @@
       <c r="AI206" t="n">
         <v>1</v>
       </c>
+      <c r="AJ206" t="n">
+        <v>0.2727272727272727</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="n">
@@ -20076,6 +20127,9 @@
       </c>
       <c r="AH207" t="n">
         <v>0.4</v>
+      </c>
+      <c r="AJ207" t="n">
+        <v>0.2222222222222222</v>
       </c>
     </row>
     <row r="208">
@@ -20185,7 +20239,7 @@
         <v>0.9658857142857143</v>
       </c>
       <c r="AJ212" t="n">
-        <v>0.936111111111111</v>
+        <v>0.8992571428571428</v>
       </c>
     </row>
     <row r="213">
@@ -20249,7 +20303,7 @@
         <v>0.8468571428571429</v>
       </c>
       <c r="AJ213" t="n">
-        <v>0.9478500000000001</v>
+        <v>0.91915</v>
       </c>
     </row>
     <row r="214">
@@ -20313,7 +20367,7 @@
         <v>0.8858333333333334</v>
       </c>
       <c r="AJ214" t="n">
-        <v>0.9270400000000001</v>
+        <v>0.9104857142857143</v>
       </c>
     </row>
     <row r="215">
@@ -20377,7 +20431,7 @@
         <v>0.9863166666666666</v>
       </c>
       <c r="AJ215" t="n">
-        <v>0.9197142857142857</v>
+        <v>0.86638</v>
       </c>
     </row>
     <row r="216">
@@ -20441,7 +20495,7 @@
         <v>0.8197333333333333</v>
       </c>
       <c r="AJ216" t="n">
-        <v>0.9202250000000001</v>
+        <v>0.9172142857142856</v>
       </c>
     </row>
     <row r="217">
@@ -20502,7 +20556,7 @@
         <v>0.9927142857142855</v>
       </c>
       <c r="AJ217" t="n">
-        <v>0.9224333333333333</v>
+        <v>0.9212833333333333</v>
       </c>
     </row>
     <row r="218">
@@ -20563,7 +20617,7 @@
         <v>0.9982200000000001</v>
       </c>
       <c r="AJ218" t="n">
-        <v>0.8960333333333333</v>
+        <v>0.91838</v>
       </c>
     </row>
     <row r="219">
@@ -20626,7 +20680,7 @@
         <v>0.8679625</v>
       </c>
       <c r="AJ219" t="n">
-        <v>0.9205</v>
+        <v>0.8862166666666665</v>
       </c>
     </row>
     <row r="220">
@@ -20689,7 +20743,7 @@
         <v>0.8760250000000001</v>
       </c>
       <c r="AJ220" t="n">
-        <v>0.8922</v>
+        <v>0.9026000000000001</v>
       </c>
     </row>
     <row r="221">
@@ -20750,7 +20804,7 @@
         <v>0.9856285714285714</v>
       </c>
       <c r="AJ221" t="n">
-        <v>0.8915166666666666</v>
+        <v>0.9098111111111111</v>
       </c>
     </row>
     <row r="222">
@@ -20805,7 +20859,7 @@
         <v>0.9943375</v>
       </c>
       <c r="AJ222" t="n">
-        <v>0.9132444444444445</v>
+        <v>0.885825</v>
       </c>
     </row>
     <row r="223">
@@ -20860,7 +20914,7 @@
         <v>0.8468199999999999</v>
       </c>
       <c r="AJ223" t="n">
-        <v>0.8975799999999999</v>
+        <v>0.9139250000000001</v>
       </c>
     </row>
     <row r="224">
@@ -20915,7 +20969,7 @@
         <v>0.9959571428571429</v>
       </c>
       <c r="AJ224" t="n">
-        <v>0.86815</v>
+        <v>0.9009</v>
       </c>
     </row>
     <row r="225">
@@ -20970,7 +21024,7 @@
         <v>0.989</v>
       </c>
       <c r="AJ225" t="n">
-        <v>0.8668142857142858</v>
+        <v>0.8681249999999999</v>
       </c>
     </row>
     <row r="226">
@@ -21025,7 +21079,7 @@
         <v>0.97255</v>
       </c>
       <c r="AJ226" t="n">
-        <v>0.8794999999999999</v>
+        <v>0.8482333333333333</v>
       </c>
     </row>
     <row r="227">
@@ -21080,7 +21134,7 @@
         <v>0.81014</v>
       </c>
       <c r="AJ227" t="n">
-        <v>0.8617833333333335</v>
+        <v>0.8643666666666666</v>
       </c>
     </row>
     <row r="228">
@@ -21135,7 +21189,7 @@
         <v>0.8912333333333334</v>
       </c>
       <c r="AJ228" t="n">
-        <v>0.8654000000000001</v>
+        <v>0.8840555555555555</v>
       </c>
     </row>
     <row r="229">
@@ -21190,7 +21244,7 @@
         <v>0.9319833333333333</v>
       </c>
       <c r="AJ229" t="n">
-        <v>0.893925</v>
+        <v>0.8273</v>
       </c>
     </row>
     <row r="230">
@@ -21245,7 +21299,7 @@
         <v>0.9897333333333332</v>
       </c>
       <c r="AJ230" t="n">
-        <v>0.8520142857142857</v>
+        <v>0.8815250000000001</v>
       </c>
     </row>
     <row r="231">
@@ -21300,7 +21354,7 @@
         <v>0.9861333333333334</v>
       </c>
       <c r="AJ231" t="n">
-        <v>0.8441599999999999</v>
+        <v>0.8689999999999999</v>
       </c>
     </row>
     <row r="232">
@@ -21355,7 +21409,7 @@
         <v>0.9921833333333333</v>
       </c>
       <c r="AJ232" t="n">
-        <v>0.8473000000000001</v>
+        <v>0.8808285714285715</v>
       </c>
     </row>
     <row r="233">
@@ -21410,7 +21464,7 @@
         <v>0.9827285714285715</v>
       </c>
       <c r="AJ233" t="n">
-        <v>0.8876000000000001</v>
+        <v>0.8465625000000001</v>
       </c>
     </row>
     <row r="234">
@@ -21465,7 +21519,7 @@
         <v>0.8867714285714285</v>
       </c>
       <c r="AJ234" t="n">
-        <v>0.8675250000000001</v>
+        <v>0.8626666666666667</v>
       </c>
     </row>
     <row r="235">
@@ -21520,7 +21574,7 @@
         <v>0.9881375</v>
       </c>
       <c r="AJ235" t="n">
-        <v>0.877</v>
+        <v>0.8592571428571427</v>
       </c>
     </row>
     <row r="236">
@@ -21575,7 +21629,7 @@
         <v>0.9941000000000001</v>
       </c>
       <c r="AJ236" t="n">
-        <v>0.8574857142857143</v>
+        <v>0.8395999999999999</v>
       </c>
     </row>
     <row r="237">
@@ -21630,7 +21684,7 @@
         <v>0.9599800000000001</v>
       </c>
       <c r="AJ237" t="n">
-        <v>0.85584</v>
+        <v>0.8627799999999999</v>
       </c>
     </row>
     <row r="238">
@@ -21685,7 +21739,7 @@
         <v>0.9938285714285714</v>
       </c>
       <c r="AJ238" t="n">
-        <v>0.8513300000000001</v>
+        <v>0.8603000000000001</v>
       </c>
     </row>
     <row r="239">
@@ -21740,7 +21794,7 @@
         <v>0.9918833333333333</v>
       </c>
       <c r="AJ239" t="n">
-        <v>0.8556833333333334</v>
+        <v>0.8609399999999999</v>
       </c>
     </row>
     <row r="240">
@@ -21795,7 +21849,7 @@
         <v>0.9929</v>
       </c>
       <c r="AJ240" t="n">
-        <v>0.863625</v>
+        <v>0.8786428571428571</v>
       </c>
     </row>
     <row r="241">
@@ -21850,7 +21904,7 @@
         <v>0.9923124999999999</v>
       </c>
       <c r="AJ241" t="n">
-        <v>0.8387500000000001</v>
+        <v>0.8101799999999999</v>
       </c>
     </row>
     <row r="242">
@@ -21905,7 +21959,7 @@
         <v>0.8736555555555554</v>
       </c>
       <c r="AJ242" t="n">
-        <v>0.8280750000000001</v>
+        <v>0.8791</v>
       </c>
     </row>
     <row r="243">
@@ -21960,7 +22014,7 @@
         <v>0.8641999999999999</v>
       </c>
       <c r="AJ243" t="n">
-        <v>0.87582</v>
+        <v>0.83655</v>
       </c>
     </row>
     <row r="244">
@@ -22015,7 +22069,7 @@
         <v>0.6879</v>
       </c>
       <c r="AJ244" t="n">
-        <v>0.8493857142857143</v>
+        <v>0.8113714285714286</v>
       </c>
     </row>
     <row r="245">
@@ -22070,7 +22124,7 @@
         <v>0.99176</v>
       </c>
       <c r="AJ245" t="n">
-        <v>0.8000666666666666</v>
+        <v>0.85868</v>
       </c>
     </row>
     <row r="246">
@@ -22125,7 +22179,7 @@
         <v>0.9963142857142858</v>
       </c>
       <c r="AJ246" t="n">
-        <v>0.8438428571428572</v>
+        <v>0.8534166666666666</v>
       </c>
     </row>
     <row r="247">
@@ -22180,7 +22234,7 @@
         <v>0.9844714285714286</v>
       </c>
       <c r="AJ247" t="n">
-        <v>0.8600000000000001</v>
+        <v>0.9068666666666667</v>
       </c>
     </row>
     <row r="248">
@@ -22235,7 +22289,7 @@
         <v>0.8516285714285715</v>
       </c>
       <c r="AJ248" t="n">
-        <v>0.84902</v>
+        <v>0.8584166666666667</v>
       </c>
     </row>
     <row r="249">
@@ -22290,7 +22344,7 @@
         <v>0.9866333333333334</v>
       </c>
       <c r="AJ249" t="n">
-        <v>0.8609499999999999</v>
+        <v>0.8535875000000001</v>
       </c>
     </row>
     <row r="250">
@@ -22345,7 +22399,7 @@
         <v>0.8845333333333333</v>
       </c>
       <c r="AJ250" t="n">
-        <v>0.86485</v>
+        <v>0.8670142857142858</v>
       </c>
     </row>
     <row r="251">
@@ -22400,7 +22454,7 @@
         <v>0.69035</v>
       </c>
       <c r="AJ251" t="n">
-        <v>0.85972</v>
+        <v>0.8413777777777778</v>
       </c>
     </row>
     <row r="252">
@@ -22455,7 +22509,7 @@
         <v>0.7249727272727272</v>
       </c>
       <c r="AJ252" t="n">
-        <v>0.8108714285714286</v>
+        <v>0.8776666666666667</v>
       </c>
     </row>
     <row r="253">
@@ -22510,7 +22564,7 @@
         <v>0.8805222222222223</v>
       </c>
       <c r="AJ253" t="n">
-        <v>0.8481099999999999</v>
+        <v>0.8770399999999998</v>
       </c>
     </row>
     <row r="254">
@@ -22565,7 +22619,7 @@
         <v>0.79576</v>
       </c>
       <c r="AJ254" t="n">
-        <v>0.8564666666666666</v>
+        <v>0.84945</v>
       </c>
     </row>
     <row r="255">
@@ -22620,7 +22674,7 @@
         <v>0.6875538461538462</v>
       </c>
       <c r="AJ255" t="n">
-        <v>0.8437749999999999</v>
+        <v>0.85295</v>
       </c>
     </row>
     <row r="256">
@@ -22675,7 +22729,7 @@
         <v>0.79863</v>
       </c>
       <c r="AJ256" t="n">
-        <v>0.810275</v>
+        <v>0.8704285714285714</v>
       </c>
     </row>
     <row r="257">
@@ -22730,7 +22784,7 @@
         <v>0.6415727272727273</v>
       </c>
       <c r="AJ257" t="n">
-        <v>0.8225857142857144</v>
+        <v>0.883</v>
       </c>
     </row>
     <row r="258">
@@ -22785,7 +22839,7 @@
         <v>0.69429</v>
       </c>
       <c r="AJ258" t="n">
-        <v>0.8418499999999999</v>
+        <v>0.8561571428571428</v>
       </c>
     </row>
     <row r="259">
@@ -22840,7 +22894,7 @@
         <v>0.6539555555555556</v>
       </c>
       <c r="AJ259" t="n">
-        <v>0.8089888888888888</v>
+        <v>0.8793000000000001</v>
       </c>
     </row>
     <row r="260">
@@ -22895,7 +22949,7 @@
         <v>0.65415</v>
       </c>
       <c r="AJ260" t="n">
-        <v>0.8360624999999999</v>
+        <v>0.8612555555555557</v>
       </c>
     </row>
     <row r="261">
@@ -22950,7 +23004,7 @@
         <v>0.8725222222222222</v>
       </c>
       <c r="AJ261" t="n">
-        <v>0.8252166666666666</v>
+        <v>0.8754777777777778</v>
       </c>
     </row>
     <row r="262">
@@ -23005,7 +23059,7 @@
         <v>0.7095181818181818</v>
       </c>
       <c r="AJ262" t="n">
-        <v>0.8382499999999999</v>
+        <v>0.8676</v>
       </c>
     </row>
     <row r="263">
@@ -23060,7 +23114,7 @@
         <v>0.8658857142857144</v>
       </c>
       <c r="AJ263" t="n">
-        <v>0.8127666666666666</v>
+        <v>0.8396250000000001</v>
       </c>
     </row>
     <row r="264">
@@ -23115,7 +23169,7 @@
         <v>0.5676285714285714</v>
       </c>
       <c r="AJ264" t="n">
-        <v>0.8460599999999999</v>
+        <v>0.8308</v>
       </c>
     </row>
     <row r="265">
@@ -23170,7 +23224,7 @@
         <v>0.4132000000000001</v>
       </c>
       <c r="AJ265" t="n">
-        <v>0.8023166666666667</v>
+        <v>0.8070000000000001</v>
       </c>
     </row>
     <row r="266">
@@ -23225,7 +23279,7 @@
         <v>0.7401</v>
       </c>
       <c r="AJ266" t="n">
-        <v>0.8532000000000001</v>
+        <v>0.8821600000000001</v>
       </c>
     </row>
     <row r="267">
@@ -23280,7 +23334,7 @@
         <v>0.6399181818181819</v>
       </c>
       <c r="AJ267" t="n">
-        <v>0.86492</v>
+        <v>0.8358166666666667</v>
       </c>
     </row>
     <row r="268">
@@ -23335,7 +23389,7 @@
         <v>0.4583555555555556</v>
       </c>
       <c r="AJ268" t="n">
-        <v>0.8317600000000001</v>
+        <v>0.8592333333333332</v>
       </c>
     </row>
     <row r="269">
@@ -23390,7 +23444,7 @@
         <v>0.9101500000000001</v>
       </c>
       <c r="AJ269" t="n">
-        <v>0.8783500000000001</v>
+        <v>0.8593999999999999</v>
       </c>
     </row>
     <row r="270">
@@ -23445,7 +23499,7 @@
         <v>0.6957083333333333</v>
       </c>
       <c r="AJ270" t="n">
-        <v>0.8458571428571429</v>
+        <v>0.849225</v>
       </c>
     </row>
     <row r="271">
@@ -23500,7 +23554,7 @@
         <v>0.7372083333333332</v>
       </c>
       <c r="AJ271" t="n">
-        <v>0.8659</v>
+        <v>0.83145</v>
       </c>
     </row>
     <row r="272">
@@ -23555,7 +23609,7 @@
         <v>0.7539166666666667</v>
       </c>
       <c r="AJ272" t="n">
-        <v>0.8267166666666667</v>
+        <v>0.8759</v>
       </c>
     </row>
     <row r="273">
@@ -23610,7 +23664,7 @@
         <v>0.4423727272727273</v>
       </c>
       <c r="AJ273" t="n">
-        <v>0.8344499999999999</v>
+        <v>0.8468</v>
       </c>
     </row>
     <row r="274">
@@ -23665,7 +23719,7 @@
         <v>0.6609333333333333</v>
       </c>
       <c r="AJ274" t="n">
-        <v>0.8324142857142857</v>
+        <v>0.84355</v>
       </c>
     </row>
     <row r="275">
@@ -23720,7 +23774,7 @@
         <v>0.654875</v>
       </c>
       <c r="AJ275" t="n">
-        <v>0.8711666666666668</v>
+        <v>0.8139199999999999</v>
       </c>
     </row>
     <row r="276">
@@ -23775,7 +23829,7 @@
         <v>0.723509090909091</v>
       </c>
       <c r="AJ276" t="n">
-        <v>0.8751599999999999</v>
+        <v>0.8504571428571428</v>
       </c>
     </row>
     <row r="277">
@@ -23830,7 +23884,7 @@
         <v>0.6337545454545453</v>
       </c>
       <c r="AJ277" t="n">
-        <v>0.8717</v>
+        <v>0.83058</v>
       </c>
     </row>
     <row r="278">
@@ -23885,7 +23939,7 @@
         <v>0.6305181818181818</v>
       </c>
       <c r="AJ278" t="n">
-        <v>0.8425428571428571</v>
+        <v>0.8725428571428572</v>
       </c>
     </row>
     <row r="279">
@@ -23940,7 +23994,7 @@
         <v>0.5742399999999999</v>
       </c>
       <c r="AJ279" t="n">
-        <v>0.8514250000000001</v>
+        <v>0.8826600000000001</v>
       </c>
     </row>
     <row r="280">
@@ -23995,7 +24049,7 @@
         <v>0.6294818181818183</v>
       </c>
       <c r="AJ280" t="n">
-        <v>0.8547399999999999</v>
+        <v>0.8270166666666667</v>
       </c>
     </row>
     <row r="281">
@@ -24050,7 +24104,7 @@
         <v>0.5350384615384616</v>
       </c>
       <c r="AJ281" t="n">
-        <v>0.8309799999999999</v>
+        <v>0.8699625000000001</v>
       </c>
     </row>
     <row r="282">
@@ -24105,7 +24159,7 @@
         <v>0.5364</v>
       </c>
       <c r="AJ282" t="n">
-        <v>0.8591499999999999</v>
+        <v>0.87125</v>
       </c>
     </row>
     <row r="283">
@@ -24160,7 +24214,7 @@
         <v>0.6825307692307692</v>
       </c>
       <c r="AJ283" t="n">
-        <v>0.8156625000000001</v>
+        <v>0.8579333333333333</v>
       </c>
     </row>
     <row r="284">
@@ -24215,7 +24269,7 @@
         <v>0.6116714285714286</v>
       </c>
       <c r="AJ284" t="n">
-        <v>0.815625</v>
+        <v>0.8507166666666666</v>
       </c>
     </row>
     <row r="285">
@@ -24270,7 +24324,7 @@
         <v>0.4963928571428571</v>
       </c>
       <c r="AJ285" t="n">
-        <v>0.8539875</v>
+        <v>0.87073</v>
       </c>
     </row>
     <row r="286">
@@ -24325,7 +24379,7 @@
         <v>0.49677</v>
       </c>
       <c r="AJ286" t="n">
-        <v>0.8410000000000001</v>
+        <v>0.8167333333333334</v>
       </c>
     </row>
     <row r="287">
@@ -24380,7 +24434,7 @@
         <v>0.4635083333333332</v>
       </c>
       <c r="AJ287" t="n">
-        <v>0.83048</v>
+        <v>0.8361600000000001</v>
       </c>
     </row>
     <row r="288">
@@ -24435,7 +24489,7 @@
         <v>0.7629461538461538</v>
       </c>
       <c r="AJ288" t="n">
-        <v>0.7994285714285715</v>
+        <v>0.85105</v>
       </c>
     </row>
     <row r="289">
@@ -24490,7 +24544,7 @@
         <v>0.5772499999999999</v>
       </c>
       <c r="AJ289" t="n">
-        <v>0.8455625000000001</v>
+        <v>0.84374</v>
       </c>
     </row>
     <row r="290">
@@ -24545,7 +24599,7 @@
         <v>0.6123000000000001</v>
       </c>
       <c r="AJ290" t="n">
-        <v>0.82806</v>
+        <v>0.8558749999999999</v>
       </c>
     </row>
     <row r="291">
@@ -24600,7 +24654,7 @@
         <v>0.584790909090909</v>
       </c>
       <c r="AJ291" t="n">
-        <v>0.82032</v>
+        <v>0.8377800000000001</v>
       </c>
     </row>
     <row r="292">
@@ -24655,7 +24709,7 @@
         <v>0.4132416666666667</v>
       </c>
       <c r="AJ292" t="n">
-        <v>0.8719571428571429</v>
+        <v>0.8409142857142858</v>
       </c>
     </row>
     <row r="293">
@@ -24710,7 +24764,7 @@
         <v>0.579175</v>
       </c>
       <c r="AJ293" t="n">
-        <v>0.8448749999999999</v>
+        <v>0.8438399999999999</v>
       </c>
     </row>
     <row r="294">
@@ -24765,7 +24819,7 @@
         <v>0.6215363636363637</v>
       </c>
       <c r="AJ294" t="n">
-        <v>0.8622</v>
+        <v>0.8594571428571429</v>
       </c>
     </row>
     <row r="295">
@@ -24820,7 +24874,7 @@
         <v>0.4937300000000001</v>
       </c>
       <c r="AJ295" t="n">
-        <v>0.8437</v>
+        <v>0.8276777777777777</v>
       </c>
     </row>
     <row r="296">
@@ -24875,7 +24929,7 @@
         <v>0.5772666666666667</v>
       </c>
       <c r="AJ296" t="n">
-        <v>0.8250166666666666</v>
+        <v>0.817025</v>
       </c>
     </row>
     <row r="297">
@@ -24930,7 +24984,7 @@
         <v>0.6120181818181818</v>
       </c>
       <c r="AJ297" t="n">
-        <v>0.8578571428571429</v>
+        <v>0.8481714285714286</v>
       </c>
     </row>
     <row r="298">
@@ -24982,7 +25036,7 @@
         <v>0.9347111111111109</v>
       </c>
       <c r="AJ298" t="n">
-        <v>0.82958</v>
+        <v>0.8610833333333332</v>
       </c>
     </row>
     <row r="299">
@@ -25037,7 +25091,7 @@
         <v>0.5577285714285715</v>
       </c>
       <c r="AJ299" t="n">
-        <v>0.84924</v>
+        <v>0.8157666666666666</v>
       </c>
     </row>
     <row r="300">
@@ -25092,7 +25146,7 @@
         <v>0.4594153846153847</v>
       </c>
       <c r="AJ300" t="n">
-        <v>0.8211999999999999</v>
+        <v>0.88574</v>
       </c>
     </row>
     <row r="301">
@@ -25147,7 +25201,7 @@
         <v>0.6131272727272727</v>
       </c>
       <c r="AJ301" t="n">
-        <v>0.8440428571428571</v>
+        <v>0.8037333333333333</v>
       </c>
     </row>
     <row r="302">
@@ -25202,7 +25256,7 @@
         <v>0.49454</v>
       </c>
       <c r="AJ302" t="n">
-        <v>0.8570399999999999</v>
+        <v>0.8636500000000001</v>
       </c>
     </row>
     <row r="303">
@@ -25256,6 +25310,9 @@
       <c r="AI303" t="n">
         <v>0.39781</v>
       </c>
+      <c r="AJ303" t="n">
+        <v>0.8760200000000001</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="n">
@@ -25308,6 +25365,9 @@
       <c r="AI304" t="n">
         <v>0.6814615384615385</v>
       </c>
+      <c r="AJ304" t="n">
+        <v>0.8511249999999999</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="n">
@@ -25360,6 +25420,9 @@
       <c r="AI305" t="n">
         <v>0.4392727272727273</v>
       </c>
+      <c r="AJ305" t="n">
+        <v>0.8675</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="n">
@@ -25412,6 +25475,9 @@
       <c r="AI306" t="n">
         <v>0.68553</v>
       </c>
+      <c r="AJ306" t="n">
+        <v>0.8625166666666667</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="n">
@@ -25464,6 +25530,9 @@
       <c r="AI307" t="n">
         <v>0.3657333333333333</v>
       </c>
+      <c r="AJ307" t="n">
+        <v>0.8500833333333334</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="n">
@@ -25516,6 +25585,9 @@
       <c r="AI308" t="n">
         <v>0.6255272727272727</v>
       </c>
+      <c r="AJ308" t="n">
+        <v>0.87418</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="n">
@@ -25568,6 +25640,9 @@
       <c r="AI309" t="n">
         <v>0.7243545454545455</v>
       </c>
+      <c r="AJ309" t="n">
+        <v>0.8195833333333334</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="n">
@@ -25620,6 +25695,9 @@
       <c r="AI310" t="n">
         <v>0.6400100000000001</v>
       </c>
+      <c r="AJ310" t="n">
+        <v>0.83875</v>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="n">
@@ -25670,6 +25748,9 @@
       </c>
       <c r="AH311" t="n">
         <v>0.9537153846153845</v>
+      </c>
+      <c r="AJ311" t="n">
+        <v>0.8205666666666667</v>
       </c>
     </row>
     <row r="312">
@@ -25779,7 +25860,7 @@
         <v>0.9558</v>
       </c>
       <c r="AJ316" t="n">
-        <v>0.0035</v>
+        <v>0.0281</v>
       </c>
     </row>
     <row r="317">
@@ -25843,7 +25924,7 @@
         <v>0</v>
       </c>
       <c r="AJ317" t="n">
-        <v>0.0004</v>
+        <v>0.0012</v>
       </c>
     </row>
     <row r="318">
@@ -25907,7 +25988,7 @@
         <v>0</v>
       </c>
       <c r="AJ318" t="n">
-        <v>0.0008</v>
+        <v>0.0607</v>
       </c>
     </row>
     <row r="319">
@@ -25971,7 +26052,7 @@
         <v>0.0044</v>
       </c>
       <c r="AJ319" t="n">
-        <v>0.0188</v>
+        <v>0.0148</v>
       </c>
     </row>
     <row r="320">
@@ -26035,7 +26116,7 @@
         <v>0.1013</v>
       </c>
       <c r="AJ320" t="n">
-        <v>0.1279</v>
+        <v>0.0166</v>
       </c>
     </row>
     <row r="321">
@@ -26096,7 +26177,7 @@
         <v>1</v>
       </c>
       <c r="AJ321" t="n">
-        <v>0.1657</v>
+        <v>0.077</v>
       </c>
     </row>
     <row r="322">
@@ -26157,7 +26238,7 @@
         <v>0.9284</v>
       </c>
       <c r="AJ322" t="n">
-        <v>0.0402</v>
+        <v>0.0448</v>
       </c>
     </row>
     <row r="323">
@@ -26218,7 +26299,7 @@
         <v>0.9044</v>
       </c>
       <c r="AJ323" t="n">
-        <v>0.1131</v>
+        <v>0.0555</v>
       </c>
     </row>
     <row r="324">
@@ -26279,7 +26360,7 @@
         <v>0.7281</v>
       </c>
       <c r="AJ324" t="n">
-        <v>0.0191</v>
+        <v>0.08119999999999999</v>
       </c>
     </row>
     <row r="325">
@@ -26340,7 +26421,7 @@
         <v>0.9208</v>
       </c>
       <c r="AJ325" t="n">
-        <v>0.105</v>
+        <v>0.1013</v>
       </c>
     </row>
     <row r="326">
@@ -26395,7 +26476,7 @@
         <v>0.9681999999999999</v>
       </c>
       <c r="AJ326" t="n">
-        <v>0.0219</v>
+        <v>0.1173</v>
       </c>
     </row>
     <row r="327">
@@ -26450,7 +26531,7 @@
         <v>0.7435</v>
       </c>
       <c r="AJ327" t="n">
-        <v>0.1532</v>
+        <v>0.0864</v>
       </c>
     </row>
     <row r="328">
@@ -26505,7 +26586,7 @@
         <v>0.5639999999999999</v>
       </c>
       <c r="AJ328" t="n">
-        <v>0.1418</v>
+        <v>0.1068</v>
       </c>
     </row>
     <row r="329">
@@ -26560,7 +26641,7 @@
         <v>0.2936</v>
       </c>
       <c r="AJ329" t="n">
-        <v>0.1263</v>
+        <v>0.0474</v>
       </c>
     </row>
     <row r="330">
@@ -26615,7 +26696,7 @@
         <v>0.846</v>
       </c>
       <c r="AJ330" t="n">
-        <v>0.0457</v>
+        <v>0.0354</v>
       </c>
     </row>
     <row r="331">
@@ -26670,7 +26751,7 @@
         <v>1</v>
       </c>
       <c r="AJ331" t="n">
-        <v>0.0926</v>
+        <v>0.1072</v>
       </c>
     </row>
     <row r="332">
@@ -26725,7 +26806,7 @@
         <v>0.9996</v>
       </c>
       <c r="AJ332" t="n">
-        <v>0.1191</v>
+        <v>0.1173</v>
       </c>
     </row>
     <row r="333">
@@ -26780,7 +26861,7 @@
         <v>0.9869</v>
       </c>
       <c r="AJ333" t="n">
-        <v>0.0677</v>
+        <v>0.0299</v>
       </c>
     </row>
     <row r="334">
@@ -26835,7 +26916,7 @@
         <v>0.9952</v>
       </c>
       <c r="AJ334" t="n">
-        <v>0.0469</v>
+        <v>0.0901</v>
       </c>
     </row>
     <row r="335">
@@ -26890,7 +26971,7 @@
         <v>0.9198</v>
       </c>
       <c r="AJ335" t="n">
-        <v>0.1161</v>
+        <v>0.07770000000000001</v>
       </c>
     </row>
     <row r="336">
@@ -26945,7 +27026,7 @@
         <v>0.9959</v>
       </c>
       <c r="AJ336" t="n">
-        <v>0.1399</v>
+        <v>0.0945</v>
       </c>
     </row>
     <row r="337">
@@ -27000,7 +27081,7 @@
         <v>0.8288</v>
       </c>
       <c r="AJ337" t="n">
-        <v>0.0672</v>
+        <v>0.0677</v>
       </c>
     </row>
     <row r="338">
@@ -27055,7 +27136,7 @@
         <v>0.9957</v>
       </c>
       <c r="AJ338" t="n">
-        <v>0.1072</v>
+        <v>0.0808</v>
       </c>
     </row>
     <row r="339">
@@ -27110,7 +27191,7 @@
         <v>1</v>
       </c>
       <c r="AJ339" t="n">
-        <v>0.0721</v>
+        <v>0.08459999999999999</v>
       </c>
     </row>
     <row r="340">
@@ -27165,7 +27246,7 @@
         <v>0.9986</v>
       </c>
       <c r="AJ340" t="n">
-        <v>0.0459</v>
+        <v>0.096</v>
       </c>
     </row>
     <row r="341">
@@ -27220,7 +27301,7 @@
         <v>0.9978</v>
       </c>
       <c r="AJ341" t="n">
-        <v>0.1061</v>
+        <v>0.1099</v>
       </c>
     </row>
     <row r="342">
@@ -27275,7 +27356,7 @@
         <v>0.9865</v>
       </c>
       <c r="AJ342" t="n">
-        <v>0.1175</v>
+        <v>0.0828</v>
       </c>
     </row>
     <row r="343">
@@ -27330,7 +27411,7 @@
         <v>0.9486</v>
       </c>
       <c r="AJ343" t="n">
-        <v>0.1197</v>
+        <v>0.1182</v>
       </c>
     </row>
     <row r="344">
@@ -27385,7 +27466,7 @@
         <v>0.9975000000000001</v>
       </c>
       <c r="AJ344" t="n">
-        <v>0.0978</v>
+        <v>0.0798</v>
       </c>
     </row>
     <row r="345">
@@ -27440,7 +27521,7 @@
         <v>0.9137999999999999</v>
       </c>
       <c r="AJ345" t="n">
-        <v>0.09470000000000001</v>
+        <v>0.08500000000000001</v>
       </c>
     </row>
     <row r="346">
@@ -27495,7 +27576,7 @@
         <v>0</v>
       </c>
       <c r="AJ346" t="n">
-        <v>0.1342</v>
+        <v>0.0898</v>
       </c>
     </row>
     <row r="347">
@@ -27550,7 +27631,7 @@
         <v>0.9943</v>
       </c>
       <c r="AJ347" t="n">
-        <v>0.1124</v>
+        <v>0.07530000000000001</v>
       </c>
     </row>
     <row r="348">
@@ -27605,7 +27686,7 @@
         <v>0</v>
       </c>
       <c r="AJ348" t="n">
-        <v>0.1427</v>
+        <v>0.09810000000000001</v>
       </c>
     </row>
     <row r="349">
@@ -27660,7 +27741,7 @@
         <v>0.0578</v>
       </c>
       <c r="AJ349" t="n">
-        <v>0.1128</v>
+        <v>0.0722</v>
       </c>
     </row>
     <row r="350">
@@ -27715,7 +27796,7 @@
         <v>0.9639</v>
       </c>
       <c r="AJ350" t="n">
-        <v>0.1134</v>
+        <v>0.0858</v>
       </c>
     </row>
     <row r="351">
@@ -27770,7 +27851,7 @@
         <v>1</v>
       </c>
       <c r="AJ351" t="n">
-        <v>0.1091</v>
+        <v>0.094</v>
       </c>
     </row>
     <row r="352">
@@ -27825,7 +27906,7 @@
         <v>0.9802999999999999</v>
       </c>
       <c r="AJ352" t="n">
-        <v>0.0788</v>
+        <v>0.07870000000000001</v>
       </c>
     </row>
     <row r="353">
@@ -27880,7 +27961,7 @@
         <v>1</v>
       </c>
       <c r="AJ353" t="n">
-        <v>0.09859999999999999</v>
+        <v>0.06710000000000001</v>
       </c>
     </row>
     <row r="354">
@@ -27935,7 +28016,7 @@
         <v>0.9728</v>
       </c>
       <c r="AJ354" t="n">
-        <v>0.1055</v>
+        <v>0.0547</v>
       </c>
     </row>
     <row r="355">
@@ -27990,7 +28071,7 @@
         <v>0</v>
       </c>
       <c r="AJ355" t="n">
-        <v>0.1042</v>
+        <v>0.07049999999999999</v>
       </c>
     </row>
     <row r="356">
@@ -28045,7 +28126,7 @@
         <v>0.1606</v>
       </c>
       <c r="AJ356" t="n">
-        <v>0.0961</v>
+        <v>0.0529</v>
       </c>
     </row>
     <row r="357">
@@ -28100,7 +28181,7 @@
         <v>0</v>
       </c>
       <c r="AJ357" t="n">
-        <v>0.1008</v>
+        <v>0.08019999999999999</v>
       </c>
     </row>
     <row r="358">
@@ -28155,7 +28236,7 @@
         <v>0</v>
       </c>
       <c r="AJ358" t="n">
-        <v>0.1019</v>
+        <v>0.0857</v>
       </c>
     </row>
     <row r="359">
@@ -28210,7 +28291,7 @@
         <v>0.8582</v>
       </c>
       <c r="AJ359" t="n">
-        <v>0.1123</v>
+        <v>0.0673</v>
       </c>
     </row>
     <row r="360">
@@ -28265,7 +28346,7 @@
         <v>0.9298</v>
       </c>
       <c r="AJ360" t="n">
-        <v>0.1037</v>
+        <v>0.09039999999999999</v>
       </c>
     </row>
     <row r="361">
@@ -28320,7 +28401,7 @@
         <v>0</v>
       </c>
       <c r="AJ361" t="n">
-        <v>0.07779999999999999</v>
+        <v>0.0898</v>
       </c>
     </row>
     <row r="362">
@@ -28375,7 +28456,7 @@
         <v>0</v>
       </c>
       <c r="AJ362" t="n">
-        <v>0.1028</v>
+        <v>0.0911</v>
       </c>
     </row>
     <row r="363">
@@ -28430,7 +28511,7 @@
         <v>0</v>
       </c>
       <c r="AJ363" t="n">
-        <v>0.0945</v>
+        <v>0.1179</v>
       </c>
     </row>
     <row r="364">
@@ -28485,7 +28566,7 @@
         <v>0</v>
       </c>
       <c r="AJ364" t="n">
-        <v>0.1214</v>
+        <v>0.0814</v>
       </c>
     </row>
     <row r="365">
@@ -28540,7 +28621,7 @@
         <v>0</v>
       </c>
       <c r="AJ365" t="n">
-        <v>0.097</v>
+        <v>0.08749999999999999</v>
       </c>
     </row>
     <row r="366">
@@ -28595,7 +28676,7 @@
         <v>1</v>
       </c>
       <c r="AJ366" t="n">
-        <v>0.0832</v>
+        <v>0.063</v>
       </c>
     </row>
     <row r="367">
@@ -28650,7 +28731,7 @@
         <v>0</v>
       </c>
       <c r="AJ367" t="n">
-        <v>0.1052</v>
+        <v>0.0701</v>
       </c>
     </row>
     <row r="368">
@@ -28705,7 +28786,7 @@
         <v>0</v>
       </c>
       <c r="AJ368" t="n">
-        <v>0.1062</v>
+        <v>0.0939</v>
       </c>
     </row>
     <row r="369">
@@ -28760,7 +28841,7 @@
         <v>0.4487</v>
       </c>
       <c r="AJ369" t="n">
-        <v>0.1004</v>
+        <v>0.1032</v>
       </c>
     </row>
     <row r="370">
@@ -28815,7 +28896,7 @@
         <v>1</v>
       </c>
       <c r="AJ370" t="n">
-        <v>0.0853</v>
+        <v>0.0769</v>
       </c>
     </row>
     <row r="371">
@@ -28870,7 +28951,7 @@
         <v>0.9911</v>
       </c>
       <c r="AJ371" t="n">
-        <v>0.09279999999999999</v>
+        <v>0.0738</v>
       </c>
     </row>
     <row r="372">
@@ -28925,7 +29006,7 @@
         <v>0.9928</v>
       </c>
       <c r="AJ372" t="n">
-        <v>0.1066</v>
+        <v>0.0707</v>
       </c>
     </row>
     <row r="373">
@@ -28980,7 +29061,7 @@
         <v>1</v>
       </c>
       <c r="AJ373" t="n">
-        <v>0.09959999999999999</v>
+        <v>0.08409999999999999</v>
       </c>
     </row>
     <row r="374">
@@ -29035,7 +29116,7 @@
         <v>0.9956</v>
       </c>
       <c r="AJ374" t="n">
-        <v>0.0888</v>
+        <v>0.0583</v>
       </c>
     </row>
     <row r="375">
@@ -29090,7 +29171,7 @@
         <v>1</v>
       </c>
       <c r="AJ375" t="n">
-        <v>0.0461</v>
+        <v>0.0448</v>
       </c>
     </row>
     <row r="376">
@@ -29145,7 +29226,7 @@
         <v>0</v>
       </c>
       <c r="AJ376" t="n">
-        <v>0.0492</v>
+        <v>0.0561</v>
       </c>
     </row>
     <row r="377">
@@ -29200,7 +29281,7 @@
         <v>0</v>
       </c>
       <c r="AJ377" t="n">
-        <v>0.0615</v>
+        <v>0.0481</v>
       </c>
     </row>
     <row r="378">
@@ -29255,7 +29336,7 @@
         <v>0</v>
       </c>
       <c r="AJ378" t="n">
-        <v>0.1055</v>
+        <v>0.0538</v>
       </c>
     </row>
     <row r="379">
@@ -29310,7 +29391,7 @@
         <v>0</v>
       </c>
       <c r="AJ379" t="n">
-        <v>0.0897</v>
+        <v>0.0631</v>
       </c>
     </row>
     <row r="380">
@@ -29365,7 +29446,7 @@
         <v>0.4348</v>
       </c>
       <c r="AJ380" t="n">
-        <v>0.0881</v>
+        <v>0.0728</v>
       </c>
     </row>
     <row r="381">
@@ -29420,7 +29501,7 @@
         <v>0.9605</v>
       </c>
       <c r="AJ381" t="n">
-        <v>0.1029</v>
+        <v>0.0873</v>
       </c>
     </row>
     <row r="382">
@@ -29475,7 +29556,7 @@
         <v>0</v>
       </c>
       <c r="AJ382" t="n">
-        <v>0.1014</v>
+        <v>0.07870000000000001</v>
       </c>
     </row>
     <row r="383">
@@ -29530,7 +29611,7 @@
         <v>0</v>
       </c>
       <c r="AJ383" t="n">
-        <v>0.1244</v>
+        <v>0.0704</v>
       </c>
     </row>
     <row r="384">
@@ -29585,7 +29666,7 @@
         <v>0</v>
       </c>
       <c r="AJ384" t="n">
-        <v>0.1071</v>
+        <v>0.0649</v>
       </c>
     </row>
     <row r="385">
@@ -29640,7 +29721,7 @@
         <v>0</v>
       </c>
       <c r="AJ385" t="n">
-        <v>0.1123</v>
+        <v>0.06759999999999999</v>
       </c>
     </row>
     <row r="386">
@@ -29695,7 +29776,7 @@
         <v>0</v>
       </c>
       <c r="AJ386" t="n">
-        <v>0.09039999999999999</v>
+        <v>0.0618</v>
       </c>
     </row>
     <row r="387">
@@ -29750,7 +29831,7 @@
         <v>0</v>
       </c>
       <c r="AJ387" t="n">
-        <v>0.07920000000000001</v>
+        <v>0.0556</v>
       </c>
     </row>
     <row r="388">
@@ -29805,7 +29886,7 @@
         <v>0.9457</v>
       </c>
       <c r="AJ388" t="n">
-        <v>0.0955</v>
+        <v>0.0901</v>
       </c>
     </row>
     <row r="389">
@@ -29860,7 +29941,7 @@
         <v>0</v>
       </c>
       <c r="AJ389" t="n">
-        <v>0.1156</v>
+        <v>0.0885</v>
       </c>
     </row>
     <row r="390">
@@ -29915,7 +29996,7 @@
         <v>0</v>
       </c>
       <c r="AJ390" t="n">
-        <v>0.1201</v>
+        <v>0.08110000000000001</v>
       </c>
     </row>
     <row r="391">
@@ -29970,7 +30051,7 @@
         <v>0</v>
       </c>
       <c r="AJ391" t="n">
-        <v>0.0934</v>
+        <v>0.0862</v>
       </c>
     </row>
     <row r="392">
@@ -30025,7 +30106,7 @@
         <v>0</v>
       </c>
       <c r="AJ392" t="n">
-        <v>0.0827</v>
+        <v>0.1021</v>
       </c>
     </row>
     <row r="393">
@@ -30080,7 +30161,7 @@
         <v>0.8885999999999999</v>
       </c>
       <c r="AJ393" t="n">
-        <v>0.0983</v>
+        <v>0.0901</v>
       </c>
     </row>
     <row r="394">
@@ -30135,7 +30216,7 @@
         <v>0</v>
       </c>
       <c r="AJ394" t="n">
-        <v>0.0919</v>
+        <v>0.1016</v>
       </c>
     </row>
     <row r="395">
@@ -30190,7 +30271,7 @@
         <v>0.004</v>
       </c>
       <c r="AJ395" t="n">
-        <v>0.1099</v>
+        <v>0.09950000000000001</v>
       </c>
     </row>
     <row r="396">
@@ -30245,7 +30326,7 @@
         <v>0</v>
       </c>
       <c r="AJ396" t="n">
-        <v>0.0964</v>
+        <v>0.07770000000000001</v>
       </c>
     </row>
     <row r="397">
@@ -30300,7 +30381,7 @@
         <v>0</v>
       </c>
       <c r="AJ397" t="n">
-        <v>0.0917</v>
+        <v>0.0536</v>
       </c>
     </row>
     <row r="398">
@@ -30355,7 +30436,7 @@
         <v>0</v>
       </c>
       <c r="AJ398" t="n">
-        <v>0.0901</v>
+        <v>0.06759999999999999</v>
       </c>
     </row>
     <row r="399">
@@ -30410,7 +30491,7 @@
         <v>0</v>
       </c>
       <c r="AJ399" t="n">
-        <v>0.0955</v>
+        <v>0.0523</v>
       </c>
     </row>
     <row r="400">
@@ -30465,7 +30546,7 @@
         <v>0.6539</v>
       </c>
       <c r="AJ400" t="n">
-        <v>0.097</v>
+        <v>0.0427</v>
       </c>
     </row>
     <row r="401">
@@ -30520,7 +30601,7 @@
         <v>0</v>
       </c>
       <c r="AJ401" t="n">
-        <v>0.1237</v>
+        <v>0.0516</v>
       </c>
     </row>
     <row r="402">
@@ -30575,7 +30656,7 @@
         <v>0</v>
       </c>
       <c r="AJ402" t="n">
-        <v>0.1138</v>
+        <v>0.0795</v>
       </c>
     </row>
     <row r="403">
@@ -30630,7 +30711,7 @@
         <v>0</v>
       </c>
       <c r="AJ403" t="n">
-        <v>0.1078</v>
+        <v>0.07770000000000001</v>
       </c>
     </row>
     <row r="404">
@@ -30685,7 +30766,7 @@
         <v>0</v>
       </c>
       <c r="AJ404" t="n">
-        <v>0.0984</v>
+        <v>0.0856</v>
       </c>
     </row>
     <row r="405">
@@ -30740,7 +30821,7 @@
         <v>0.0023</v>
       </c>
       <c r="AJ405" t="n">
-        <v>0.1093</v>
+        <v>0.0725</v>
       </c>
     </row>
     <row r="406">
@@ -30795,7 +30876,7 @@
         <v>1</v>
       </c>
       <c r="AJ406" t="n">
-        <v>0.1216</v>
+        <v>0.083</v>
       </c>
     </row>
     <row r="407">
@@ -30849,6 +30930,9 @@
       <c r="AI407" t="n">
         <v>1</v>
       </c>
+      <c r="AJ407" t="n">
+        <v>0.0885</v>
+      </c>
     </row>
     <row r="408">
       <c r="A408" s="1" t="n">
@@ -30901,6 +30985,9 @@
       <c r="AI408" t="n">
         <v>0</v>
       </c>
+      <c r="AJ408" t="n">
+        <v>0.118</v>
+      </c>
     </row>
     <row r="409">
       <c r="A409" s="1" t="n">
@@ -30953,6 +31040,9 @@
       <c r="AI409" t="n">
         <v>0</v>
       </c>
+      <c r="AJ409" t="n">
+        <v>0.0916</v>
+      </c>
     </row>
     <row r="410">
       <c r="A410" s="1" t="n">
@@ -31005,6 +31095,9 @@
       <c r="AI410" t="n">
         <v>0.2872</v>
       </c>
+      <c r="AJ410" t="n">
+        <v>0.09619999999999999</v>
+      </c>
     </row>
     <row r="411">
       <c r="A411" s="1" t="n">
@@ -31057,6 +31150,9 @@
       <c r="AI411" t="n">
         <v>0</v>
       </c>
+      <c r="AJ411" t="n">
+        <v>0.08260000000000001</v>
+      </c>
     </row>
     <row r="412">
       <c r="A412" s="1" t="n">
@@ -31109,6 +31205,9 @@
       <c r="AI412" t="n">
         <v>0.9851</v>
       </c>
+      <c r="AJ412" t="n">
+        <v>0.0925</v>
+      </c>
     </row>
     <row r="413">
       <c r="A413" s="1" t="n">
@@ -31161,6 +31260,9 @@
       <c r="AI413" t="n">
         <v>0</v>
       </c>
+      <c r="AJ413" t="n">
+        <v>0.0693</v>
+      </c>
     </row>
     <row r="414">
       <c r="A414" s="1" t="n">
@@ -31213,6 +31315,9 @@
       <c r="AI414" t="n">
         <v>0</v>
       </c>
+      <c r="AJ414" t="n">
+        <v>0.0795</v>
+      </c>
     </row>
     <row r="415">
       <c r="A415" s="1" t="n">
@@ -31264,6 +31369,9 @@
       </c>
       <c r="AI415" t="n">
         <v>0</v>
+      </c>
+      <c r="AJ415" t="n">
+        <v>0.079</v>
       </c>
     </row>
     <row r="416">

</xml_diff>

<commit_message>
Ran my algorithm federated evaluated by benign
</commit_message>
<xml_diff>
--- a/CIFAR_Global.xlsx
+++ b/CIFAR_Global.xlsx
@@ -1345,7 +1345,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1407,7 +1407,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2205,7 +2205,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2267,7 +2267,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2305,7 +2305,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -3431,7 +3431,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -3493,7 +3493,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -3531,7 +3531,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -4658,7 +4658,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -4720,7 +4720,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -4758,7 +4758,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -5560,7 +5560,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -5622,7 +5622,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -5660,7 +5660,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -6791,7 +6791,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -6853,7 +6853,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -6891,7 +6891,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -7688,7 +7688,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -7750,7 +7750,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -7788,7 +7788,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -8575,7 +8575,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -8637,7 +8637,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -8675,7 +8675,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -9594,6 +9594,9 @@
       <c r="AK5" t="n">
         <v>0.1386380281690141</v>
       </c>
+      <c r="AL5" t="n">
+        <v>0.1257924444444445</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -9665,6 +9668,9 @@
       <c r="AK6" t="n">
         <v>0.1263564516129032</v>
       </c>
+      <c r="AL6" t="n">
+        <v>0.2064377777777778</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -9736,6 +9742,9 @@
       <c r="AK7" t="n">
         <v>0.2278352112676056</v>
       </c>
+      <c r="AL7" t="n">
+        <v>0.2912142222222222</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -9807,6 +9816,9 @@
       <c r="AK8" t="n">
         <v>0.3192188405797101</v>
       </c>
+      <c r="AL8" t="n">
+        <v>0.2724973333333334</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -9878,6 +9890,9 @@
       <c r="AK9" t="n">
         <v>0.3822619718309859</v>
       </c>
+      <c r="AL9" t="n">
+        <v>0.4219419354838709</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -9946,6 +9961,9 @@
       <c r="AK10" t="n">
         <v>0.2692161290322581</v>
       </c>
+      <c r="AL10" t="n">
+        <v>0.4521516129032258</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -10014,6 +10032,9 @@
       <c r="AK11" t="n">
         <v>0.4131238095238096</v>
       </c>
+      <c r="AL11" t="n">
+        <v>0.613716129032258</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -10082,6 +10103,9 @@
       <c r="AK12" t="n">
         <v>0.5052111111111111</v>
       </c>
+      <c r="AL12" t="n">
+        <v>0.6452322580645162</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -10150,6 +10174,9 @@
       <c r="AK13" t="n">
         <v>0.5099348484848485</v>
       </c>
+      <c r="AL13" t="n">
+        <v>0.7020000000000001</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -10218,6 +10245,9 @@
       <c r="AK14" t="n">
         <v>0.3749688524590164</v>
       </c>
+      <c r="AL14" t="n">
+        <v>0.7480032258064517</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -10280,6 +10310,9 @@
       <c r="AK15" t="n">
         <v>0.4214145161290322</v>
       </c>
+      <c r="AL15" t="n">
+        <v>0.7608903225806452</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -10342,6 +10375,9 @@
       <c r="AK16" t="n">
         <v>0.5007138888888888</v>
       </c>
+      <c r="AL16" t="n">
+        <v>0.7893354838709676</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -10404,6 +10440,9 @@
       <c r="AK17" t="n">
         <v>0.5127846153846154</v>
       </c>
+      <c r="AL17" t="n">
+        <v>0.678616129032258</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -10466,6 +10505,9 @@
       <c r="AK18" t="n">
         <v>0.5511027397260275</v>
       </c>
+      <c r="AL18" t="n">
+        <v>0.799683870967742</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -10528,6 +10570,9 @@
       <c r="AK19" t="n">
         <v>0.5746581081081081</v>
       </c>
+      <c r="AL19" t="n">
+        <v>0.806683870967742</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -10590,6 +10635,9 @@
       <c r="AK20" t="n">
         <v>0.6574028985507248</v>
       </c>
+      <c r="AL20" t="n">
+        <v>0.7787569444444444</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -10652,6 +10700,9 @@
       <c r="AK21" t="n">
         <v>0.6831257575757576</v>
       </c>
+      <c r="AL21" t="n">
+        <v>0.7809166666666667</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -10714,6 +10765,9 @@
       <c r="AK22" t="n">
         <v>0.6550805555555556</v>
       </c>
+      <c r="AL22" t="n">
+        <v>0.7907125000000002</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -10776,6 +10830,9 @@
       <c r="AK23" t="n">
         <v>0.613557627118644</v>
       </c>
+      <c r="AL23" t="n">
+        <v>0.7956861111111111</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -10835,6 +10892,9 @@
       <c r="AK24" t="n">
         <v>0.6791958333333333</v>
       </c>
+      <c r="AL24" t="n">
+        <v>0.70665</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -10897,6 +10957,9 @@
       <c r="AK25" t="n">
         <v>0.7276928571428571</v>
       </c>
+      <c r="AL25" t="n">
+        <v>0.6999527777777778</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -10959,6 +11022,9 @@
       <c r="AK26" t="n">
         <v>0.7134131147540983</v>
       </c>
+      <c r="AL26" t="n">
+        <v>0.7919349397590361</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -11021,6 +11087,9 @@
       <c r="AK27" t="n">
         <v>0.6768915492957748</v>
       </c>
+      <c r="AL27" t="n">
+        <v>0.7334602409638553</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -11083,6 +11152,9 @@
       <c r="AK28" t="n">
         <v>0.7085553571428571</v>
       </c>
+      <c r="AL28" t="n">
+        <v>0.8108012048192771</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -11145,6 +11217,9 @@
       <c r="AK29" t="n">
         <v>0.6852384615384616</v>
       </c>
+      <c r="AL29" t="n">
+        <v>0.8244975903614457</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -11207,6 +11282,9 @@
       <c r="AK30" t="n">
         <v>0.7506045454545455</v>
       </c>
+      <c r="AL30" t="n">
+        <v>0.820410891089109</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -11269,6 +11347,9 @@
       <c r="AK31" t="n">
         <v>0.6440066666666666</v>
       </c>
+      <c r="AL31" t="n">
+        <v>0.8277792079207921</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -11331,6 +11412,9 @@
       <c r="AK32" t="n">
         <v>0.7112148648648648</v>
       </c>
+      <c r="AL32" t="n">
+        <v>0.8313495049504952</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -11393,6 +11477,9 @@
       <c r="AK33" t="n">
         <v>0.6834353846153844</v>
       </c>
+      <c r="AL33" t="n">
+        <v>0.8318485148514851</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -11455,6 +11542,9 @@
       <c r="AK34" t="n">
         <v>0.733590277777778</v>
       </c>
+      <c r="AL34" t="n">
+        <v>0.8316237623762376</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -11517,6 +11607,9 @@
       <c r="AK35" t="n">
         <v>0.7530107692307693</v>
       </c>
+      <c r="AL35" t="n">
+        <v>0.8332514851485149</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -11579,6 +11672,9 @@
       <c r="AK36" t="n">
         <v>0.7217968253968254</v>
       </c>
+      <c r="AL36" t="n">
+        <v>0.8387316831683169</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -11641,6 +11737,9 @@
       <c r="AK37" t="n">
         <v>0.6556320512820513</v>
       </c>
+      <c r="AL37" t="n">
+        <v>0.8406821782178218</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -11703,6 +11802,9 @@
       <c r="AK38" t="n">
         <v>0.7118328358208956</v>
       </c>
+      <c r="AL38" t="n">
+        <v>0.8404247524752473</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -11765,6 +11867,9 @@
       <c r="AK39" t="n">
         <v>0.727708064516129</v>
       </c>
+      <c r="AL39" t="n">
+        <v>0.815509900990099</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -11827,6 +11932,9 @@
       <c r="AK40" t="n">
         <v>0.7886147058823529</v>
       </c>
+      <c r="AL40" t="n">
+        <v>0.759640594059406</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -11889,6 +11997,9 @@
       <c r="AK41" t="n">
         <v>0.730413924050633</v>
       </c>
+      <c r="AL41" t="n">
+        <v>0.8379663366336634</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -11951,6 +12062,9 @@
       <c r="AK42" t="n">
         <v>0.7489522388059702</v>
       </c>
+      <c r="AL42" t="n">
+        <v>0.8441514851485149</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
@@ -12013,6 +12127,9 @@
       <c r="AK43" t="n">
         <v>0.8208923076923078</v>
       </c>
+      <c r="AL43" t="n">
+        <v>0.8480742574257425</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -12075,6 +12192,9 @@
       <c r="AK44" t="n">
         <v>0.7826338983050848</v>
       </c>
+      <c r="AL44" t="n">
+        <v>0.8473623762376237</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
@@ -12137,6 +12257,9 @@
       <c r="AK45" t="n">
         <v>0.7787951612903227</v>
       </c>
+      <c r="AL45" t="n">
+        <v>0.8486405940594061</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
@@ -12199,6 +12322,9 @@
       <c r="AK46" t="n">
         <v>0.7767076923076923</v>
       </c>
+      <c r="AL46" t="n">
+        <v>0.8488920792079209</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
@@ -12261,6 +12387,9 @@
       <c r="AK47" t="n">
         <v>0.7021123287671233</v>
       </c>
+      <c r="AL47" t="n">
+        <v>0.8508752475247526</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
@@ -12323,6 +12452,9 @@
       <c r="AK48" t="n">
         <v>0.7712261538461539</v>
       </c>
+      <c r="AL48" t="n">
+        <v>0.8473059405940595</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -12385,6 +12517,9 @@
       <c r="AK49" t="n">
         <v>0.7681384615384615</v>
       </c>
+      <c r="AL49" t="n">
+        <v>0.8531970297029702</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
@@ -12447,6 +12582,9 @@
       <c r="AK50" t="n">
         <v>0.7171411764705882</v>
       </c>
+      <c r="AL50" t="n">
+        <v>0.8547524752475247</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
@@ -12509,6 +12647,9 @@
       <c r="AK51" t="n">
         <v>0.8009735294117647</v>
       </c>
+      <c r="AL51" t="n">
+        <v>0.8533653465346536</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
@@ -12571,6 +12712,9 @@
       <c r="AK52" t="n">
         <v>0.7202890410958904</v>
       </c>
+      <c r="AL52" t="n">
+        <v>0.852157425742574</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
@@ -12633,6 +12777,9 @@
       <c r="AK53" t="n">
         <v>0.8416580645161291</v>
       </c>
+      <c r="AL53" t="n">
+        <v>0.8567633663366339</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
@@ -12695,6 +12842,9 @@
       <c r="AK54" t="n">
         <v>0.7825277777777777</v>
       </c>
+      <c r="AL54" t="n">
+        <v>0.8566742574257424</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
@@ -12757,6 +12907,9 @@
       <c r="AK55" t="n">
         <v>0.7369144927536232</v>
       </c>
+      <c r="AL55" t="n">
+        <v>0.857609900990099</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -12819,6 +12972,9 @@
       <c r="AK56" t="n">
         <v>0.7390823529411765</v>
       </c>
+      <c r="AL56" t="n">
+        <v>0.8575356435643562</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -12881,6 +13037,9 @@
       <c r="AK57" t="n">
         <v>0.7775129870129872</v>
       </c>
+      <c r="AL57" t="n">
+        <v>0.8549257425742576</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
@@ -12943,6 +13102,9 @@
       <c r="AK58" t="n">
         <v>0.7486031746031747</v>
       </c>
+      <c r="AL58" t="n">
+        <v>0.8533702970297031</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
@@ -13005,6 +13167,9 @@
       <c r="AK59" t="n">
         <v>0.7671826086956521</v>
       </c>
+      <c r="AL59" t="n">
+        <v>0.8534118811881187</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
@@ -13067,6 +13232,9 @@
       <c r="AK60" t="n">
         <v>0.7363104477611941</v>
       </c>
+      <c r="AL60" t="n">
+        <v>0.8553277227722773</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -13129,6 +13297,9 @@
       <c r="AK61" t="n">
         <v>0.7403500000000001</v>
       </c>
+      <c r="AL61" t="n">
+        <v>0.8560514851485148</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -13191,6 +13362,9 @@
       <c r="AK62" t="n">
         <v>0.7158892307692311</v>
       </c>
+      <c r="AL62" t="n">
+        <v>0.8540465346534654</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
@@ -13253,6 +13427,9 @@
       <c r="AK63" t="n">
         <v>0.7896105263157897</v>
       </c>
+      <c r="AL63" t="n">
+        <v>0.8577435643564357</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
@@ -13315,6 +13492,9 @@
       <c r="AK64" t="n">
         <v>0.814346875</v>
       </c>
+      <c r="AL64" t="n">
+        <v>0.8582801980198017</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
@@ -13377,6 +13557,9 @@
       <c r="AK65" t="n">
         <v>0.8171692307692306</v>
       </c>
+      <c r="AL65" t="n">
+        <v>0.8607544554455445</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
@@ -13439,6 +13622,9 @@
       <c r="AK66" t="n">
         <v>0.8209578125</v>
       </c>
+      <c r="AL66" t="n">
+        <v>0.8574138613861384</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
@@ -13501,6 +13687,9 @@
       <c r="AK67" t="n">
         <v>0.761528813559322</v>
       </c>
+      <c r="AL67" t="n">
+        <v>0.8573910891089108</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
@@ -13563,6 +13752,9 @@
       <c r="AK68" t="n">
         <v>0.7867015625000001</v>
       </c>
+      <c r="AL68" t="n">
+        <v>0.8564237623762374</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
@@ -13625,6 +13817,9 @@
       <c r="AK69" t="n">
         <v>0.7044828124999999</v>
       </c>
+      <c r="AL69" t="n">
+        <v>0.8576514851485149</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
@@ -13687,6 +13882,9 @@
       <c r="AK70" t="n">
         <v>0.7776037974683545</v>
       </c>
+      <c r="AL70" t="n">
+        <v>0.8563851485148515</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
@@ -13749,6 +13947,9 @@
       <c r="AK71" t="n">
         <v>0.7818285714285714</v>
       </c>
+      <c r="AL71" t="n">
+        <v>0.8533762376237624</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
@@ -13811,6 +14012,9 @@
       <c r="AK72" t="n">
         <v>0.8061909090909091</v>
       </c>
+      <c r="AL72" t="n">
+        <v>0.8248316831683168</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
@@ -13873,6 +14077,9 @@
       <c r="AK73" t="n">
         <v>0.7662701492537314</v>
       </c>
+      <c r="AL73" t="n">
+        <v>0.8533960396039604</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
@@ -13935,6 +14142,9 @@
       <c r="AK74" t="n">
         <v>0.7658607594936709</v>
       </c>
+      <c r="AL74" t="n">
+        <v>0.8568435643564355</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
@@ -13997,6 +14207,9 @@
       <c r="AK75" t="n">
         <v>0.7839774647887323</v>
       </c>
+      <c r="AL75" t="n">
+        <v>0.8583366336633663</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
@@ -14059,6 +14272,9 @@
       <c r="AK76" t="n">
         <v>0.8069718309859155</v>
       </c>
+      <c r="AL76" t="n">
+        <v>0.8568079207920793</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
@@ -14121,6 +14337,9 @@
       <c r="AK77" t="n">
         <v>0.7310378787878788</v>
       </c>
+      <c r="AL77" t="n">
+        <v>0.8567465346534653</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
@@ -14183,6 +14402,9 @@
       <c r="AK78" t="n">
         <v>0.8205750000000001</v>
       </c>
+      <c r="AL78" t="n">
+        <v>0.8502207920792079</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
@@ -14245,6 +14467,9 @@
       <c r="AK79" t="n">
         <v>0.7998083333333335</v>
       </c>
+      <c r="AL79" t="n">
+        <v>0.8551613861386139</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
@@ -14307,6 +14532,9 @@
       <c r="AK80" t="n">
         <v>0.7687053333333332</v>
       </c>
+      <c r="AL80" t="n">
+        <v>0.8564306930693069</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
@@ -14369,6 +14597,9 @@
       <c r="AK81" t="n">
         <v>0.7361242424242423</v>
       </c>
+      <c r="AL81" t="n">
+        <v>0.8601782178217823</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
@@ -14431,6 +14662,9 @@
       <c r="AK82" t="n">
         <v>0.7815644736842104</v>
       </c>
+      <c r="AL82" t="n">
+        <v>0.8631752475247524</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
@@ -14493,6 +14727,9 @@
       <c r="AK83" t="n">
         <v>0.7586675675675676</v>
       </c>
+      <c r="AL83" t="n">
+        <v>0.860357425742574</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
@@ -14555,6 +14792,9 @@
       <c r="AK84" t="n">
         <v>0.7499753424657535</v>
       </c>
+      <c r="AL84" t="n">
+        <v>0.8586079207920793</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
@@ -14617,6 +14857,9 @@
       <c r="AK85" t="n">
         <v>0.7529120481927711</v>
       </c>
+      <c r="AL85" t="n">
+        <v>0.860190099009901</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
@@ -14679,6 +14922,9 @@
       <c r="AK86" t="n">
         <v>0.822119696969697</v>
       </c>
+      <c r="AL86" t="n">
+        <v>0.8616356435643563</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
@@ -14741,6 +14987,9 @@
       <c r="AK87" t="n">
         <v>0.7708620253164559</v>
       </c>
+      <c r="AL87" t="n">
+        <v>0.8628950495049506</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
@@ -14803,6 +15052,9 @@
       <c r="AK88" t="n">
         <v>0.7890983333333333</v>
       </c>
+      <c r="AL88" t="n">
+        <v>0.8622138613861385</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
@@ -14865,6 +15117,9 @@
       <c r="AK89" t="n">
         <v>0.7864472222222223</v>
       </c>
+      <c r="AL89" t="n">
+        <v>0.8618584158415841</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
@@ -14927,6 +15182,9 @@
       <c r="AK90" t="n">
         <v>0.8617999999999999</v>
       </c>
+      <c r="AL90" t="n">
+        <v>0.8626693069306932</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
@@ -14989,6 +15247,9 @@
       <c r="AK91" t="n">
         <v>0.7949593749999999</v>
       </c>
+      <c r="AL91" t="n">
+        <v>0.863278217821782</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
@@ -15051,6 +15312,9 @@
       <c r="AK92" t="n">
         <v>0.7444309859154931</v>
       </c>
+      <c r="AL92" t="n">
+        <v>0.8649485148514851</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
@@ -15113,6 +15377,9 @@
       <c r="AK93" t="n">
         <v>0.7964983606557376</v>
       </c>
+      <c r="AL93" t="n">
+        <v>0.8657425742574256</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
@@ -15175,6 +15442,9 @@
       <c r="AK94" t="n">
         <v>0.7408680555555555</v>
       </c>
+      <c r="AL94" t="n">
+        <v>0.8632188118811879</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
@@ -15237,6 +15507,9 @@
       <c r="AK95" t="n">
         <v>0.7842112676056338</v>
       </c>
+      <c r="AL95" t="n">
+        <v>0.8626455445544554</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
@@ -15299,6 +15572,9 @@
       <c r="AK96" t="n">
         <v>0.7533506849315068</v>
       </c>
+      <c r="AL96" t="n">
+        <v>0.8630930693069305</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
@@ -15361,6 +15637,9 @@
       <c r="AK97" t="n">
         <v>0.7617279411764707</v>
       </c>
+      <c r="AL97" t="n">
+        <v>0.8640217821782178</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
@@ -15423,6 +15702,9 @@
       <c r="AK98" t="n">
         <v>0.8191549295774647</v>
       </c>
+      <c r="AL98" t="n">
+        <v>0.8638712871287128</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
@@ -15485,6 +15767,9 @@
       <c r="AK99" t="n">
         <v>0.7839013888888888</v>
       </c>
+      <c r="AL99" t="n">
+        <v>0.8640188118811879</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
@@ -15547,6 +15832,9 @@
       <c r="AK100" t="n">
         <v>0.7579888888888889</v>
       </c>
+      <c r="AL100" t="n">
+        <v>0.8624108910891091</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
@@ -15609,6 +15897,9 @@
       <c r="AK101" t="n">
         <v>0.7934216216216218</v>
       </c>
+      <c r="AL101" t="n">
+        <v>0.8657178217821783</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
@@ -15671,6 +15962,9 @@
       <c r="AK102" t="n">
         <v>0.8001478873239436</v>
       </c>
+      <c r="AL102" t="n">
+        <v>0.8638841584158417</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
@@ -15733,6 +16027,9 @@
       <c r="AK103" t="n">
         <v>0.7302142857142857</v>
       </c>
+      <c r="AL103" t="n">
+        <v>0.8634346534653465</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
@@ -15794,6 +16091,9 @@
       </c>
       <c r="AK104" t="n">
         <v>0.7005187500000001</v>
+      </c>
+      <c r="AL104" t="n">
+        <v>0.8626009900990097</v>
       </c>
     </row>
     <row r="105">
@@ -15901,6 +16201,9 @@
       <c r="AK108" t="n">
         <v>0.8666666666666667</v>
       </c>
+      <c r="AL108" t="n">
+        <v>0.9333333333333333</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
@@ -15965,6 +16268,9 @@
       <c r="AK109" t="n">
         <v>0.6666666666666666</v>
       </c>
+      <c r="AL109" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
@@ -16029,6 +16335,9 @@
       <c r="AK110" t="n">
         <v>0.1333333333333333</v>
       </c>
+      <c r="AL110" t="n">
+        <v>0.7333333333333333</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
@@ -16093,6 +16402,9 @@
       <c r="AK111" t="n">
         <v>0.6666666666666666</v>
       </c>
+      <c r="AL111" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
@@ -16157,6 +16469,9 @@
       <c r="AK112" t="n">
         <v>0.8</v>
       </c>
+      <c r="AL112" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
@@ -16218,6 +16533,9 @@
       <c r="AK113" t="n">
         <v>0.5333333333333333</v>
       </c>
+      <c r="AL113" t="n">
+        <v>0.3846153846153846</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
@@ -16279,6 +16597,9 @@
       <c r="AK114" t="n">
         <v>0.6</v>
       </c>
+      <c r="AL114" t="n">
+        <v>0.5833333333333334</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
@@ -16340,6 +16661,9 @@
       <c r="AK115" t="n">
         <v>0.5</v>
       </c>
+      <c r="AL115" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
@@ -16401,6 +16725,9 @@
       <c r="AK116" t="n">
         <v>0.6</v>
       </c>
+      <c r="AL116" t="n">
+        <v>0.8181818181818182</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
@@ -16462,6 +16789,9 @@
       <c r="AK117" t="n">
         <v>0.5333333333333333</v>
       </c>
+      <c r="AL117" t="n">
+        <v>0.7692307692307693</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
@@ -16517,6 +16847,9 @@
       <c r="AK118" t="n">
         <v>0.5714285714285714</v>
       </c>
+      <c r="AL118" t="n">
+        <v>0.9166666666666666</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
@@ -16572,6 +16905,9 @@
       <c r="AK119" t="n">
         <v>0.5333333333333333</v>
       </c>
+      <c r="AL119" t="n">
+        <v>0.7692307692307693</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
@@ -16627,6 +16963,9 @@
       <c r="AK120" t="n">
         <v>0.5333333333333333</v>
       </c>
+      <c r="AL120" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
@@ -16682,6 +17021,9 @@
       <c r="AK121" t="n">
         <v>0.6666666666666666</v>
       </c>
+      <c r="AL121" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
@@ -16737,6 +17079,9 @@
       <c r="AK122" t="n">
         <v>0.5333333333333333</v>
       </c>
+      <c r="AL122" t="n">
+        <v>0.6428571428571429</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
@@ -16792,6 +17137,9 @@
       <c r="AK123" t="n">
         <v>0.5333333333333333</v>
       </c>
+      <c r="AL123" t="n">
+        <v>0.9166666666666666</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
@@ -16847,6 +17195,9 @@
       <c r="AK124" t="n">
         <v>0.6</v>
       </c>
+      <c r="AL124" t="n">
+        <v>0.6428571428571429</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
@@ -16902,6 +17253,9 @@
       <c r="AK125" t="n">
         <v>0.5333333333333333</v>
       </c>
+      <c r="AL125" t="n">
+        <v>0.5714285714285714</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
@@ -16957,6 +17311,9 @@
       <c r="AK126" t="n">
         <v>0.4666666666666667</v>
       </c>
+      <c r="AL126" t="n">
+        <v>0.7272727272727273</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
@@ -17012,6 +17369,9 @@
       <c r="AK127" t="n">
         <v>0.8571428571428571</v>
       </c>
+      <c r="AL127" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
@@ -17067,6 +17427,9 @@
       <c r="AK128" t="n">
         <v>0.5714285714285714</v>
       </c>
+      <c r="AL128" t="n">
+        <v>0.4545454545454545</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
@@ -17122,6 +17485,9 @@
       <c r="AK129" t="n">
         <v>0.5714285714285714</v>
       </c>
+      <c r="AL129" t="n">
+        <v>0.9230769230769231</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
@@ -17177,6 +17543,9 @@
       <c r="AK130" t="n">
         <v>0.5333333333333333</v>
       </c>
+      <c r="AL130" t="n">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
@@ -17232,6 +17601,9 @@
       <c r="AK131" t="n">
         <v>0.6153846153846154</v>
       </c>
+      <c r="AL131" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
@@ -17287,6 +17659,9 @@
       <c r="AK132" t="n">
         <v>0.4615384615384616</v>
       </c>
+      <c r="AL132" t="n">
+        <v>0.8181818181818182</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
@@ -17342,6 +17717,9 @@
       <c r="AK133" t="n">
         <v>0.6</v>
       </c>
+      <c r="AL133" t="n">
+        <v>0.875</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
@@ -17397,6 +17775,9 @@
       <c r="AK134" t="n">
         <v>0.5</v>
       </c>
+      <c r="AL134" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
@@ -17452,6 +17833,9 @@
       <c r="AK135" t="n">
         <v>0.5714285714285714</v>
       </c>
+      <c r="AL135" t="n">
+        <v>0.8181818181818182</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
@@ -17507,6 +17891,9 @@
       <c r="AK136" t="n">
         <v>0.4615384615384616</v>
       </c>
+      <c r="AL136" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
@@ -17562,6 +17949,9 @@
       <c r="AK137" t="n">
         <v>0.5</v>
       </c>
+      <c r="AL137" t="n">
+        <v>0.9090909090909091</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
@@ -17617,6 +18007,9 @@
       <c r="AK138" t="n">
         <v>0.5384615384615384</v>
       </c>
+      <c r="AL138" t="n">
+        <v>0.9166666666666666</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
@@ -17672,6 +18065,9 @@
       <c r="AK139" t="n">
         <v>0.7142857142857143</v>
       </c>
+      <c r="AL139" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
@@ -17727,6 +18123,9 @@
       <c r="AK140" t="n">
         <v>0.7333333333333333</v>
       </c>
+      <c r="AL140" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
@@ -17782,6 +18181,9 @@
       <c r="AK141" t="n">
         <v>0.6</v>
       </c>
+      <c r="AL141" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
@@ -17837,6 +18239,9 @@
       <c r="AK142" t="n">
         <v>0.6</v>
       </c>
+      <c r="AL142" t="n">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
@@ -17892,6 +18297,9 @@
       <c r="AK143" t="n">
         <v>0.4615384615384616</v>
       </c>
+      <c r="AL143" t="n">
+        <v>0.1666666666666667</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
@@ -17947,6 +18355,9 @@
       <c r="AK144" t="n">
         <v>0.4285714285714285</v>
       </c>
+      <c r="AL144" t="n">
+        <v>0.875</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
@@ -18002,6 +18413,9 @@
       <c r="AK145" t="n">
         <v>0.5714285714285714</v>
       </c>
+      <c r="AL145" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
@@ -18057,6 +18471,9 @@
       <c r="AK146" t="n">
         <v>0.6153846153846154</v>
       </c>
+      <c r="AL146" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
@@ -18112,6 +18529,9 @@
       <c r="AK147" t="n">
         <v>0.4666666666666667</v>
       </c>
+      <c r="AL147" t="n">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
@@ -18167,6 +18587,9 @@
       <c r="AK148" t="n">
         <v>0.6666666666666666</v>
       </c>
+      <c r="AL148" t="n">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
@@ -18222,6 +18645,9 @@
       <c r="AK149" t="n">
         <v>0.6666666666666666</v>
       </c>
+      <c r="AL149" t="n">
+        <v>0.875</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
@@ -18277,6 +18703,9 @@
       <c r="AK150" t="n">
         <v>0.8666666666666667</v>
       </c>
+      <c r="AL150" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
@@ -18332,6 +18761,9 @@
       <c r="AK151" t="n">
         <v>0.6</v>
       </c>
+      <c r="AL151" t="n">
+        <v>0.7777777777777778</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
@@ -18387,6 +18819,9 @@
       <c r="AK152" t="n">
         <v>0.6428571428571429</v>
       </c>
+      <c r="AL152" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
@@ -18442,6 +18877,9 @@
       <c r="AK153" t="n">
         <v>0.6923076923076923</v>
       </c>
+      <c r="AL153" t="n">
+        <v>0.8181818181818182</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
@@ -18497,6 +18935,9 @@
       <c r="AK154" t="n">
         <v>0.8571428571428571</v>
       </c>
+      <c r="AL154" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
@@ -18552,6 +18993,9 @@
       <c r="AK155" t="n">
         <v>0.6428571428571429</v>
       </c>
+      <c r="AL155" t="n">
+        <v>0.7777777777777778</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
@@ -18607,6 +19051,9 @@
       <c r="AK156" t="n">
         <v>0.5833333333333334</v>
       </c>
+      <c r="AL156" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="n">
@@ -18662,6 +19109,9 @@
       <c r="AK157" t="n">
         <v>0.6923076923076923</v>
       </c>
+      <c r="AL157" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="n">
@@ -18717,6 +19167,9 @@
       <c r="AK158" t="n">
         <v>0.5714285714285714</v>
       </c>
+      <c r="AL158" t="n">
+        <v>0.9090909090909091</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="n">
@@ -18772,6 +19225,9 @@
       <c r="AK159" t="n">
         <v>0.4285714285714285</v>
       </c>
+      <c r="AL159" t="n">
+        <v>0.6666666666666666</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="n">
@@ -18827,6 +19283,9 @@
       <c r="AK160" t="n">
         <v>0.6</v>
       </c>
+      <c r="AL160" t="n">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="n">
@@ -18882,6 +19341,9 @@
       <c r="AK161" t="n">
         <v>0.5714285714285714</v>
       </c>
+      <c r="AL161" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
@@ -18937,6 +19399,9 @@
       <c r="AK162" t="n">
         <v>0.5714285714285714</v>
       </c>
+      <c r="AL162" t="n">
+        <v>0.8181818181818182</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="n">
@@ -18992,6 +19457,9 @@
       <c r="AK163" t="n">
         <v>0.2857142857142857</v>
       </c>
+      <c r="AL163" t="n">
+        <v>0.7142857142857143</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="n">
@@ -19047,6 +19515,9 @@
       <c r="AK164" t="n">
         <v>0.3846153846153846</v>
       </c>
+      <c r="AL164" t="n">
+        <v>0.9166666666666666</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="n">
@@ -19102,6 +19573,9 @@
       <c r="AK165" t="n">
         <v>0.6</v>
       </c>
+      <c r="AL165" t="n">
+        <v>0.7777777777777778</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="n">
@@ -19157,6 +19631,9 @@
       <c r="AK166" t="n">
         <v>0.6153846153846154</v>
       </c>
+      <c r="AL166" t="n">
+        <v>0.7777777777777778</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="n">
@@ -19212,6 +19689,9 @@
       <c r="AK167" t="n">
         <v>0.5714285714285714</v>
       </c>
+      <c r="AL167" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="n">
@@ -19267,6 +19747,9 @@
       <c r="AK168" t="n">
         <v>0.6923076923076923</v>
       </c>
+      <c r="AL168" t="n">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="n">
@@ -19322,6 +19805,9 @@
       <c r="AK169" t="n">
         <v>0.5833333333333334</v>
       </c>
+      <c r="AL169" t="n">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="n">
@@ -19377,6 +19863,9 @@
       <c r="AK170" t="n">
         <v>0.5384615384615384</v>
       </c>
+      <c r="AL170" t="n">
+        <v>0.7777777777777778</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="1" t="n">
@@ -19432,6 +19921,9 @@
       <c r="AK171" t="n">
         <v>0.5</v>
       </c>
+      <c r="AL171" t="n">
+        <v>0.6666666666666666</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="n">
@@ -19487,6 +19979,9 @@
       <c r="AK172" t="n">
         <v>0.5714285714285714</v>
       </c>
+      <c r="AL172" t="n">
+        <v>0.8181818181818182</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="n">
@@ -19542,6 +20037,9 @@
       <c r="AK173" t="n">
         <v>0.5384615384615384</v>
       </c>
+      <c r="AL173" t="n">
+        <v>0.2727272727272727</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="n">
@@ -19597,6 +20095,9 @@
       <c r="AK174" t="n">
         <v>0.7142857142857143</v>
       </c>
+      <c r="AL174" t="n">
+        <v>0.2727272727272727</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="n">
@@ -19652,6 +20153,9 @@
       <c r="AK175" t="n">
         <v>0.6153846153846154</v>
       </c>
+      <c r="AL175" t="n">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="1" t="n">
@@ -19707,6 +20211,9 @@
       <c r="AK176" t="n">
         <v>0.3333333333333333</v>
       </c>
+      <c r="AL176" t="n">
+        <v>0.7777777777777778</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="1" t="n">
@@ -19762,6 +20269,9 @@
       <c r="AK177" t="n">
         <v>0.5384615384615384</v>
       </c>
+      <c r="AL177" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="n">
@@ -19817,6 +20327,9 @@
       <c r="AK178" t="n">
         <v>0.5833333333333334</v>
       </c>
+      <c r="AL178" t="n">
+        <v>0.8571428571428571</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="n">
@@ -19872,6 +20385,9 @@
       <c r="AK179" t="n">
         <v>1</v>
       </c>
+      <c r="AL179" t="n">
+        <v>0.1818181818181818</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="n">
@@ -19927,6 +20443,9 @@
       <c r="AK180" t="n">
         <v>0.6428571428571429</v>
       </c>
+      <c r="AL180" t="n">
+        <v>0.8181818181818182</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="n">
@@ -19982,6 +20501,9 @@
       <c r="AK181" t="n">
         <v>0.4615384615384616</v>
       </c>
+      <c r="AL181" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="n">
@@ -20037,6 +20559,9 @@
       <c r="AK182" t="n">
         <v>0.6153846153846154</v>
       </c>
+      <c r="AL182" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="n">
@@ -20092,6 +20617,9 @@
       <c r="AK183" t="n">
         <v>0.4</v>
       </c>
+      <c r="AL183" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="n">
@@ -20147,6 +20675,9 @@
       <c r="AK184" t="n">
         <v>0.3846153846153846</v>
       </c>
+      <c r="AL184" t="n">
+        <v>0.8181818181818182</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="n">
@@ -20202,6 +20733,9 @@
       <c r="AK185" t="n">
         <v>0.5384615384615384</v>
       </c>
+      <c r="AL185" t="n">
+        <v>0.8571428571428571</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="n">
@@ -20257,6 +20791,9 @@
       <c r="AK186" t="n">
         <v>0.3076923076923077</v>
       </c>
+      <c r="AL186" t="n">
+        <v>0.6666666666666666</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="n">
@@ -20312,6 +20849,9 @@
       <c r="AK187" t="n">
         <v>0.6428571428571429</v>
       </c>
+      <c r="AL187" t="n">
+        <v>0.7777777777777778</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="n">
@@ -20367,6 +20907,9 @@
       <c r="AK188" t="n">
         <v>0.5384615384615384</v>
       </c>
+      <c r="AL188" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="n">
@@ -20422,6 +20965,9 @@
       <c r="AK189" t="n">
         <v>0.7142857142857143</v>
       </c>
+      <c r="AL189" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="n">
@@ -20477,6 +21023,9 @@
       <c r="AK190" t="n">
         <v>1</v>
       </c>
+      <c r="AL190" t="n">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="n">
@@ -20532,6 +21081,9 @@
       <c r="AK191" t="n">
         <v>0.5714285714285714</v>
       </c>
+      <c r="AL191" t="n">
+        <v>0.9090909090909091</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="n">
@@ -20587,6 +21139,9 @@
       <c r="AK192" t="n">
         <v>0.6153846153846154</v>
       </c>
+      <c r="AL192" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="n">
@@ -20642,6 +21197,9 @@
       <c r="AK193" t="n">
         <v>0.5333333333333333</v>
       </c>
+      <c r="AL193" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="n">
@@ -20697,6 +21255,9 @@
       <c r="AK194" t="n">
         <v>0.5384615384615384</v>
       </c>
+      <c r="AL194" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="n">
@@ -20752,6 +21313,9 @@
       <c r="AK195" t="n">
         <v>0.7142857142857143</v>
       </c>
+      <c r="AL195" t="n">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="n">
@@ -20807,6 +21371,9 @@
       <c r="AK196" t="n">
         <v>0.4285714285714285</v>
       </c>
+      <c r="AL196" t="n">
+        <v>0.9166666666666666</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="n">
@@ -20862,6 +21429,9 @@
       <c r="AK197" t="n">
         <v>0.6153846153846154</v>
       </c>
+      <c r="AL197" t="n">
+        <v>0.8181818181818182</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="n">
@@ -20917,6 +21487,9 @@
       <c r="AK198" t="n">
         <v>0.5833333333333334</v>
       </c>
+      <c r="AL198" t="n">
+        <v>0.8571428571428571</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="n">
@@ -20972,6 +21545,9 @@
       <c r="AK199" t="n">
         <v>0.3571428571428572</v>
       </c>
+      <c r="AL199" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="n">
@@ -21027,6 +21603,9 @@
       <c r="AK200" t="n">
         <v>0.2857142857142857</v>
       </c>
+      <c r="AL200" t="n">
+        <v>0.8888888888888888</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="n">
@@ -21082,6 +21661,9 @@
       <c r="AK201" t="n">
         <v>0.4545454545454545</v>
       </c>
+      <c r="AL201" t="n">
+        <v>0.7272727272727273</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="n">
@@ -21137,6 +21719,9 @@
       <c r="AK202" t="n">
         <v>0.5</v>
       </c>
+      <c r="AL202" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="n">
@@ -21192,6 +21777,9 @@
       <c r="AK203" t="n">
         <v>0.5333333333333333</v>
       </c>
+      <c r="AL203" t="n">
+        <v>0.9090909090909091</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="n">
@@ -21247,6 +21835,9 @@
       <c r="AK204" t="n">
         <v>0.4</v>
       </c>
+      <c r="AL204" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="n">
@@ -21302,6 +21893,9 @@
       <c r="AK205" t="n">
         <v>0.6</v>
       </c>
+      <c r="AL205" t="n">
+        <v>0.6666666666666666</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="n">
@@ -21357,6 +21951,9 @@
       <c r="AK206" t="n">
         <v>0.6153846153846154</v>
       </c>
+      <c r="AL206" t="n">
+        <v>0.8181818181818182</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="n">
@@ -21411,6 +22008,9 @@
       </c>
       <c r="AK207" t="n">
         <v>0.5714285714285714</v>
+      </c>
+      <c r="AL207" t="n">
+        <v>0.7142857142857143</v>
       </c>
     </row>
     <row r="208">
@@ -21522,6 +22122,9 @@
       <c r="AK212" t="n">
         <v>0.9234142857142859</v>
       </c>
+      <c r="AL212" t="n">
+        <v>0.931325</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="n">
@@ -21586,6 +22189,9 @@
       <c r="AK213" t="n">
         <v>0.928675</v>
       </c>
+      <c r="AL213" t="n">
+        <v>0.93224</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="n">
@@ -21650,6 +22256,9 @@
       <c r="AK214" t="n">
         <v>0.9277166666666665</v>
       </c>
+      <c r="AL214" t="n">
+        <v>0.9252600000000001</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="n">
@@ -21714,6 +22323,9 @@
       <c r="AK215" t="n">
         <v>0.9521500000000001</v>
       </c>
+      <c r="AL215" t="n">
+        <v>0.8901000000000001</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="n">
@@ -21778,6 +22390,9 @@
       <c r="AK216" t="n">
         <v>0.96014</v>
       </c>
+      <c r="AL216" t="n">
+        <v>0.9435428571428572</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="n">
@@ -21839,6 +22454,9 @@
       <c r="AK217" t="n">
         <v>0.9616999999999999</v>
       </c>
+      <c r="AL217" t="n">
+        <v>0.9278666666666666</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="n">
@@ -21900,6 +22518,9 @@
       <c r="AK218" t="n">
         <v>0.9511142857142857</v>
       </c>
+      <c r="AL218" t="n">
+        <v>0.9022999999999999</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="n">
@@ -21963,6 +22584,9 @@
       <c r="AK219" t="n">
         <v>0.9538142857142857</v>
       </c>
+      <c r="AL219" t="n">
+        <v>0.8905999999999999</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="n">
@@ -22026,6 +22650,9 @@
       <c r="AK220" t="n">
         <v>0.9679399999999999</v>
       </c>
+      <c r="AL220" t="n">
+        <v>0.9401833333333333</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="n">
@@ -22087,6 +22714,9 @@
       <c r="AK221" t="n">
         <v>0.9442142857142857</v>
       </c>
+      <c r="AL221" t="n">
+        <v>0.91234</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="n">
@@ -22142,6 +22772,9 @@
       <c r="AK222" t="n">
         <v>0.8791375</v>
       </c>
+      <c r="AL222" t="n">
+        <v>0.9351</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="n">
@@ -22197,6 +22830,9 @@
       <c r="AK223" t="n">
         <v>0.941342857142857</v>
       </c>
+      <c r="AL223" t="n">
+        <v>0.9156599999999999</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="1" t="n">
@@ -22252,6 +22888,9 @@
       <c r="AK224" t="n">
         <v>0.9188166666666667</v>
       </c>
+      <c r="AL224" t="n">
+        <v>0.8979857142857143</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="n">
@@ -22307,6 +22946,9 @@
       <c r="AK225" t="n">
         <v>0.944742857142857</v>
       </c>
+      <c r="AL225" t="n">
+        <v>0.8933444444444445</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="n">
@@ -22362,6 +23004,9 @@
       <c r="AK226" t="n">
         <v>0.9272666666666666</v>
       </c>
+      <c r="AL226" t="n">
+        <v>0.9359000000000001</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="n">
@@ -22417,6 +23062,9 @@
       <c r="AK227" t="n">
         <v>0.9517166666666667</v>
       </c>
+      <c r="AL227" t="n">
+        <v>0.9597000000000001</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="1" t="n">
@@ -22472,6 +23120,9 @@
       <c r="AK228" t="n">
         <v>0.9434666666666667</v>
       </c>
+      <c r="AL228" t="n">
+        <v>0.9311000000000001</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="1" t="n">
@@ -22527,6 +23178,9 @@
       <c r="AK229" t="n">
         <v>0.9695999999999999</v>
       </c>
+      <c r="AL229" t="n">
+        <v>0.9164571428571427</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="1" t="n">
@@ -22582,6 +23236,9 @@
       <c r="AK230" t="n">
         <v>0.9595166666666667</v>
       </c>
+      <c r="AL230" t="n">
+        <v>0.9412714285714285</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="1" t="n">
@@ -22637,6 +23294,9 @@
       <c r="AK231" t="n">
         <v>0.9349333333333334</v>
       </c>
+      <c r="AL231" t="n">
+        <v>0.9440875</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="1" t="n">
@@ -22692,6 +23352,9 @@
       <c r="AK232" t="n">
         <v>0.9292285714285714</v>
       </c>
+      <c r="AL232" t="n">
+        <v>0.9350625000000001</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="1" t="n">
@@ -22747,6 +23410,9 @@
       <c r="AK233" t="n">
         <v>0.9402666666666666</v>
       </c>
+      <c r="AL233" t="n">
+        <v>0.9423499999999999</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="1" t="n">
@@ -22802,6 +23468,9 @@
       <c r="AK234" t="n">
         <v>0.9615499999999999</v>
       </c>
+      <c r="AL234" t="n">
+        <v>0.9471857142857143</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="1" t="n">
@@ -22857,6 +23526,9 @@
       <c r="AK235" t="n">
         <v>0.9381857142857143</v>
       </c>
+      <c r="AL235" t="n">
+        <v>0.93145</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="1" t="n">
@@ -22912,6 +23584,9 @@
       <c r="AK236" t="n">
         <v>0.9203714285714286</v>
       </c>
+      <c r="AL236" t="n">
+        <v>0.8386166666666667</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="1" t="n">
@@ -22967,6 +23642,9 @@
       <c r="AK237" t="n">
         <v>0.9512999999999999</v>
       </c>
+      <c r="AL237" t="n">
+        <v>0.8813111111111112</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="1" t="n">
@@ -23022,6 +23700,9 @@
       <c r="AK238" t="n">
         <v>0.955557142857143</v>
       </c>
+      <c r="AL238" t="n">
+        <v>0.9318166666666667</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="1" t="n">
@@ -23077,6 +23758,9 @@
       <c r="AK239" t="n">
         <v>0.90438</v>
       </c>
+      <c r="AL239" t="n">
+        <v>0.9227000000000001</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="n">
@@ -23132,6 +23816,9 @@
       <c r="AK240" t="n">
         <v>0.9602749999999999</v>
       </c>
+      <c r="AL240" t="n">
+        <v>0.9375</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="n">
@@ -23187,6 +23874,9 @@
       <c r="AK241" t="n">
         <v>0.9457</v>
       </c>
+      <c r="AL241" t="n">
+        <v>0.92286</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="1" t="n">
@@ -23242,6 +23932,9 @@
       <c r="AK242" t="n">
         <v>0.956225</v>
       </c>
+      <c r="AL242" t="n">
+        <v>0.916075</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="n">
@@ -23297,6 +23990,9 @@
       <c r="AK243" t="n">
         <v>0.9604199999999998</v>
       </c>
+      <c r="AL243" t="n">
+        <v>0.85334</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="1" t="n">
@@ -23352,6 +24048,9 @@
       <c r="AK244" t="n">
         <v>0.9639999999999999</v>
       </c>
+      <c r="AL244" t="n">
+        <v>0.9238499999999999</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="n">
@@ -23407,6 +24106,9 @@
       <c r="AK245" t="n">
         <v>0.9513750000000001</v>
       </c>
+      <c r="AL245" t="n">
+        <v>0.9060400000000002</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="1" t="n">
@@ -23462,6 +24164,9 @@
       <c r="AK246" t="n">
         <v>0.9569333333333333</v>
       </c>
+      <c r="AL246" t="n">
+        <v>0.9267</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="1" t="n">
@@ -23517,6 +24222,9 @@
       <c r="AK247" t="n">
         <v>0.9393888888888888</v>
       </c>
+      <c r="AL247" t="n">
+        <v>0.922175</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="1" t="n">
@@ -23572,6 +24280,9 @@
       <c r="AK248" t="n">
         <v>0.9691</v>
       </c>
+      <c r="AL248" t="n">
+        <v>0.8397857142857142</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="1" t="n">
@@ -23627,6 +24338,9 @@
       <c r="AK249" t="n">
         <v>0.9608166666666667</v>
       </c>
+      <c r="AL249" t="n">
+        <v>0.9059333333333334</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="1" t="n">
@@ -23682,6 +24396,9 @@
       <c r="AK250" t="n">
         <v>0.9698285714285715</v>
       </c>
+      <c r="AL250" t="n">
+        <v>0.908</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="1" t="n">
@@ -23737,6 +24454,9 @@
       <c r="AK251" t="n">
         <v>0.9695714285714285</v>
       </c>
+      <c r="AL251" t="n">
+        <v>0.9016999999999999</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="1" t="n">
@@ -23792,6 +24512,9 @@
       <c r="AK252" t="n">
         <v>0.9761666666666667</v>
       </c>
+      <c r="AL252" t="n">
+        <v>0.90358</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="1" t="n">
@@ -23847,6 +24570,9 @@
       <c r="AK253" t="n">
         <v>0.9565857142857144</v>
       </c>
+      <c r="AL253" t="n">
+        <v>0.9084142857142857</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="1" t="n">
@@ -23902,6 +24628,9 @@
       <c r="AK254" t="n">
         <v>0.96565</v>
       </c>
+      <c r="AL254" t="n">
+        <v>0.9245000000000001</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="1" t="n">
@@ -23957,6 +24686,9 @@
       <c r="AK255" t="n">
         <v>0.9622000000000001</v>
       </c>
+      <c r="AL255" t="n">
+        <v>0.9242</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="1" t="n">
@@ -24012,6 +24744,9 @@
       <c r="AK256" t="n">
         <v>0.971525</v>
       </c>
+      <c r="AL256" t="n">
+        <v>0.9340000000000001</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="1" t="n">
@@ -24067,6 +24802,9 @@
       <c r="AK257" t="n">
         <v>0.8904000000000001</v>
       </c>
+      <c r="AL257" t="n">
+        <v>0.93344</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="1" t="n">
@@ -24122,6 +24860,9 @@
       <c r="AK258" t="n">
         <v>0.9167500000000001</v>
       </c>
+      <c r="AL258" t="n">
+        <v>0.9218374999999999</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="1" t="n">
@@ -24177,6 +24918,9 @@
       <c r="AK259" t="n">
         <v>0.9031666666666668</v>
       </c>
+      <c r="AL259" t="n">
+        <v>0.9323714285714286</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="1" t="n">
@@ -24232,6 +24976,9 @@
       <c r="AK260" t="n">
         <v>0.9232624999999999</v>
       </c>
+      <c r="AL260" t="n">
+        <v>0.9307</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="1" t="n">
@@ -24287,6 +25034,9 @@
       <c r="AK261" t="n">
         <v>0.9395625000000001</v>
       </c>
+      <c r="AL261" t="n">
+        <v>0.9276857142857142</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="1" t="n">
@@ -24342,6 +25092,9 @@
       <c r="AK262" t="n">
         <v>0.9276333333333332</v>
       </c>
+      <c r="AL262" t="n">
+        <v>0.8508</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="1" t="n">
@@ -24397,6 +25150,9 @@
       <c r="AK263" t="n">
         <v>0.96855</v>
       </c>
+      <c r="AL263" t="n">
+        <v>0.9155750000000001</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="1" t="n">
@@ -24452,6 +25208,9 @@
       <c r="AK264" t="n">
         <v>0.9761000000000001</v>
       </c>
+      <c r="AL264" t="n">
+        <v>0.9184833333333332</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="1" t="n">
@@ -24507,6 +25266,9 @@
       <c r="AK265" t="n">
         <v>0.9752624999999999</v>
       </c>
+      <c r="AL265" t="n">
+        <v>0.9153625</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="1" t="n">
@@ -24562,6 +25324,9 @@
       <c r="AK266" t="n">
         <v>0.8939199999999999</v>
       </c>
+      <c r="AL266" t="n">
+        <v>0.89458</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="1" t="n">
@@ -24617,6 +25382,9 @@
       <c r="AK267" t="n">
         <v>0.9657</v>
       </c>
+      <c r="AL267" t="n">
+        <v>0.9073500000000001</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="1" t="n">
@@ -24672,6 +25440,9 @@
       <c r="AK268" t="n">
         <v>0.9323375</v>
       </c>
+      <c r="AL268" t="n">
+        <v>0.89745</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="1" t="n">
@@ -24727,6 +25498,9 @@
       <c r="AK269" t="n">
         <v>0.9784</v>
       </c>
+      <c r="AL269" t="n">
+        <v>0.9156857142857142</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="1" t="n">
@@ -24782,6 +25556,9 @@
       <c r="AK270" t="n">
         <v>0.9554999999999999</v>
       </c>
+      <c r="AL270" t="n">
+        <v>0.9327142857142857</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
@@ -24837,6 +25614,9 @@
       <c r="AK271" t="n">
         <v>0.9751500000000002</v>
       </c>
+      <c r="AL271" t="n">
+        <v>0.8998333333333334</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
@@ -24892,6 +25672,9 @@
       <c r="AK272" t="n">
         <v>0.76898</v>
       </c>
+      <c r="AL272" t="n">
+        <v>0.9416166666666669</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
@@ -24947,6 +25730,9 @@
       <c r="AK273" t="n">
         <v>0.9248749999999999</v>
       </c>
+      <c r="AL273" t="n">
+        <v>0.95128</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
@@ -25002,6 +25788,9 @@
       <c r="AK274" t="n">
         <v>0.9533111111111112</v>
       </c>
+      <c r="AL274" t="n">
+        <v>0.9404</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
@@ -25057,6 +25846,9 @@
       <c r="AK275" t="n">
         <v>0.9154874999999999</v>
       </c>
+      <c r="AL275" t="n">
+        <v>0.9392857142857143</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
@@ -25112,6 +25904,9 @@
       <c r="AK276" t="n">
         <v>0.9205000000000001</v>
       </c>
+      <c r="AL276" t="n">
+        <v>0.9520500000000001</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
@@ -25167,6 +25962,9 @@
       <c r="AK277" t="n">
         <v>0.9105125000000001</v>
       </c>
+      <c r="AL277" t="n">
+        <v>0.9341199999999998</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
@@ -25222,6 +26020,9 @@
       <c r="AK278" t="n">
         <v>0.9320333333333334</v>
       </c>
+      <c r="AL278" t="n">
+        <v>0.94374</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
@@ -25277,6 +26078,9 @@
       <c r="AK279" t="n">
         <v>0.9031833333333333</v>
       </c>
+      <c r="AL279" t="n">
+        <v>0.94098</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
@@ -25332,6 +26136,9 @@
       <c r="AK280" t="n">
         <v>0.9307800000000001</v>
       </c>
+      <c r="AL280" t="n">
+        <v>0.9321</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
@@ -25387,6 +26194,9 @@
       <c r="AK281" t="n">
         <v>0.887625</v>
       </c>
+      <c r="AL281" t="n">
+        <v>0.927675</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="n">
@@ -25442,6 +26252,9 @@
       <c r="AK282" t="n">
         <v>0.9702875000000001</v>
       </c>
+      <c r="AL282" t="n">
+        <v>0.95495</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
@@ -25497,6 +26310,9 @@
       <c r="AK283" t="n">
         <v>0.8214600000000001</v>
       </c>
+      <c r="AL283" t="n">
+        <v>0.94316</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
@@ -25552,6 +26368,9 @@
       <c r="AK284" t="n">
         <v>0.9089571428571429</v>
       </c>
+      <c r="AL284" t="n">
+        <v>0.9449799999999999</v>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
@@ -25607,6 +26426,9 @@
       <c r="AK285" t="n">
         <v>0.9274777777777778</v>
       </c>
+      <c r="AL285" t="n">
+        <v>0.934642857142857</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
@@ -25662,6 +26484,9 @@
       <c r="AK286" t="n">
         <v>0.9525333333333332</v>
       </c>
+      <c r="AL286" t="n">
+        <v>0.91616</v>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
@@ -25717,6 +26542,9 @@
       <c r="AK287" t="n">
         <v>0.9794428571428572</v>
       </c>
+      <c r="AL287" t="n">
+        <v>0.94125</v>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
@@ -25772,6 +26600,9 @@
       <c r="AK288" t="n">
         <v>0.9242125</v>
       </c>
+      <c r="AL288" t="n">
+        <v>0.90412</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
@@ -25827,6 +26658,9 @@
       <c r="AK289" t="n">
         <v>0.9079444444444444</v>
       </c>
+      <c r="AL289" t="n">
+        <v>0.9233625</v>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
@@ -25882,6 +26716,9 @@
       <c r="AK290" t="n">
         <v>0.9758500000000001</v>
       </c>
+      <c r="AL290" t="n">
+        <v>0.9205444444444445</v>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
@@ -25937,6 +26774,9 @@
       <c r="AK291" t="n">
         <v>0.9763125</v>
       </c>
+      <c r="AL291" t="n">
+        <v>0.9487499999999999</v>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
@@ -25992,6 +26832,9 @@
       <c r="AK292" t="n">
         <v>0.96155</v>
       </c>
+      <c r="AL292" t="n">
+        <v>0.9234</v>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="n">
@@ -26047,6 +26890,9 @@
       <c r="AK293" t="n">
         <v>0.970675</v>
       </c>
+      <c r="AL293" t="n">
+        <v>0.94446</v>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="n">
@@ -26102,6 +26948,9 @@
       <c r="AK294" t="n">
         <v>0.95748</v>
       </c>
+      <c r="AL294" t="n">
+        <v>0.9338500000000001</v>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="n">
@@ -26157,6 +27006,9 @@
       <c r="AK295" t="n">
         <v>0.9533444444444444</v>
       </c>
+      <c r="AL295" t="n">
+        <v>0.9437166666666666</v>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="n">
@@ -26212,6 +27064,9 @@
       <c r="AK296" t="n">
         <v>0.8929400000000001</v>
       </c>
+      <c r="AL296" t="n">
+        <v>0.9023</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="n">
@@ -26267,6 +27122,9 @@
       <c r="AK297" t="n">
         <v>0.9756166666666667</v>
       </c>
+      <c r="AL297" t="n">
+        <v>0.9024428571428571</v>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="n">
@@ -26322,6 +27180,9 @@
       <c r="AK298" t="n">
         <v>0.9476222222222224</v>
       </c>
+      <c r="AL298" t="n">
+        <v>0.9085</v>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="n">
@@ -26377,6 +27238,9 @@
       <c r="AK299" t="n">
         <v>0.84368</v>
       </c>
+      <c r="AL299" t="n">
+        <v>0.9461666666666666</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="n">
@@ -26432,6 +27296,9 @@
       <c r="AK300" t="n">
         <v>0.9693750000000001</v>
       </c>
+      <c r="AL300" t="n">
+        <v>0.9084</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="n">
@@ -26487,6 +27354,9 @@
       <c r="AK301" t="n">
         <v>0.8427666666666668</v>
       </c>
+      <c r="AL301" t="n">
+        <v>0.9345800000000001</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="n">
@@ -26542,6 +27412,9 @@
       <c r="AK302" t="n">
         <v>0.8727545454545456</v>
       </c>
+      <c r="AL302" t="n">
+        <v>0.9203375</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="n">
@@ -26597,6 +27470,9 @@
       <c r="AK303" t="n">
         <v>0.9712000000000002</v>
       </c>
+      <c r="AL303" t="n">
+        <v>0.8888285714285713</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="n">
@@ -26652,6 +27528,9 @@
       <c r="AK304" t="n">
         <v>0.9714375</v>
       </c>
+      <c r="AL304" t="n">
+        <v>0.9393166666666667</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="n">
@@ -26707,6 +27586,9 @@
       <c r="AK305" t="n">
         <v>0.8745111111111111</v>
       </c>
+      <c r="AL305" t="n">
+        <v>0.9506333333333332</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="n">
@@ -26762,6 +27644,9 @@
       <c r="AK306" t="n">
         <v>0.900475</v>
       </c>
+      <c r="AL306" t="n">
+        <v>0.9536166666666667</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="n">
@@ -26817,6 +27702,9 @@
       <c r="AK307" t="n">
         <v>0.9775333333333331</v>
       </c>
+      <c r="AL307" t="n">
+        <v>0.915875</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="n">
@@ -26872,6 +27760,9 @@
       <c r="AK308" t="n">
         <v>0.9787333333333331</v>
       </c>
+      <c r="AL308" t="n">
+        <v>0.9108333333333333</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="n">
@@ -26927,6 +27818,9 @@
       <c r="AK309" t="n">
         <v>0.9787142857142858</v>
       </c>
+      <c r="AL309" t="n">
+        <v>0.9468333333333333</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="n">
@@ -26982,6 +27876,9 @@
       <c r="AK310" t="n">
         <v>0.9100000000000001</v>
       </c>
+      <c r="AL310" t="n">
+        <v>0.94325</v>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="n">
@@ -27036,6 +27933,9 @@
       </c>
       <c r="AK311" t="n">
         <v>0.976757142857143</v>
+      </c>
+      <c r="AL311" t="n">
+        <v>0.900825</v>
       </c>
     </row>
     <row r="312">
@@ -27147,6 +28047,9 @@
       <c r="AK316" t="n">
         <v>0.0107</v>
       </c>
+      <c r="AL316" t="n">
+        <v>0.0089</v>
+      </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="n">
@@ -27211,6 +28114,9 @@
       <c r="AK317" t="n">
         <v>0.0177</v>
       </c>
+      <c r="AL317" t="n">
+        <v>0.0126</v>
+      </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="n">
@@ -27275,6 +28181,9 @@
       <c r="AK318" t="n">
         <v>0.7292</v>
       </c>
+      <c r="AL318" t="n">
+        <v>0.0241</v>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="n">
@@ -27339,6 +28248,9 @@
       <c r="AK319" t="n">
         <v>0.1263</v>
       </c>
+      <c r="AL319" t="n">
+        <v>0.0594</v>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="n">
@@ -27403,6 +28315,9 @@
       <c r="AK320" t="n">
         <v>0.5432</v>
       </c>
+      <c r="AL320" t="n">
+        <v>0.0508</v>
+      </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="n">
@@ -27464,6 +28379,9 @@
       <c r="AK321" t="n">
         <v>0.0214</v>
       </c>
+      <c r="AL321" t="n">
+        <v>0.0115</v>
+      </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="n">
@@ -27525,6 +28443,9 @@
       <c r="AK322" t="n">
         <v>0.5604</v>
       </c>
+      <c r="AL322" t="n">
+        <v>0.1132</v>
+      </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="n">
@@ -27586,6 +28507,9 @@
       <c r="AK323" t="n">
         <v>0.738</v>
       </c>
+      <c r="AL323" t="n">
+        <v>0.2205</v>
+      </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="n">
@@ -27647,6 +28571,9 @@
       <c r="AK324" t="n">
         <v>0.8437</v>
       </c>
+      <c r="AL324" t="n">
+        <v>0.2434</v>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="n">
@@ -27708,6 +28635,9 @@
       <c r="AK325" t="n">
         <v>0.623</v>
       </c>
+      <c r="AL325" t="n">
+        <v>0.2845</v>
+      </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="n">
@@ -27763,6 +28693,9 @@
       <c r="AK326" t="n">
         <v>0.6113</v>
       </c>
+      <c r="AL326" t="n">
+        <v>0.313</v>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="n">
@@ -27818,6 +28751,9 @@
       <c r="AK327" t="n">
         <v>0.2872</v>
       </c>
+      <c r="AL327" t="n">
+        <v>0.3369</v>
+      </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="n">
@@ -27873,6 +28809,9 @@
       <c r="AK328" t="n">
         <v>0.761</v>
       </c>
+      <c r="AL328" t="n">
+        <v>0.2533</v>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="n">
@@ -27928,6 +28867,9 @@
       <c r="AK329" t="n">
         <v>0.6369</v>
       </c>
+      <c r="AL329" t="n">
+        <v>0.5447</v>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="n">
@@ -27983,6 +28925,9 @@
       <c r="AK330" t="n">
         <v>0.7791</v>
       </c>
+      <c r="AL330" t="n">
+        <v>0.7426</v>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="n">
@@ -28038,6 +28983,9 @@
       <c r="AK331" t="n">
         <v>0.9051</v>
       </c>
+      <c r="AL331" t="n">
+        <v>0.7345</v>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="n">
@@ -28093,6 +29041,9 @@
       <c r="AK332" t="n">
         <v>0.8895</v>
       </c>
+      <c r="AL332" t="n">
+        <v>0.6671</v>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="n">
@@ -28148,6 +29099,9 @@
       <c r="AK333" t="n">
         <v>0.9349</v>
       </c>
+      <c r="AL333" t="n">
+        <v>0.7753</v>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="n">
@@ -28203,6 +29157,9 @@
       <c r="AK334" t="n">
         <v>0.7105</v>
       </c>
+      <c r="AL334" t="n">
+        <v>0.7947</v>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="n">
@@ -28258,6 +29215,9 @@
       <c r="AK335" t="n">
         <v>0.7983</v>
       </c>
+      <c r="AL335" t="n">
+        <v>0.7077</v>
+      </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="n">
@@ -28313,6 +29273,9 @@
       <c r="AK336" t="n">
         <v>0.8174</v>
       </c>
+      <c r="AL336" t="n">
+        <v>0.4733</v>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="n">
@@ -28368,6 +29331,9 @@
       <c r="AK337" t="n">
         <v>0.883</v>
       </c>
+      <c r="AL337" t="n">
+        <v>0.5746</v>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="1" t="n">
@@ -28423,6 +29389,9 @@
       <c r="AK338" t="n">
         <v>0.9278999999999999</v>
       </c>
+      <c r="AL338" t="n">
+        <v>0.2351</v>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="1" t="n">
@@ -28478,6 +29447,9 @@
       <c r="AK339" t="n">
         <v>0.9481000000000001</v>
       </c>
+      <c r="AL339" t="n">
+        <v>0.4727</v>
+      </c>
     </row>
     <row r="340">
       <c r="A340" s="1" t="n">
@@ -28533,6 +29505,9 @@
       <c r="AK340" t="n">
         <v>0.8835</v>
       </c>
+      <c r="AL340" t="n">
+        <v>0.5871</v>
+      </c>
     </row>
     <row r="341">
       <c r="A341" s="1" t="n">
@@ -28588,6 +29563,9 @@
       <c r="AK341" t="n">
         <v>0.9258999999999999</v>
       </c>
+      <c r="AL341" t="n">
+        <v>0.6556999999999999</v>
+      </c>
     </row>
     <row r="342">
       <c r="A342" s="1" t="n">
@@ -28643,6 +29621,9 @@
       <c r="AK342" t="n">
         <v>0.8378</v>
       </c>
+      <c r="AL342" t="n">
+        <v>0.6911</v>
+      </c>
     </row>
     <row r="343">
       <c r="A343" s="1" t="n">
@@ -28698,6 +29679,9 @@
       <c r="AK343" t="n">
         <v>0.9206</v>
       </c>
+      <c r="AL343" t="n">
+        <v>0.7198</v>
+      </c>
     </row>
     <row r="344">
       <c r="A344" s="1" t="n">
@@ -28753,6 +29737,9 @@
       <c r="AK344" t="n">
         <v>0.9482</v>
       </c>
+      <c r="AL344" t="n">
+        <v>0.7431</v>
+      </c>
     </row>
     <row r="345">
       <c r="A345" s="1" t="n">
@@ -28808,6 +29795,9 @@
       <c r="AK345" t="n">
         <v>0.946</v>
       </c>
+      <c r="AL345" t="n">
+        <v>0.7573</v>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="1" t="n">
@@ -28863,6 +29853,9 @@
       <c r="AK346" t="n">
         <v>0.9533</v>
       </c>
+      <c r="AL346" t="n">
+        <v>0.7464</v>
+      </c>
     </row>
     <row r="347">
       <c r="A347" s="1" t="n">
@@ -28918,6 +29911,9 @@
       <c r="AK347" t="n">
         <v>0.9453</v>
       </c>
+      <c r="AL347" t="n">
+        <v>0.7292999999999999</v>
+      </c>
     </row>
     <row r="348">
       <c r="A348" s="1" t="n">
@@ -28973,6 +29969,9 @@
       <c r="AK348" t="n">
         <v>0.9406</v>
       </c>
+      <c r="AL348" t="n">
+        <v>0.7313</v>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="1" t="n">
@@ -29028,6 +30027,9 @@
       <c r="AK349" t="n">
         <v>0.8991</v>
       </c>
+      <c r="AL349" t="n">
+        <v>0.7282999999999999</v>
+      </c>
     </row>
     <row r="350">
       <c r="A350" s="1" t="n">
@@ -29083,6 +30085,9 @@
       <c r="AK350" t="n">
         <v>0.9386</v>
       </c>
+      <c r="AL350" t="n">
+        <v>0.472</v>
+      </c>
     </row>
     <row r="351">
       <c r="A351" s="1" t="n">
@@ -29138,6 +30143,9 @@
       <c r="AK351" t="n">
         <v>0.9575</v>
       </c>
+      <c r="AL351" t="n">
+        <v>0.5149</v>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="1" t="n">
@@ -29193,6 +30201,9 @@
       <c r="AK352" t="n">
         <v>0.9748</v>
       </c>
+      <c r="AL352" t="n">
+        <v>0.5433</v>
+      </c>
     </row>
     <row r="353">
       <c r="A353" s="1" t="n">
@@ -29248,6 +30259,9 @@
       <c r="AK353" t="n">
         <v>0.9671</v>
       </c>
+      <c r="AL353" t="n">
+        <v>0.5747</v>
+      </c>
     </row>
     <row r="354">
       <c r="A354" s="1" t="n">
@@ -29303,6 +30317,9 @@
       <c r="AK354" t="n">
         <v>0.9665</v>
       </c>
+      <c r="AL354" t="n">
+        <v>0.6355</v>
+      </c>
     </row>
     <row r="355">
       <c r="A355" s="1" t="n">
@@ -29358,6 +30375,9 @@
       <c r="AK355" t="n">
         <v>0.961</v>
       </c>
+      <c r="AL355" t="n">
+        <v>0.6669</v>
+      </c>
     </row>
     <row r="356">
       <c r="A356" s="1" t="n">
@@ -29413,6 +30433,9 @@
       <c r="AK356" t="n">
         <v>0.9676</v>
       </c>
+      <c r="AL356" t="n">
+        <v>0.5778</v>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="1" t="n">
@@ -29468,6 +30491,9 @@
       <c r="AK357" t="n">
         <v>0.9621</v>
       </c>
+      <c r="AL357" t="n">
+        <v>0.624</v>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="1" t="n">
@@ -29523,6 +30549,9 @@
       <c r="AK358" t="n">
         <v>0.9564</v>
       </c>
+      <c r="AL358" t="n">
+        <v>0.599</v>
+      </c>
     </row>
     <row r="359">
       <c r="A359" s="1" t="n">
@@ -29578,6 +30607,9 @@
       <c r="AK359" t="n">
         <v>0.9504</v>
       </c>
+      <c r="AL359" t="n">
+        <v>0.6332</v>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="1" t="n">
@@ -29633,6 +30665,9 @@
       <c r="AK360" t="n">
         <v>0.9086</v>
       </c>
+      <c r="AL360" t="n">
+        <v>0.7316</v>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="1" t="n">
@@ -29688,6 +30723,9 @@
       <c r="AK361" t="n">
         <v>0.9409999999999999</v>
       </c>
+      <c r="AL361" t="n">
+        <v>0.7899</v>
+      </c>
     </row>
     <row r="362">
       <c r="A362" s="1" t="n">
@@ -29743,6 +30781,9 @@
       <c r="AK362" t="n">
         <v>0.9598</v>
       </c>
+      <c r="AL362" t="n">
+        <v>0.7783</v>
+      </c>
     </row>
     <row r="363">
       <c r="A363" s="1" t="n">
@@ -29798,6 +30839,9 @@
       <c r="AK363" t="n">
         <v>0.9587</v>
       </c>
+      <c r="AL363" t="n">
+        <v>0.7603</v>
+      </c>
     </row>
     <row r="364">
       <c r="A364" s="1" t="n">
@@ -29853,6 +30897,9 @@
       <c r="AK364" t="n">
         <v>0.9675</v>
       </c>
+      <c r="AL364" t="n">
+        <v>0.765</v>
+      </c>
     </row>
     <row r="365">
       <c r="A365" s="1" t="n">
@@ -29908,6 +30955,9 @@
       <c r="AK365" t="n">
         <v>0.9722</v>
       </c>
+      <c r="AL365" t="n">
+        <v>0.7526</v>
+      </c>
     </row>
     <row r="366">
       <c r="A366" s="1" t="n">
@@ -29963,6 +31013,9 @@
       <c r="AK366" t="n">
         <v>0.9719</v>
       </c>
+      <c r="AL366" t="n">
+        <v>0.7314000000000001</v>
+      </c>
     </row>
     <row r="367">
       <c r="A367" s="1" t="n">
@@ -30018,6 +31071,9 @@
       <c r="AK367" t="n">
         <v>0.9677</v>
       </c>
+      <c r="AL367" t="n">
+        <v>0.7802</v>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="1" t="n">
@@ -30073,6 +31129,9 @@
       <c r="AK368" t="n">
         <v>0.9679</v>
       </c>
+      <c r="AL368" t="n">
+        <v>0.8155</v>
+      </c>
     </row>
     <row r="369">
       <c r="A369" s="1" t="n">
@@ -30128,6 +31187,9 @@
       <c r="AK369" t="n">
         <v>0.9742</v>
       </c>
+      <c r="AL369" t="n">
+        <v>0.8442</v>
+      </c>
     </row>
     <row r="370">
       <c r="A370" s="1" t="n">
@@ -30183,6 +31245,9 @@
       <c r="AK370" t="n">
         <v>0.9703000000000001</v>
       </c>
+      <c r="AL370" t="n">
+        <v>0.8464</v>
+      </c>
     </row>
     <row r="371">
       <c r="A371" s="1" t="n">
@@ -30238,6 +31303,9 @@
       <c r="AK371" t="n">
         <v>0.9567</v>
       </c>
+      <c r="AL371" t="n">
+        <v>0.8151</v>
+      </c>
     </row>
     <row r="372">
       <c r="A372" s="1" t="n">
@@ -30293,6 +31361,9 @@
       <c r="AK372" t="n">
         <v>0.9675</v>
       </c>
+      <c r="AL372" t="n">
+        <v>0.7921</v>
+      </c>
     </row>
     <row r="373">
       <c r="A373" s="1" t="n">
@@ -30348,6 +31419,9 @@
       <c r="AK373" t="n">
         <v>0.9771</v>
       </c>
+      <c r="AL373" t="n">
+        <v>0.8169999999999999</v>
+      </c>
     </row>
     <row r="374">
       <c r="A374" s="1" t="n">
@@ -30403,6 +31477,9 @@
       <c r="AK374" t="n">
         <v>0.9751</v>
       </c>
+      <c r="AL374" t="n">
+        <v>0.7999000000000001</v>
+      </c>
     </row>
     <row r="375">
       <c r="A375" s="1" t="n">
@@ -30458,6 +31535,9 @@
       <c r="AK375" t="n">
         <v>0.9715</v>
       </c>
+      <c r="AL375" t="n">
+        <v>0.8289</v>
+      </c>
     </row>
     <row r="376">
       <c r="A376" s="1" t="n">
@@ -30513,6 +31593,9 @@
       <c r="AK376" t="n">
         <v>0.9712</v>
       </c>
+      <c r="AL376" t="n">
+        <v>0.8406</v>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="1" t="n">
@@ -30568,6 +31651,9 @@
       <c r="AK377" t="n">
         <v>0.9788</v>
       </c>
+      <c r="AL377" t="n">
+        <v>0.8452</v>
+      </c>
     </row>
     <row r="378">
       <c r="A378" s="1" t="n">
@@ -30623,6 +31709,9 @@
       <c r="AK378" t="n">
         <v>0.9814000000000001</v>
       </c>
+      <c r="AL378" t="n">
+        <v>0.8502</v>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="1" t="n">
@@ -30678,6 +31767,9 @@
       <c r="AK379" t="n">
         <v>0.9818</v>
       </c>
+      <c r="AL379" t="n">
+        <v>0.8938</v>
+      </c>
     </row>
     <row r="380">
       <c r="A380" s="1" t="n">
@@ -30733,6 +31825,9 @@
       <c r="AK380" t="n">
         <v>0.9796</v>
       </c>
+      <c r="AL380" t="n">
+        <v>0.8748</v>
+      </c>
     </row>
     <row r="381">
       <c r="A381" s="1" t="n">
@@ -30788,6 +31883,9 @@
       <c r="AK381" t="n">
         <v>0.9796</v>
       </c>
+      <c r="AL381" t="n">
+        <v>0.7267</v>
+      </c>
     </row>
     <row r="382">
       <c r="A382" s="1" t="n">
@@ -30843,6 +31941,9 @@
       <c r="AK382" t="n">
         <v>0.9796</v>
       </c>
+      <c r="AL382" t="n">
+        <v>0.6847</v>
+      </c>
     </row>
     <row r="383">
       <c r="A383" s="1" t="n">
@@ -30898,6 +31999,9 @@
       <c r="AK383" t="n">
         <v>0.9752</v>
       </c>
+      <c r="AL383" t="n">
+        <v>0.6011</v>
+      </c>
     </row>
     <row r="384">
       <c r="A384" s="1" t="n">
@@ -30953,6 +32057,9 @@
       <c r="AK384" t="n">
         <v>0.9767</v>
       </c>
+      <c r="AL384" t="n">
+        <v>0.7789</v>
+      </c>
     </row>
     <row r="385">
       <c r="A385" s="1" t="n">
@@ -31008,6 +32115,9 @@
       <c r="AK385" t="n">
         <v>0.9789</v>
       </c>
+      <c r="AL385" t="n">
+        <v>0.8401</v>
+      </c>
     </row>
     <row r="386">
       <c r="A386" s="1" t="n">
@@ -31063,6 +32173,9 @@
       <c r="AK386" t="n">
         <v>0.9751</v>
       </c>
+      <c r="AL386" t="n">
+        <v>0.8865</v>
+      </c>
     </row>
     <row r="387">
       <c r="A387" s="1" t="n">
@@ -31118,6 +32231,9 @@
       <c r="AK387" t="n">
         <v>0.9679</v>
       </c>
+      <c r="AL387" t="n">
+        <v>0.7979000000000001</v>
+      </c>
     </row>
     <row r="388">
       <c r="A388" s="1" t="n">
@@ -31173,6 +32289,9 @@
       <c r="AK388" t="n">
         <v>0.9698</v>
       </c>
+      <c r="AL388" t="n">
+        <v>0.8171</v>
+      </c>
     </row>
     <row r="389">
       <c r="A389" s="1" t="n">
@@ -31228,6 +32347,9 @@
       <c r="AK389" t="n">
         <v>0.9776</v>
       </c>
+      <c r="AL389" t="n">
+        <v>0.7969000000000001</v>
+      </c>
     </row>
     <row r="390">
       <c r="A390" s="1" t="n">
@@ -31283,6 +32405,9 @@
       <c r="AK390" t="n">
         <v>0.9784</v>
       </c>
+      <c r="AL390" t="n">
+        <v>0.7825</v>
+      </c>
     </row>
     <row r="391">
       <c r="A391" s="1" t="n">
@@ -31338,6 +32463,9 @@
       <c r="AK391" t="n">
         <v>0.9777</v>
       </c>
+      <c r="AL391" t="n">
+        <v>0.7829</v>
+      </c>
     </row>
     <row r="392">
       <c r="A392" s="1" t="n">
@@ -31393,6 +32521,9 @@
       <c r="AK392" t="n">
         <v>0.9799</v>
       </c>
+      <c r="AL392" t="n">
+        <v>0.7756999999999999</v>
+      </c>
     </row>
     <row r="393">
       <c r="A393" s="1" t="n">
@@ -31448,6 +32579,9 @@
       <c r="AK393" t="n">
         <v>0.985</v>
       </c>
+      <c r="AL393" t="n">
+        <v>0.7816</v>
+      </c>
     </row>
     <row r="394">
       <c r="A394" s="1" t="n">
@@ -31503,6 +32637,9 @@
       <c r="AK394" t="n">
         <v>0.9774</v>
       </c>
+      <c r="AL394" t="n">
+        <v>0.8124</v>
+      </c>
     </row>
     <row r="395">
       <c r="A395" s="1" t="n">
@@ -31558,6 +32695,9 @@
       <c r="AK395" t="n">
         <v>0.9665</v>
       </c>
+      <c r="AL395" t="n">
+        <v>0.8264</v>
+      </c>
     </row>
     <row r="396">
       <c r="A396" s="1" t="n">
@@ -31613,6 +32753,9 @@
       <c r="AK396" t="n">
         <v>0.9686</v>
       </c>
+      <c r="AL396" t="n">
+        <v>0.8048</v>
+      </c>
     </row>
     <row r="397">
       <c r="A397" s="1" t="n">
@@ -31668,6 +32811,9 @@
       <c r="AK397" t="n">
         <v>0.9414</v>
       </c>
+      <c r="AL397" t="n">
+        <v>0.7065</v>
+      </c>
     </row>
     <row r="398">
       <c r="A398" s="1" t="n">
@@ -31723,6 +32869,9 @@
       <c r="AK398" t="n">
         <v>0.9338</v>
       </c>
+      <c r="AL398" t="n">
+        <v>0.7691</v>
+      </c>
     </row>
     <row r="399">
       <c r="A399" s="1" t="n">
@@ -31778,6 +32927,9 @@
       <c r="AK399" t="n">
         <v>0.9701</v>
       </c>
+      <c r="AL399" t="n">
+        <v>0.8087</v>
+      </c>
     </row>
     <row r="400">
       <c r="A400" s="1" t="n">
@@ -31833,6 +32985,9 @@
       <c r="AK400" t="n">
         <v>0.9801</v>
       </c>
+      <c r="AL400" t="n">
+        <v>0.7674</v>
+      </c>
     </row>
     <row r="401">
       <c r="A401" s="1" t="n">
@@ -31888,6 +33043,9 @@
       <c r="AK401" t="n">
         <v>0.9802</v>
       </c>
+      <c r="AL401" t="n">
+        <v>0.8303</v>
+      </c>
     </row>
     <row r="402">
       <c r="A402" s="1" t="n">
@@ -31943,6 +33101,9 @@
       <c r="AK402" t="n">
         <v>0.9775</v>
       </c>
+      <c r="AL402" t="n">
+        <v>0.8729</v>
+      </c>
     </row>
     <row r="403">
       <c r="A403" s="1" t="n">
@@ -31998,6 +33159,9 @@
       <c r="AK403" t="n">
         <v>0.9806</v>
       </c>
+      <c r="AL403" t="n">
+        <v>0.8695000000000001</v>
+      </c>
     </row>
     <row r="404">
       <c r="A404" s="1" t="n">
@@ -32053,6 +33217,9 @@
       <c r="AK404" t="n">
         <v>0.9795</v>
       </c>
+      <c r="AL404" t="n">
+        <v>0.87</v>
+      </c>
     </row>
     <row r="405">
       <c r="A405" s="1" t="n">
@@ -32108,6 +33275,9 @@
       <c r="AK405" t="n">
         <v>0.9821</v>
       </c>
+      <c r="AL405" t="n">
+        <v>0.8831</v>
+      </c>
     </row>
     <row r="406">
       <c r="A406" s="1" t="n">
@@ -32163,6 +33333,9 @@
       <c r="AK406" t="n">
         <v>0.9827</v>
       </c>
+      <c r="AL406" t="n">
+        <v>0.8893</v>
+      </c>
     </row>
     <row r="407">
       <c r="A407" s="1" t="n">
@@ -32218,6 +33391,9 @@
       <c r="AK407" t="n">
         <v>0.9823</v>
       </c>
+      <c r="AL407" t="n">
+        <v>0.8922</v>
+      </c>
     </row>
     <row r="408">
       <c r="A408" s="1" t="n">
@@ -32273,6 +33449,9 @@
       <c r="AK408" t="n">
         <v>0.9786</v>
       </c>
+      <c r="AL408" t="n">
+        <v>0.9031</v>
+      </c>
     </row>
     <row r="409">
       <c r="A409" s="1" t="n">
@@ -32328,6 +33507,9 @@
       <c r="AK409" t="n">
         <v>0.9791</v>
       </c>
+      <c r="AL409" t="n">
+        <v>0.9071</v>
+      </c>
     </row>
     <row r="410">
       <c r="A410" s="1" t="n">
@@ -32383,6 +33565,9 @@
       <c r="AK410" t="n">
         <v>0.9799</v>
       </c>
+      <c r="AL410" t="n">
+        <v>0.9253</v>
+      </c>
     </row>
     <row r="411">
       <c r="A411" s="1" t="n">
@@ -32438,6 +33623,9 @@
       <c r="AK411" t="n">
         <v>0.9814000000000001</v>
       </c>
+      <c r="AL411" t="n">
+        <v>0.9103</v>
+      </c>
     </row>
     <row r="412">
       <c r="A412" s="1" t="n">
@@ -32493,6 +33681,9 @@
       <c r="AK412" t="n">
         <v>0.9848</v>
       </c>
+      <c r="AL412" t="n">
+        <v>0.9077</v>
+      </c>
     </row>
     <row r="413">
       <c r="A413" s="1" t="n">
@@ -32548,6 +33739,9 @@
       <c r="AK413" t="n">
         <v>0.9819</v>
       </c>
+      <c r="AL413" t="n">
+        <v>0.9049</v>
+      </c>
     </row>
     <row r="414">
       <c r="A414" s="1" t="n">
@@ -32603,6 +33797,9 @@
       <c r="AK414" t="n">
         <v>0.9782999999999999</v>
       </c>
+      <c r="AL414" t="n">
+        <v>0.8942</v>
+      </c>
     </row>
     <row r="415">
       <c r="A415" s="1" t="n">
@@ -32657,6 +33854,9 @@
       </c>
       <c r="AK415" t="n">
         <v>0.9786</v>
+      </c>
+      <c r="AL415" t="n">
+        <v>0.903</v>
       </c>
     </row>
     <row r="416">

</xml_diff>